<commit_message>
Fix V1 formatting: safe fonts, explicit row heights, embedded thumbnails, T status default, rotated status/date headers
</commit_message>
<xml_diff>
--- a/material_package_fitout/260727_K5M_Material Package_Fitout.xlsx
+++ b/material_package_fitout/260727_K5M_Material Package_Fitout.xlsx
@@ -26,42 +26,42 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Playfair Display"/>
+      <name val="Cambria"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="18"/>
     </font>
     <font>
-      <name val="Lato"/>
+      <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00292B2B"/>
       <sz val="9"/>
     </font>
     <font>
-      <name val="Playfair Display"/>
+      <name val="Cambria"/>
       <b val="1"/>
       <color rgb="00292B2B"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Lato"/>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Lato"/>
+      <name val="Calibri"/>
       <color rgb="00292B2B"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Lato"/>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00292B2B"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Lato"/>
+      <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00E4572E"/>
       <sz val="8"/>
@@ -141,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -171,6 +171,9 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom" textRotation="90"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
@@ -182,6 +185,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -562,12 +568,12 @@
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="11" customWidth="1" min="17" max="17"/>
-    <col width="11" customWidth="1" min="18" max="18"/>
+    <col width="6" customWidth="1" min="13" max="13"/>
+    <col width="7" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="7" customWidth="1" min="16" max="16"/>
+    <col width="7" customWidth="1" min="17" max="17"/>
+    <col width="7" customWidth="1" min="18" max="18"/>
     <col width="34" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
@@ -691,12 +697,12 @@
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>Same proposed status-color extension as the FFE sheet (B/S colors not officially brand-defined) — confirm or replace.</t>
+          <t>Same proposed status-color extension as the FFE sheet (B/S colors not officially brand-defined) — confirm or replace. Status defaulted to T (To be Submitted) for every row as a starting point.</t>
         </is>
       </c>
     </row>
     <row r="12"/>
-    <row r="13" ht="34" customHeight="1">
+    <row r="13" ht="68" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
           <t>No.</t>
@@ -757,32 +763,32 @@
           <t>High-Res Link</t>
         </is>
       </c>
-      <c r="M13" s="12" t="inlineStr">
+      <c r="M13" s="13" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="N13" s="12" t="inlineStr">
+      <c r="N13" s="13" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="O13" s="12" t="inlineStr">
+      <c r="O13" s="13" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="P13" s="12" t="inlineStr">
+      <c r="P13" s="13" t="inlineStr">
         <is>
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="Q13" s="12" t="inlineStr">
+      <c r="Q13" s="13" t="inlineStr">
         <is>
           <t>2026-08-17</t>
         </is>
       </c>
-      <c r="R13" s="12" t="inlineStr">
+      <c r="R13" s="13" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
@@ -793,46 +799,46 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="60" customHeight="1">
-      <c r="A14" s="13" t="n">
+    <row r="14" ht="62" customHeight="1">
+      <c r="A14" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B14" s="14" t="inlineStr">
         <is>
           <t>A-ST-01c</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr"/>
-      <c r="D14" s="13" t="inlineStr">
+      <c r="C14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr">
         <is>
           <t>Stone</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr">
+      <c r="E14" s="15" t="inlineStr">
         <is>
           <t>Beige clair</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
+      <c r="F14" s="15" t="inlineStr">
         <is>
           <t>Light beige stone</t>
         </is>
       </c>
-      <c r="G14" s="13" t="inlineStr">
+      <c r="G14" s="14" t="inlineStr">
         <is>
           <t>Adouci / Honed</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr">
+      <c r="H14" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT-A/? (seuil), K5M-T1B1-SDB-B/6, K5M-T1B1-SDB-B/12, K5M-T1B1-CHA-C/2, K5M-T1B1-CHA-C/3</t>
         </is>
       </c>
-      <c r="I14" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
+      <c r="I14" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
               <color rgb="00292B2B"/>
               <sz val="1000"/>
             </rPr>
@@ -840,7 +846,7 @@
           </r>
           <r>
             <rPr>
-              <rFont val="Lato"/>
+              <rFont val="Calibri"/>
               <color rgb="00E4572E"/>
               <sz val="1000"/>
               <u val="single"/>
@@ -849,7 +855,7 @@
           </r>
           <r>
             <rPr>
-              <rFont val="Lato"/>
+              <rFont val="Calibri"/>
               <color rgb="00E4572E"/>
               <sz val="1000"/>
               <u val="single"/>
@@ -858,69 +864,73 @@
           </r>
         </is>
       </c>
-      <c r="J14" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K14" s="16" t="inlineStr">
+      <c r="J14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K14" s="17" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L14" s="17" t="inlineStr"/>
-      <c r="M14" s="17" t="inlineStr"/>
-      <c r="N14" s="17" t="inlineStr"/>
-      <c r="O14" s="17" t="inlineStr"/>
-      <c r="P14" s="17" t="inlineStr"/>
-      <c r="Q14" s="17" t="inlineStr"/>
-      <c r="R14" s="17" t="inlineStr"/>
-      <c r="S14" s="14" t="inlineStr">
+      <c r="L14" s="18" t="inlineStr"/>
+      <c r="M14" s="19" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="N14" s="18" t="inlineStr"/>
+      <c r="O14" s="18" t="inlineStr"/>
+      <c r="P14" s="18" t="inlineStr"/>
+      <c r="Q14" s="18" t="inlineStr"/>
+      <c r="R14" s="18" t="inlineStr"/>
+      <c r="S14" s="15" t="inlineStr">
         <is>
           <t>See FM-007, FM-009, FM-010 — all still open, to re-raise with Adil</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="60" customHeight="1">
-      <c r="A15" s="13" t="n">
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="14" t="inlineStr">
         <is>
           <t>A-ST-01d</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr"/>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="C15" s="14" t="inlineStr"/>
+      <c r="D15" s="14" t="inlineStr">
         <is>
           <t>Stone</t>
         </is>
       </c>
-      <c r="E15" s="14" t="inlineStr">
+      <c r="E15" s="15" t="inlineStr">
         <is>
           <t>Beige clair</t>
         </is>
       </c>
-      <c r="F15" s="14" t="inlineStr">
+      <c r="F15" s="15" t="inlineStr">
         <is>
           <t>Light beige stone</t>
         </is>
       </c>
-      <c r="G15" s="13" t="inlineStr">
+      <c r="G15" s="14" t="inlineStr">
         <is>
           <t>Anti-dérapant / Anti-slip</t>
         </is>
       </c>
-      <c r="H15" s="14" t="inlineStr">
+      <c r="H15" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-SDB-B/2, K5M-T1B1-SDB-B/5</t>
         </is>
       </c>
-      <c r="I15" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
               <color rgb="00292B2B"/>
               <sz val="1000"/>
             </rPr>
@@ -928,7 +938,7 @@
           </r>
           <r>
             <rPr>
-              <rFont val="Lato"/>
+              <rFont val="Calibri"/>
               <color rgb="00E4572E"/>
               <sz val="1000"/>
               <u val="single"/>
@@ -937,69 +947,73 @@
           </r>
         </is>
       </c>
-      <c r="J15" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K15" s="16" t="inlineStr">
+      <c r="J15" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K15" s="17" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L15" s="17" t="inlineStr"/>
-      <c r="M15" s="17" t="inlineStr"/>
-      <c r="N15" s="17" t="inlineStr"/>
-      <c r="O15" s="17" t="inlineStr"/>
-      <c r="P15" s="17" t="inlineStr"/>
-      <c r="Q15" s="17" t="inlineStr"/>
-      <c r="R15" s="17" t="inlineStr"/>
-      <c r="S15" s="14" t="inlineStr">
+      <c r="L15" s="18" t="inlineStr"/>
+      <c r="M15" s="19" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="N15" s="18" t="inlineStr"/>
+      <c r="O15" s="18" t="inlineStr"/>
+      <c r="P15" s="18" t="inlineStr"/>
+      <c r="Q15" s="18" t="inlineStr"/>
+      <c r="R15" s="18" t="inlineStr"/>
+      <c r="S15" s="15" t="inlineStr">
         <is>
           <t>See FM-005, FM-012</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="60" customHeight="1">
-      <c r="A16" s="13" t="n">
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B16" s="14" t="inlineStr">
         <is>
           <t>A-ST-01e</t>
         </is>
       </c>
-      <c r="C16" s="13" t="inlineStr"/>
-      <c r="D16" s="13" t="inlineStr">
+      <c r="C16" s="14" t="inlineStr"/>
+      <c r="D16" s="14" t="inlineStr">
         <is>
           <t>Stone</t>
         </is>
       </c>
-      <c r="E16" s="14" t="inlineStr">
+      <c r="E16" s="15" t="inlineStr">
         <is>
           <t>Beige clair</t>
         </is>
       </c>
-      <c r="F16" s="14" t="inlineStr">
+      <c r="F16" s="15" t="inlineStr">
         <is>
           <t>Light beige stone</t>
         </is>
       </c>
-      <c r="G16" s="13" t="inlineStr">
+      <c r="G16" s="14" t="inlineStr">
         <is>
           <t>Martelé / Hammered</t>
         </is>
       </c>
-      <c r="H16" s="14" t="inlineStr">
+      <c r="H16" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT-A/1, K5M-T1B1-SDB-B/1</t>
         </is>
       </c>
-      <c r="I16" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
+      <c r="I16" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
               <color rgb="00292B2B"/>
               <sz val="1000"/>
             </rPr>
@@ -1007,65 +1021,69 @@
           </r>
         </is>
       </c>
-      <c r="J16" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K16" s="16" t="inlineStr">
+      <c r="J16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K16" s="17" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L16" s="17" t="inlineStr"/>
-      <c r="M16" s="17" t="inlineStr"/>
-      <c r="N16" s="17" t="inlineStr"/>
-      <c r="O16" s="17" t="inlineStr"/>
-      <c r="P16" s="17" t="inlineStr"/>
-      <c r="Q16" s="17" t="inlineStr"/>
-      <c r="R16" s="17" t="inlineStr"/>
-      <c r="S16" s="14" t="inlineStr"/>
-    </row>
-    <row r="17" ht="60" customHeight="1">
-      <c r="A17" s="13" t="n">
+      <c r="L16" s="18" t="inlineStr"/>
+      <c r="M16" s="19" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="N16" s="18" t="inlineStr"/>
+      <c r="O16" s="18" t="inlineStr"/>
+      <c r="P16" s="18" t="inlineStr"/>
+      <c r="Q16" s="18" t="inlineStr"/>
+      <c r="R16" s="18" t="inlineStr"/>
+      <c r="S16" s="15" t="inlineStr"/>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B17" s="14" t="inlineStr">
         <is>
           <t>A-ST-02c</t>
         </is>
       </c>
-      <c r="C17" s="13" t="inlineStr"/>
-      <c r="D17" s="13" t="inlineStr">
+      <c r="C17" s="14" t="inlineStr"/>
+      <c r="D17" s="14" t="inlineStr">
         <is>
           <t>Stone</t>
         </is>
       </c>
-      <c r="E17" s="14" t="inlineStr">
+      <c r="E17" s="15" t="inlineStr">
         <is>
           <t>Beige foncé</t>
         </is>
       </c>
-      <c r="F17" s="14" t="inlineStr">
+      <c r="F17" s="15" t="inlineStr">
         <is>
           <t>Dark beige stone</t>
         </is>
       </c>
-      <c r="G17" s="13" t="inlineStr">
+      <c r="G17" s="14" t="inlineStr">
         <is>
           <t>Adouci / Honed</t>
         </is>
       </c>
-      <c r="H17" s="14" t="inlineStr">
+      <c r="H17" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT-A/1, K5M-T1B1-SDB-B/1, K5M-T1B1-SDB-B/3, K5M-T1B1-CHA-C/2</t>
         </is>
       </c>
-      <c r="I17" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
               <color rgb="00292B2B"/>
               <sz val="1000"/>
             </rPr>
@@ -1073,7 +1091,7 @@
           </r>
           <r>
             <rPr>
-              <rFont val="Lato"/>
+              <rFont val="Calibri"/>
               <color rgb="00E4572E"/>
               <sz val="1000"/>
               <u val="single"/>
@@ -1082,69 +1100,73 @@
           </r>
         </is>
       </c>
-      <c r="J17" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K17" s="16" t="inlineStr">
+      <c r="J17" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K17" s="17" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L17" s="17" t="inlineStr"/>
-      <c r="M17" s="17" t="inlineStr"/>
-      <c r="N17" s="17" t="inlineStr"/>
-      <c r="O17" s="17" t="inlineStr"/>
-      <c r="P17" s="17" t="inlineStr"/>
-      <c r="Q17" s="17" t="inlineStr"/>
-      <c r="R17" s="17" t="inlineStr"/>
-      <c r="S17" s="14" t="inlineStr">
+      <c r="L17" s="18" t="inlineStr"/>
+      <c r="M17" s="19" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="N17" s="18" t="inlineStr"/>
+      <c r="O17" s="18" t="inlineStr"/>
+      <c r="P17" s="18" t="inlineStr"/>
+      <c r="Q17" s="18" t="inlineStr"/>
+      <c r="R17" s="18" t="inlineStr"/>
+      <c r="S17" s="15" t="inlineStr">
         <is>
           <t>See FM-009</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="60" customHeight="1">
-      <c r="A18" s="13" t="n">
+    <row r="18" ht="62" customHeight="1">
+      <c r="A18" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>A-ST-07a</t>
         </is>
       </c>
-      <c r="C18" s="13" t="inlineStr"/>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="C18" s="14" t="inlineStr"/>
+      <c r="D18" s="14" t="inlineStr">
         <is>
           <t>Stone</t>
         </is>
       </c>
-      <c r="E18" s="14" t="inlineStr">
+      <c r="E18" s="15" t="inlineStr">
         <is>
           <t>Onyx miel — REMPLACÉ PAR Taj Mahal</t>
         </is>
       </c>
-      <c r="F18" s="14" t="inlineStr">
+      <c r="F18" s="15" t="inlineStr">
         <is>
           <t>Onyx Honey — REPLACED BY Taj Mahal</t>
         </is>
       </c>
-      <c r="G18" s="13" t="inlineStr">
+      <c r="G18" s="14" t="inlineStr">
         <is>
           <t>Poli / Polished</t>
         </is>
       </c>
-      <c r="H18" s="14" t="inlineStr">
+      <c r="H18" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT-A (arche/porte-bagage), K5M-T1B1-SDB-B/7, K5M-T1B1-SDB-B/8, K5M-T1B1-SDB-B/9, K5M-T1B1-SDB-B/10, K5M-T1B1-SDB-B/11, K5M-T1B1-SDB-B/12, K5M-T1B1-CHA-C/4</t>
         </is>
       </c>
-      <c r="I18" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
+      <c r="I18" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
               <color rgb="00292B2B"/>
               <sz val="1000"/>
             </rPr>
@@ -1152,7 +1174,7 @@
           </r>
           <r>
             <rPr>
-              <rFont val="Lato"/>
+              <rFont val="Calibri"/>
               <color rgb="00E4572E"/>
               <sz val="1000"/>
               <u val="single"/>
@@ -1161,7 +1183,7 @@
           </r>
           <r>
             <rPr>
-              <rFont val="Lato"/>
+              <rFont val="Calibri"/>
               <color rgb="00292B2B"/>
               <sz val="1000"/>
             </rPr>
@@ -1169,69 +1191,73 @@
           </r>
         </is>
       </c>
-      <c r="J18" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K18" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L18" s="17" t="inlineStr"/>
-      <c r="M18" s="17" t="inlineStr"/>
-      <c r="N18" s="17" t="inlineStr"/>
-      <c r="O18" s="17" t="inlineStr"/>
-      <c r="P18" s="17" t="inlineStr"/>
-      <c r="Q18" s="17" t="inlineStr"/>
-      <c r="R18" s="17" t="inlineStr"/>
-      <c r="S18" s="14" t="inlineStr">
+      <c r="J18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr"/>
+      <c r="M18" s="19" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="N18" s="18" t="inlineStr"/>
+      <c r="O18" s="18" t="inlineStr"/>
+      <c r="P18" s="18" t="inlineStr"/>
+      <c r="Q18" s="18" t="inlineStr"/>
+      <c r="R18" s="18" t="inlineStr"/>
+      <c r="S18" s="15" t="inlineStr">
         <is>
           <t>SUBSTITUTED as of 21 Jul 2026 update. See FM-002, FM-007 — confirm Taj Mahal applies everywhere, honey onyx no longer valid anywhere</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="60" customHeight="1">
-      <c r="A19" s="13" t="n">
+    <row r="19" ht="48" customHeight="1">
+      <c r="A19" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="B19" s="13" t="inlineStr">
+      <c r="B19" s="14" t="inlineStr">
         <is>
           <t>A-WD-01b</t>
         </is>
       </c>
-      <c r="C19" s="13" t="inlineStr"/>
-      <c r="D19" s="13" t="inlineStr">
+      <c r="C19" s="14" t="inlineStr"/>
+      <c r="D19" s="14" t="inlineStr">
         <is>
           <t>Wood</t>
         </is>
       </c>
-      <c r="E19" s="14" t="inlineStr">
+      <c r="E19" s="15" t="inlineStr">
         <is>
           <t>Noyer — REMPLACÉ PAR chêne teinté moyen</t>
         </is>
       </c>
-      <c r="F19" s="14" t="inlineStr">
+      <c r="F19" s="15" t="inlineStr">
         <is>
           <t>Walnut — REPLACED BY medium-tinted oak</t>
         </is>
       </c>
-      <c r="G19" s="13" t="inlineStr">
+      <c r="G19" s="14" t="inlineStr">
         <is>
           <t>Satin</t>
         </is>
       </c>
-      <c r="H19" s="14" t="inlineStr">
+      <c r="H19" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT-A/7, K5M-T1B1-CHA-C/7</t>
         </is>
       </c>
-      <c r="I19" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
               <color rgb="00E4572E"/>
               <sz val="1000"/>
               <u val="single"/>
@@ -1240,7 +1266,7 @@
           </r>
           <r>
             <rPr>
-              <rFont val="Lato"/>
+              <rFont val="Calibri"/>
               <color rgb="00E4572E"/>
               <sz val="1000"/>
               <u val="single"/>
@@ -1249,65 +1275,69 @@
           </r>
         </is>
       </c>
-      <c r="J19" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K19" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L19" s="17" t="inlineStr"/>
-      <c r="M19" s="17" t="inlineStr"/>
-      <c r="N19" s="17" t="inlineStr"/>
-      <c r="O19" s="17" t="inlineStr"/>
-      <c r="P19" s="17" t="inlineStr"/>
-      <c r="Q19" s="17" t="inlineStr"/>
-      <c r="R19" s="17" t="inlineStr"/>
-      <c r="S19" s="14" t="inlineStr">
+      <c r="J19" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K19" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L19" s="18" t="inlineStr"/>
+      <c r="M19" s="19" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="N19" s="18" t="inlineStr"/>
+      <c r="O19" s="18" t="inlineStr"/>
+      <c r="P19" s="18" t="inlineStr"/>
+      <c r="Q19" s="18" t="inlineStr"/>
+      <c r="R19" s="18" t="inlineStr"/>
+      <c r="S19" s="15" t="inlineStr">
         <is>
           <t>SUBSTITUTED as of 21 Jul 2026. See FM-001 — confirm all four applications follow this code/finish</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="60" customHeight="1">
-      <c r="A20" s="13" t="n">
+    <row r="20" ht="34" customHeight="1">
+      <c r="A20" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="B20" s="13" t="inlineStr">
+      <c r="B20" s="14" t="inlineStr">
         <is>
           <t>A-WD-01d</t>
         </is>
       </c>
-      <c r="C20" s="13" t="inlineStr"/>
-      <c r="D20" s="13" t="inlineStr">
+      <c r="C20" s="14" t="inlineStr"/>
+      <c r="D20" s="14" t="inlineStr">
         <is>
           <t>Wood</t>
         </is>
       </c>
-      <c r="E20" s="14" t="inlineStr">
+      <c r="E20" s="15" t="inlineStr">
         <is>
           <t>(absent de la liste officielle des matériaux)</t>
         </is>
       </c>
-      <c r="F20" s="14" t="inlineStr">
+      <c r="F20" s="15" t="inlineStr">
         <is>
           <t>(does not appear in the official material list at all)</t>
         </is>
       </c>
-      <c r="G20" s="13" t="inlineStr"/>
-      <c r="H20" s="14" t="inlineStr">
+      <c r="G20" s="14" t="inlineStr"/>
+      <c r="H20" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT-A/2, K5M-T1B1-ENT-A/4</t>
         </is>
       </c>
-      <c r="I20" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
+      <c r="I20" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
               <color rgb="00E4572E"/>
               <sz val="1000"/>
               <u val="single"/>
@@ -1316,69 +1346,73 @@
           </r>
         </is>
       </c>
-      <c r="J20" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K20" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L20" s="17" t="inlineStr"/>
-      <c r="M20" s="17" t="inlineStr"/>
-      <c r="N20" s="17" t="inlineStr"/>
-      <c r="O20" s="17" t="inlineStr"/>
-      <c r="P20" s="17" t="inlineStr"/>
-      <c r="Q20" s="17" t="inlineStr"/>
-      <c r="R20" s="17" t="inlineStr"/>
-      <c r="S20" s="14" t="inlineStr">
+      <c r="J20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L20" s="18" t="inlineStr"/>
+      <c r="M20" s="19" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="N20" s="18" t="inlineStr"/>
+      <c r="O20" s="18" t="inlineStr"/>
+      <c r="P20" s="18" t="inlineStr"/>
+      <c r="Q20" s="18" t="inlineStr"/>
+      <c r="R20" s="18" t="inlineStr"/>
+      <c r="S20" s="15" t="inlineStr">
         <is>
           <t>See FM-001. RFI already flags: no material reference image provided for this code</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="60" customHeight="1">
-      <c r="A21" s="13" t="n">
+    <row r="21" ht="48" customHeight="1">
+      <c r="A21" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B21" s="14" t="inlineStr">
         <is>
           <t>A-WD-02c</t>
         </is>
       </c>
-      <c r="C21" s="13" t="inlineStr"/>
-      <c r="D21" s="13" t="inlineStr">
+      <c r="C21" s="14" t="inlineStr"/>
+      <c r="D21" s="14" t="inlineStr">
         <is>
           <t>Wood</t>
         </is>
       </c>
-      <c r="E21" s="14" t="inlineStr">
+      <c r="E21" s="15" t="inlineStr">
         <is>
           <t>Chêne cérusé blanc</t>
         </is>
       </c>
-      <c r="F21" s="14" t="inlineStr">
+      <c r="F21" s="15" t="inlineStr">
         <is>
           <t>White cerused oak</t>
         </is>
       </c>
-      <c r="G21" s="13" t="inlineStr">
+      <c r="G21" s="14" t="inlineStr">
         <is>
           <t>Mat / Matte</t>
         </is>
       </c>
-      <c r="H21" s="14" t="inlineStr">
+      <c r="H21" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT-A/8, K5M-T1B1-SDB-B/14, K5M-T1B1-CHA-C/6</t>
         </is>
       </c>
-      <c r="I21" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
+      <c r="I21" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
               <color rgb="00292B2B"/>
               <sz val="1000"/>
             </rPr>
@@ -1386,7 +1420,7 @@
           </r>
           <r>
             <rPr>
-              <rFont val="Lato"/>
+              <rFont val="Calibri"/>
               <color rgb="00E4572E"/>
               <sz val="1000"/>
               <u val="single"/>
@@ -1395,69 +1429,73 @@
           </r>
         </is>
       </c>
-      <c r="J21" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K21" s="16" t="inlineStr">
+      <c r="J21" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K21" s="17" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L21" s="17" t="inlineStr"/>
-      <c r="M21" s="17" t="inlineStr"/>
-      <c r="N21" s="17" t="inlineStr"/>
-      <c r="O21" s="17" t="inlineStr"/>
-      <c r="P21" s="17" t="inlineStr"/>
-      <c r="Q21" s="17" t="inlineStr"/>
-      <c r="R21" s="17" t="inlineStr"/>
-      <c r="S21" s="14" t="inlineStr">
+      <c r="L21" s="18" t="inlineStr"/>
+      <c r="M21" s="19" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="N21" s="18" t="inlineStr"/>
+      <c r="O21" s="18" t="inlineStr"/>
+      <c r="P21" s="18" t="inlineStr"/>
+      <c r="Q21" s="18" t="inlineStr"/>
+      <c r="R21" s="18" t="inlineStr"/>
+      <c r="S21" s="15" t="inlineStr">
         <is>
           <t>See FM-011</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="60" customHeight="1">
-      <c r="A22" s="13" t="n">
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B22" s="14" t="inlineStr">
         <is>
           <t>A-WD-04b</t>
         </is>
       </c>
-      <c r="C22" s="13" t="inlineStr"/>
-      <c r="D22" s="13" t="inlineStr">
+      <c r="C22" s="14" t="inlineStr"/>
+      <c r="D22" s="14" t="inlineStr">
         <is>
           <t>Wood</t>
         </is>
       </c>
-      <c r="E22" s="14" t="inlineStr">
+      <c r="E22" s="15" t="inlineStr">
         <is>
           <t>Parquet chêne teinté moyen (Hakwood Idéal)</t>
         </is>
       </c>
-      <c r="F22" s="14" t="inlineStr">
+      <c r="F22" s="15" t="inlineStr">
         <is>
           <t>Medium-tinted oak parquet (Hakwood Idéal)</t>
         </is>
       </c>
-      <c r="G22" s="13" t="inlineStr">
+      <c r="G22" s="14" t="inlineStr">
         <is>
           <t>Satin</t>
         </is>
       </c>
-      <c r="H22" s="14" t="inlineStr">
+      <c r="H22" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-CHA-C/1</t>
         </is>
       </c>
-      <c r="I22" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
+      <c r="I22" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
               <color rgb="00E4572E"/>
               <sz val="1000"/>
               <u val="single"/>
@@ -1466,7 +1504,7 @@
           </r>
           <r>
             <rPr>
-              <rFont val="Lato"/>
+              <rFont val="Calibri"/>
               <color rgb="00E4572E"/>
               <sz val="1000"/>
               <u val="single"/>
@@ -1475,69 +1513,73 @@
           </r>
         </is>
       </c>
-      <c r="J22" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K22" s="16" t="inlineStr">
+      <c r="J22" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K22" s="17" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L22" s="17" t="inlineStr"/>
-      <c r="M22" s="17" t="inlineStr"/>
-      <c r="N22" s="17" t="inlineStr"/>
-      <c r="O22" s="17" t="inlineStr"/>
-      <c r="P22" s="17" t="inlineStr"/>
-      <c r="Q22" s="17" t="inlineStr"/>
-      <c r="R22" s="17" t="inlineStr"/>
-      <c r="S22" s="14" t="inlineStr">
+      <c r="L22" s="18" t="inlineStr"/>
+      <c r="M22" s="19" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="N22" s="18" t="inlineStr"/>
+      <c r="O22" s="18" t="inlineStr"/>
+      <c r="P22" s="18" t="inlineStr"/>
+      <c r="Q22" s="18" t="inlineStr"/>
+      <c r="R22" s="18" t="inlineStr"/>
+      <c r="S22" s="15" t="inlineStr">
         <is>
           <t>SUBSTITUTED from dark-tinted to medium-tinted oak, 21 Jul 2026, real product ref (Hakwood, Idéal). See FM-008</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="60" customHeight="1">
-      <c r="A23" s="13" t="n">
+    <row r="23" ht="62" customHeight="1">
+      <c r="A23" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B23" s="14" t="inlineStr">
         <is>
           <t>A-ME-01a</t>
         </is>
       </c>
-      <c r="C23" s="13" t="inlineStr"/>
-      <c r="D23" s="13" t="inlineStr">
+      <c r="C23" s="14" t="inlineStr"/>
+      <c r="D23" s="14" t="inlineStr">
         <is>
           <t>Metal</t>
         </is>
       </c>
-      <c r="E23" s="14" t="inlineStr">
+      <c r="E23" s="15" t="inlineStr">
         <is>
           <t>Acier inoxydable poli</t>
         </is>
       </c>
-      <c r="F23" s="14" t="inlineStr">
+      <c r="F23" s="15" t="inlineStr">
         <is>
           <t>Polished stainless steel</t>
         </is>
       </c>
-      <c r="G23" s="13" t="inlineStr">
+      <c r="G23" s="14" t="inlineStr">
         <is>
           <t>Finition poli miroir</t>
         </is>
       </c>
-      <c r="H23" s="14" t="inlineStr">
+      <c r="H23" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-SDB-B/8, K5M-T1B1-SDB-B/14</t>
         </is>
       </c>
-      <c r="I23" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
+      <c r="I23" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
               <color rgb="00E4572E"/>
               <sz val="1000"/>
               <u val="single"/>
@@ -1546,7 +1588,7 @@
           </r>
           <r>
             <rPr>
-              <rFont val="Lato"/>
+              <rFont val="Calibri"/>
               <color rgb="00E4572E"/>
               <sz val="1000"/>
               <u val="single"/>
@@ -1555,69 +1597,73 @@
           </r>
         </is>
       </c>
-      <c r="J23" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K23" s="16" t="inlineStr">
+      <c r="J23" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K23" s="17" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L23" s="17" t="inlineStr"/>
-      <c r="M23" s="17" t="inlineStr"/>
-      <c r="N23" s="17" t="inlineStr"/>
-      <c r="O23" s="17" t="inlineStr"/>
-      <c r="P23" s="17" t="inlineStr"/>
-      <c r="Q23" s="17" t="inlineStr"/>
-      <c r="R23" s="17" t="inlineStr"/>
-      <c r="S23" s="14" t="inlineStr">
+      <c r="L23" s="18" t="inlineStr"/>
+      <c r="M23" s="19" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="N23" s="18" t="inlineStr"/>
+      <c r="O23" s="18" t="inlineStr"/>
+      <c r="P23" s="18" t="inlineStr"/>
+      <c r="Q23" s="18" t="inlineStr"/>
+      <c r="R23" s="18" t="inlineStr"/>
+      <c r="S23" s="15" t="inlineStr">
         <is>
           <t>See FM-006. Location changed between material list versions — confirm current assignment</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="60" customHeight="1">
-      <c r="A24" s="13" t="n">
+    <row r="24" ht="34" customHeight="1">
+      <c r="A24" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B24" s="14" t="inlineStr">
         <is>
           <t>A-ME-01h</t>
         </is>
       </c>
-      <c r="C24" s="13" t="inlineStr"/>
-      <c r="D24" s="13" t="inlineStr">
+      <c r="C24" s="14" t="inlineStr"/>
+      <c r="D24" s="14" t="inlineStr">
         <is>
           <t>Metal</t>
         </is>
       </c>
-      <c r="E24" s="14" t="inlineStr">
+      <c r="E24" s="15" t="inlineStr">
         <is>
           <t>Acier inoxydable brossé (NOUVEAU 21 Jul)</t>
         </is>
       </c>
-      <c r="F24" s="14" t="inlineStr">
+      <c r="F24" s="15" t="inlineStr">
         <is>
           <t>Brushed stainless steel (NEW 21 Jul)</t>
         </is>
       </c>
-      <c r="G24" s="13" t="inlineStr">
+      <c r="G24" s="14" t="inlineStr">
         <is>
           <t>Finition brossé</t>
         </is>
       </c>
-      <c r="H24" s="14" t="inlineStr">
+      <c r="H24" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT</t>
         </is>
       </c>
-      <c r="I24" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
+      <c r="I24" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
               <color rgb="00E4572E"/>
               <sz val="1000"/>
               <u val="single"/>
@@ -1626,69 +1672,73 @@
           </r>
         </is>
       </c>
-      <c r="J24" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K24" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L24" s="17" t="inlineStr"/>
-      <c r="M24" s="17" t="inlineStr"/>
-      <c r="N24" s="17" t="inlineStr"/>
-      <c r="O24" s="17" t="inlineStr"/>
-      <c r="P24" s="17" t="inlineStr"/>
-      <c r="Q24" s="17" t="inlineStr"/>
-      <c r="R24" s="17" t="inlineStr"/>
-      <c r="S24" s="14" t="inlineStr">
+      <c r="J24" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K24" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L24" s="18" t="inlineStr"/>
+      <c r="M24" s="19" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="N24" s="18" t="inlineStr"/>
+      <c r="O24" s="18" t="inlineStr"/>
+      <c r="P24" s="18" t="inlineStr"/>
+      <c r="Q24" s="18" t="inlineStr"/>
+      <c r="R24" s="18" t="inlineStr"/>
+      <c r="S24" s="15" t="inlineStr">
         <is>
           <t>New code as of 21 Jul 2026 update — confirm with Adil this is the correct replacement for the rail location</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="60" customHeight="1">
-      <c r="A25" s="13" t="n">
+    <row r="25" ht="34" customHeight="1">
+      <c r="A25" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="B25" s="13" t="inlineStr">
+      <c r="B25" s="14" t="inlineStr">
         <is>
           <t>A-ME-02h</t>
         </is>
       </c>
-      <c r="C25" s="13" t="inlineStr"/>
-      <c r="D25" s="13" t="inlineStr">
+      <c r="C25" s="14" t="inlineStr"/>
+      <c r="D25" s="14" t="inlineStr">
         <is>
           <t>Metal</t>
         </is>
       </c>
-      <c r="E25" s="14" t="inlineStr">
+      <c r="E25" s="15" t="inlineStr">
         <is>
           <t>Laiton patiné foncé</t>
         </is>
       </c>
-      <c r="F25" s="14" t="inlineStr">
+      <c r="F25" s="15" t="inlineStr">
         <is>
           <t>Dark patinated brass</t>
         </is>
       </c>
-      <c r="G25" s="13" t="inlineStr">
+      <c r="G25" s="14" t="inlineStr">
         <is>
           <t>Vernis mat / Matte varnish</t>
         </is>
       </c>
-      <c r="H25" s="14" t="inlineStr">
+      <c r="H25" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT-A/7, K5M-T1B1-ENT-A/8, K5M-T1B1-SDB-B/13, K5M-T1B1-CHA-C/7</t>
         </is>
       </c>
-      <c r="I25" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
+      <c r="I25" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
               <color rgb="00292B2B"/>
               <sz val="1000"/>
             </rPr>
@@ -1696,65 +1746,69 @@
           </r>
         </is>
       </c>
-      <c r="J25" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K25" s="16" t="inlineStr">
+      <c r="J25" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K25" s="17" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L25" s="17" t="inlineStr"/>
-      <c r="M25" s="17" t="inlineStr"/>
-      <c r="N25" s="17" t="inlineStr"/>
-      <c r="O25" s="17" t="inlineStr"/>
-      <c r="P25" s="17" t="inlineStr"/>
-      <c r="Q25" s="17" t="inlineStr"/>
-      <c r="R25" s="17" t="inlineStr"/>
-      <c r="S25" s="14" t="inlineStr"/>
-    </row>
-    <row r="26" ht="60" customHeight="1">
-      <c r="A26" s="13" t="n">
+      <c r="L25" s="18" t="inlineStr"/>
+      <c r="M25" s="19" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="N25" s="18" t="inlineStr"/>
+      <c r="O25" s="18" t="inlineStr"/>
+      <c r="P25" s="18" t="inlineStr"/>
+      <c r="Q25" s="18" t="inlineStr"/>
+      <c r="R25" s="18" t="inlineStr"/>
+      <c r="S25" s="15" t="inlineStr"/>
+    </row>
+    <row r="26" ht="34" customHeight="1">
+      <c r="A26" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="B26" s="13" t="inlineStr">
+      <c r="B26" s="14" t="inlineStr">
         <is>
           <t>A-ME-02i</t>
         </is>
       </c>
-      <c r="C26" s="13" t="inlineStr"/>
-      <c r="D26" s="13" t="inlineStr">
+      <c r="C26" s="14" t="inlineStr"/>
+      <c r="D26" s="14" t="inlineStr">
         <is>
           <t>Metal</t>
         </is>
       </c>
-      <c r="E26" s="14" t="inlineStr">
+      <c r="E26" s="15" t="inlineStr">
         <is>
           <t>Laiton patiné foncé martelé</t>
         </is>
       </c>
-      <c r="F26" s="14" t="inlineStr">
+      <c r="F26" s="15" t="inlineStr">
         <is>
           <t>Dark patinated hammered brass</t>
         </is>
       </c>
-      <c r="G26" s="13" t="inlineStr">
+      <c r="G26" s="14" t="inlineStr">
         <is>
           <t>Martelé, vernis mat</t>
         </is>
       </c>
-      <c r="H26" s="14" t="inlineStr">
+      <c r="H26" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT-A/8, K5M-T1B1-SDB-B/14</t>
         </is>
       </c>
-      <c r="I26" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
+      <c r="I26" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
               <color rgb="00292B2B"/>
               <sz val="1000"/>
             </rPr>
@@ -1762,69 +1816,73 @@
           </r>
         </is>
       </c>
-      <c r="J26" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K26" s="16" t="inlineStr">
+      <c r="J26" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K26" s="17" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L26" s="17" t="inlineStr"/>
-      <c r="M26" s="17" t="inlineStr"/>
-      <c r="N26" s="17" t="inlineStr"/>
-      <c r="O26" s="17" t="inlineStr"/>
-      <c r="P26" s="17" t="inlineStr"/>
-      <c r="Q26" s="17" t="inlineStr"/>
-      <c r="R26" s="17" t="inlineStr"/>
-      <c r="S26" s="14" t="inlineStr">
+      <c r="L26" s="18" t="inlineStr"/>
+      <c r="M26" s="19" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="N26" s="18" t="inlineStr"/>
+      <c r="O26" s="18" t="inlineStr"/>
+      <c r="P26" s="18" t="inlineStr"/>
+      <c r="Q26" s="18" t="inlineStr"/>
+      <c r="R26" s="18" t="inlineStr"/>
+      <c r="S26" s="15" t="inlineStr">
         <is>
           <t>Compound finish: dark patina base + hammered (martelé) texture applied on top — the only clear compound case in Fit-out</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="60" customHeight="1">
-      <c r="A27" s="13" t="n">
+    <row r="27" ht="34" customHeight="1">
+      <c r="A27" s="14" t="n">
         <v>14</v>
       </c>
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B27" s="14" t="inlineStr">
         <is>
           <t>A-GL-01a</t>
         </is>
       </c>
-      <c r="C27" s="13" t="inlineStr"/>
-      <c r="D27" s="13" t="inlineStr">
+      <c r="C27" s="14" t="inlineStr"/>
+      <c r="D27" s="14" t="inlineStr">
         <is>
           <t>Glass/Mirror</t>
         </is>
       </c>
-      <c r="E27" s="14" t="inlineStr">
+      <c r="E27" s="15" t="inlineStr">
         <is>
           <t>Miroir extra-clair</t>
         </is>
       </c>
-      <c r="F27" s="14" t="inlineStr">
+      <c r="F27" s="15" t="inlineStr">
         <is>
           <t>Extra-clear mirror</t>
         </is>
       </c>
-      <c r="G27" s="13" t="inlineStr">
+      <c r="G27" s="14" t="inlineStr">
         <is>
           <t>Extra-clair</t>
         </is>
       </c>
-      <c r="H27" s="14" t="inlineStr">
+      <c r="H27" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-SDB-B/13, K5M-T1B1-CHA-C/7</t>
         </is>
       </c>
-      <c r="I27" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
+      <c r="I27" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
               <color rgb="00E4572E"/>
               <sz val="1000"/>
               <u val="single"/>
@@ -1833,69 +1891,73 @@
           </r>
         </is>
       </c>
-      <c r="J27" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K27" s="16" t="inlineStr">
+      <c r="J27" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K27" s="17" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L27" s="17" t="inlineStr"/>
-      <c r="M27" s="17" t="inlineStr"/>
-      <c r="N27" s="17" t="inlineStr"/>
-      <c r="O27" s="17" t="inlineStr"/>
-      <c r="P27" s="17" t="inlineStr"/>
-      <c r="Q27" s="17" t="inlineStr"/>
-      <c r="R27" s="17" t="inlineStr"/>
-      <c r="S27" s="14" t="inlineStr">
+      <c r="L27" s="18" t="inlineStr"/>
+      <c r="M27" s="19" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="N27" s="18" t="inlineStr"/>
+      <c r="O27" s="18" t="inlineStr"/>
+      <c r="P27" s="18" t="inlineStr"/>
+      <c r="Q27" s="18" t="inlineStr"/>
+      <c r="R27" s="18" t="inlineStr"/>
+      <c r="S27" s="15" t="inlineStr">
         <is>
           <t>Confirm scope boundary on B/13's inter-panel lighting (per RFI remark)</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="60" customHeight="1">
-      <c r="A28" s="13" t="n">
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="B28" s="13" t="inlineStr">
+      <c r="B28" s="14" t="inlineStr">
         <is>
           <t>A-GL-02a</t>
         </is>
       </c>
-      <c r="C28" s="13" t="inlineStr"/>
-      <c r="D28" s="13" t="inlineStr">
+      <c r="C28" s="14" t="inlineStr"/>
+      <c r="D28" s="14" t="inlineStr">
         <is>
           <t>Glass/Mirror</t>
         </is>
       </c>
-      <c r="E28" s="14" t="inlineStr">
+      <c r="E28" s="15" t="inlineStr">
         <is>
           <t>Miroir extra-clair antique</t>
         </is>
       </c>
-      <c r="F28" s="14" t="inlineStr">
+      <c r="F28" s="15" t="inlineStr">
         <is>
           <t>Antique extra-clear mirror</t>
         </is>
       </c>
-      <c r="G28" s="13" t="inlineStr">
+      <c r="G28" s="14" t="inlineStr">
         <is>
           <t>Antique</t>
         </is>
       </c>
-      <c r="H28" s="14" t="inlineStr">
+      <c r="H28" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT</t>
         </is>
       </c>
-      <c r="I28" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
+      <c r="I28" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
               <color rgb="00292B2B"/>
               <sz val="1000"/>
             </rPr>
@@ -1903,61 +1965,65 @@
           </r>
         </is>
       </c>
-      <c r="J28" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K28" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L28" s="17" t="inlineStr"/>
-      <c r="M28" s="17" t="inlineStr"/>
-      <c r="N28" s="17" t="inlineStr"/>
-      <c r="O28" s="17" t="inlineStr"/>
-      <c r="P28" s="17" t="inlineStr"/>
-      <c r="Q28" s="17" t="inlineStr"/>
-      <c r="R28" s="17" t="inlineStr"/>
-      <c r="S28" s="14" t="inlineStr"/>
-    </row>
-    <row r="29" ht="60" customHeight="1">
-      <c r="A29" s="13" t="n">
+      <c r="J28" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K28" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L28" s="18" t="inlineStr"/>
+      <c r="M28" s="19" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="N28" s="18" t="inlineStr"/>
+      <c r="O28" s="18" t="inlineStr"/>
+      <c r="P28" s="18" t="inlineStr"/>
+      <c r="Q28" s="18" t="inlineStr"/>
+      <c r="R28" s="18" t="inlineStr"/>
+      <c r="S28" s="15" t="inlineStr"/>
+    </row>
+    <row r="29" ht="34" customHeight="1">
+      <c r="A29" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="B29" s="14" t="inlineStr">
         <is>
           <t>A-GL-03a</t>
         </is>
       </c>
-      <c r="C29" s="13" t="inlineStr"/>
-      <c r="D29" s="13" t="inlineStr">
+      <c r="C29" s="14" t="inlineStr"/>
+      <c r="D29" s="14" t="inlineStr">
         <is>
           <t>Glass</t>
         </is>
       </c>
-      <c r="E29" s="14" t="inlineStr">
+      <c r="E29" s="15" t="inlineStr">
         <is>
           <t>Verre extra-clair + lin</t>
         </is>
       </c>
-      <c r="F29" s="14" t="inlineStr">
+      <c r="F29" s="15" t="inlineStr">
         <is>
           <t>Extra-clear glass + linen</t>
         </is>
       </c>
-      <c r="G29" s="13" t="inlineStr"/>
-      <c r="H29" s="14" t="inlineStr">
+      <c r="G29" s="14" t="inlineStr"/>
+      <c r="H29" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT-A/8, K5M-T1B1-SDB-B/14</t>
         </is>
       </c>
-      <c r="I29" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
+      <c r="I29" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
               <color rgb="00E4572E"/>
               <sz val="1000"/>
               <u val="single"/>
@@ -1966,61 +2032,65 @@
           </r>
         </is>
       </c>
-      <c r="J29" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K29" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L29" s="17" t="inlineStr"/>
-      <c r="M29" s="17" t="inlineStr"/>
-      <c r="N29" s="17" t="inlineStr"/>
-      <c r="O29" s="17" t="inlineStr"/>
-      <c r="P29" s="17" t="inlineStr"/>
-      <c r="Q29" s="17" t="inlineStr"/>
-      <c r="R29" s="17" t="inlineStr"/>
-      <c r="S29" s="14" t="inlineStr"/>
-    </row>
-    <row r="30" ht="60" customHeight="1">
-      <c r="A30" s="13" t="n">
+      <c r="J29" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K29" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L29" s="18" t="inlineStr"/>
+      <c r="M29" s="19" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="N29" s="18" t="inlineStr"/>
+      <c r="O29" s="18" t="inlineStr"/>
+      <c r="P29" s="18" t="inlineStr"/>
+      <c r="Q29" s="18" t="inlineStr"/>
+      <c r="R29" s="18" t="inlineStr"/>
+      <c r="S29" s="15" t="inlineStr"/>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="14" t="n">
         <v>17</v>
       </c>
-      <c r="B30" s="13" t="inlineStr">
+      <c r="B30" s="14" t="inlineStr">
         <is>
           <t>A-GL-04a</t>
         </is>
       </c>
-      <c r="C30" s="13" t="inlineStr"/>
-      <c r="D30" s="13" t="inlineStr">
+      <c r="C30" s="14" t="inlineStr"/>
+      <c r="D30" s="14" t="inlineStr">
         <is>
           <t>Glass</t>
         </is>
       </c>
-      <c r="E30" s="14" t="inlineStr">
+      <c r="E30" s="15" t="inlineStr">
         <is>
           <t>Verre extra-clair</t>
         </is>
       </c>
-      <c r="F30" s="14" t="inlineStr">
+      <c r="F30" s="15" t="inlineStr">
         <is>
           <t>Extra-clear glass</t>
         </is>
       </c>
-      <c r="G30" s="13" t="inlineStr"/>
-      <c r="H30" s="14" t="inlineStr">
+      <c r="G30" s="14" t="inlineStr"/>
+      <c r="H30" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-SDB</t>
         </is>
       </c>
-      <c r="I30" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
+      <c r="I30" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
               <color rgb="00292B2B"/>
               <sz val="1000"/>
             </rPr>
@@ -2028,61 +2098,65 @@
           </r>
         </is>
       </c>
-      <c r="J30" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K30" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L30" s="17" t="inlineStr"/>
-      <c r="M30" s="17" t="inlineStr"/>
-      <c r="N30" s="17" t="inlineStr"/>
-      <c r="O30" s="17" t="inlineStr"/>
-      <c r="P30" s="17" t="inlineStr"/>
-      <c r="Q30" s="17" t="inlineStr"/>
-      <c r="R30" s="17" t="inlineStr"/>
-      <c r="S30" s="14" t="inlineStr"/>
-    </row>
-    <row r="31" ht="60" customHeight="1">
-      <c r="A31" s="13" t="n">
+      <c r="J30" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K30" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L30" s="18" t="inlineStr"/>
+      <c r="M30" s="19" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="N30" s="18" t="inlineStr"/>
+      <c r="O30" s="18" t="inlineStr"/>
+      <c r="P30" s="18" t="inlineStr"/>
+      <c r="Q30" s="18" t="inlineStr"/>
+      <c r="R30" s="18" t="inlineStr"/>
+      <c r="S30" s="15" t="inlineStr"/>
+    </row>
+    <row r="31" ht="34" customHeight="1">
+      <c r="A31" s="14" t="n">
         <v>18</v>
       </c>
-      <c r="B31" s="13" t="inlineStr">
+      <c r="B31" s="14" t="inlineStr">
         <is>
           <t>A-PT-01</t>
         </is>
       </c>
-      <c r="C31" s="13" t="inlineStr"/>
-      <c r="D31" s="13" t="inlineStr">
+      <c r="C31" s="14" t="inlineStr"/>
+      <c r="D31" s="14" t="inlineStr">
         <is>
           <t>Paint</t>
         </is>
       </c>
-      <c r="E31" s="14" t="inlineStr">
+      <c r="E31" s="15" t="inlineStr">
         <is>
           <t>Peinture texturée blanche</t>
         </is>
       </c>
-      <c r="F31" s="14" t="inlineStr">
+      <c r="F31" s="15" t="inlineStr">
         <is>
           <t>White textured paint</t>
         </is>
       </c>
-      <c r="G31" s="13" t="inlineStr"/>
-      <c r="H31" s="14" t="inlineStr">
+      <c r="G31" s="14" t="inlineStr"/>
+      <c r="H31" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT, K5M-T1B1-SDB, K5M-T1B1-CHA</t>
         </is>
       </c>
-      <c r="I31" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
+      <c r="I31" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
               <color rgb="00292B2B"/>
               <sz val="1000"/>
             </rPr>
@@ -2090,65 +2164,69 @@
           </r>
         </is>
       </c>
-      <c r="J31" s="16" t="inlineStr">
+      <c r="J31" s="17" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K31" s="16" t="inlineStr">
+      <c r="K31" s="17" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="L31" s="17" t="inlineStr"/>
-      <c r="M31" s="17" t="inlineStr"/>
-      <c r="N31" s="17" t="inlineStr"/>
-      <c r="O31" s="17" t="inlineStr"/>
-      <c r="P31" s="17" t="inlineStr"/>
-      <c r="Q31" s="17" t="inlineStr"/>
-      <c r="R31" s="17" t="inlineStr"/>
-      <c r="S31" s="14" t="inlineStr">
+      <c r="L31" s="18" t="inlineStr"/>
+      <c r="M31" s="19" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="N31" s="18" t="inlineStr"/>
+      <c r="O31" s="18" t="inlineStr"/>
+      <c r="P31" s="18" t="inlineStr"/>
+      <c r="Q31" s="18" t="inlineStr"/>
+      <c r="R31" s="18" t="inlineStr"/>
+      <c r="S31" s="15" t="inlineStr">
         <is>
           <t>Painting is EXCLUDED from the awarded BOQ scope per client — tracked here for material reference only</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="60" customHeight="1">
-      <c r="A32" s="13" t="n">
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="14" t="n">
         <v>19</v>
       </c>
-      <c r="B32" s="13" t="inlineStr">
+      <c r="B32" s="14" t="inlineStr">
         <is>
           <t>A-PT-02</t>
         </is>
       </c>
-      <c r="C32" s="13" t="inlineStr"/>
-      <c r="D32" s="13" t="inlineStr">
+      <c r="C32" s="14" t="inlineStr"/>
+      <c r="D32" s="14" t="inlineStr">
         <is>
           <t>Paint</t>
         </is>
       </c>
-      <c r="E32" s="14" t="inlineStr">
+      <c r="E32" s="15" t="inlineStr">
         <is>
           <t>Peinture texturée beige</t>
         </is>
       </c>
-      <c r="F32" s="14" t="inlineStr">
+      <c r="F32" s="15" t="inlineStr">
         <is>
           <t>Beige textured paint</t>
         </is>
       </c>
-      <c r="G32" s="13" t="inlineStr"/>
-      <c r="H32" s="14" t="inlineStr">
+      <c r="G32" s="14" t="inlineStr"/>
+      <c r="H32" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-CHA</t>
         </is>
       </c>
-      <c r="I32" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
+      <c r="I32" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
               <color rgb="00292B2B"/>
               <sz val="1000"/>
             </rPr>
@@ -2156,65 +2234,69 @@
           </r>
         </is>
       </c>
-      <c r="J32" s="16" t="inlineStr">
+      <c r="J32" s="17" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K32" s="16" t="inlineStr">
+      <c r="K32" s="17" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="L32" s="17" t="inlineStr"/>
-      <c r="M32" s="17" t="inlineStr"/>
-      <c r="N32" s="17" t="inlineStr"/>
-      <c r="O32" s="17" t="inlineStr"/>
-      <c r="P32" s="17" t="inlineStr"/>
-      <c r="Q32" s="17" t="inlineStr"/>
-      <c r="R32" s="17" t="inlineStr"/>
-      <c r="S32" s="14" t="inlineStr">
+      <c r="L32" s="18" t="inlineStr"/>
+      <c r="M32" s="19" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="N32" s="18" t="inlineStr"/>
+      <c r="O32" s="18" t="inlineStr"/>
+      <c r="P32" s="18" t="inlineStr"/>
+      <c r="Q32" s="18" t="inlineStr"/>
+      <c r="R32" s="18" t="inlineStr"/>
+      <c r="S32" s="15" t="inlineStr">
         <is>
           <t>Excluded from awarded BOQ scope</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="60" customHeight="1">
-      <c r="A33" s="13" t="n">
+    <row r="33" ht="34" customHeight="1">
+      <c r="A33" s="14" t="n">
         <v>20</v>
       </c>
-      <c r="B33" s="13" t="inlineStr">
+      <c r="B33" s="14" t="inlineStr">
         <is>
           <t>A-WP-01</t>
         </is>
       </c>
-      <c r="C33" s="13" t="inlineStr"/>
-      <c r="D33" s="13" t="inlineStr">
+      <c r="C33" s="14" t="inlineStr"/>
+      <c r="D33" s="14" t="inlineStr">
         <is>
           <t>Wallpaper</t>
         </is>
       </c>
-      <c r="E33" s="14" t="inlineStr">
+      <c r="E33" s="15" t="inlineStr">
         <is>
           <t>Papier peint (Omexco)</t>
         </is>
       </c>
-      <c r="F33" s="14" t="inlineStr">
+      <c r="F33" s="15" t="inlineStr">
         <is>
           <t>Wallpaper (Omexco)</t>
         </is>
       </c>
-      <c r="G33" s="13" t="inlineStr"/>
-      <c r="H33" s="14" t="inlineStr">
+      <c r="G33" s="14" t="inlineStr"/>
+      <c r="H33" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-CHA-C/6</t>
         </is>
       </c>
-      <c r="I33" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
+      <c r="I33" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
               <color rgb="00E4572E"/>
               <sz val="1000"/>
               <u val="single"/>
@@ -2223,65 +2305,69 @@
           </r>
         </is>
       </c>
-      <c r="J33" s="16" t="inlineStr">
+      <c r="J33" s="17" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K33" s="16" t="inlineStr">
+      <c r="K33" s="17" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="L33" s="17" t="inlineStr"/>
-      <c r="M33" s="17" t="inlineStr"/>
-      <c r="N33" s="17" t="inlineStr"/>
-      <c r="O33" s="17" t="inlineStr"/>
-      <c r="P33" s="17" t="inlineStr"/>
-      <c r="Q33" s="17" t="inlineStr"/>
-      <c r="R33" s="17" t="inlineStr"/>
-      <c r="S33" s="14" t="inlineStr">
+      <c r="L33" s="18" t="inlineStr"/>
+      <c r="M33" s="19" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="N33" s="18" t="inlineStr"/>
+      <c r="O33" s="18" t="inlineStr"/>
+      <c r="P33" s="18" t="inlineStr"/>
+      <c r="Q33" s="18" t="inlineStr"/>
+      <c r="R33" s="18" t="inlineStr"/>
+      <c r="S33" s="15" t="inlineStr">
         <is>
           <t>Supply/installation of this wallpaper is explicitly excluded in our BOQ offer (see C/6)</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="60" customHeight="1">
-      <c r="A34" s="13" t="n">
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="14" t="n">
         <v>21</v>
       </c>
-      <c r="B34" s="13" t="inlineStr">
+      <c r="B34" s="14" t="inlineStr">
         <is>
           <t>A-WP-02</t>
         </is>
       </c>
-      <c r="C34" s="13" t="inlineStr"/>
-      <c r="D34" s="13" t="inlineStr">
+      <c r="C34" s="14" t="inlineStr"/>
+      <c r="D34" s="14" t="inlineStr">
         <is>
           <t>Wallpaper</t>
         </is>
       </c>
-      <c r="E34" s="14" t="inlineStr">
+      <c r="E34" s="15" t="inlineStr">
         <is>
           <t>Papier peint (Biobject)</t>
         </is>
       </c>
-      <c r="F34" s="14" t="inlineStr">
+      <c r="F34" s="15" t="inlineStr">
         <is>
           <t>Wallpaper (Biobject)</t>
         </is>
       </c>
-      <c r="G34" s="13" t="inlineStr"/>
-      <c r="H34" s="14" t="inlineStr">
+      <c r="G34" s="14" t="inlineStr"/>
+      <c r="H34" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT</t>
         </is>
       </c>
-      <c r="I34" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
+      <c r="I34" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
               <color rgb="00292B2B"/>
               <sz val="1000"/>
             </rPr>
@@ -2289,65 +2375,69 @@
           </r>
         </is>
       </c>
-      <c r="J34" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K34" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L34" s="17" t="inlineStr"/>
-      <c r="M34" s="17" t="inlineStr"/>
-      <c r="N34" s="17" t="inlineStr"/>
-      <c r="O34" s="17" t="inlineStr"/>
-      <c r="P34" s="17" t="inlineStr"/>
-      <c r="Q34" s="17" t="inlineStr"/>
-      <c r="R34" s="17" t="inlineStr"/>
-      <c r="S34" s="14" t="inlineStr"/>
-    </row>
-    <row r="35" ht="60" customHeight="1">
-      <c r="A35" s="13" t="n">
+      <c r="J34" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K34" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L34" s="18" t="inlineStr"/>
+      <c r="M34" s="19" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="N34" s="18" t="inlineStr"/>
+      <c r="O34" s="18" t="inlineStr"/>
+      <c r="P34" s="18" t="inlineStr"/>
+      <c r="Q34" s="18" t="inlineStr"/>
+      <c r="R34" s="18" t="inlineStr"/>
+      <c r="S34" s="15" t="inlineStr"/>
+    </row>
+    <row r="35" ht="48" customHeight="1">
+      <c r="A35" s="14" t="n">
         <v>22</v>
       </c>
-      <c r="B35" s="13" t="inlineStr">
+      <c r="B35" s="14" t="inlineStr">
         <is>
           <t>A-CA-01</t>
         </is>
       </c>
-      <c r="C35" s="13" t="inlineStr"/>
-      <c r="D35" s="13" t="inlineStr">
+      <c r="C35" s="14" t="inlineStr"/>
+      <c r="D35" s="14" t="inlineStr">
         <is>
           <t>Carpet</t>
         </is>
       </c>
-      <c r="E35" s="14" t="inlineStr">
+      <c r="E35" s="15" t="inlineStr">
         <is>
           <t>Moquette (Design Carpet - Ali Laraqui)</t>
         </is>
       </c>
-      <c r="F35" s="14" t="inlineStr">
+      <c r="F35" s="15" t="inlineStr">
         <is>
           <t>Carpet (Design Carpet - Ali Laraqui)</t>
         </is>
       </c>
-      <c r="G35" s="13" t="inlineStr">
+      <c r="G35" s="14" t="inlineStr">
         <is>
           <t>Tapis encastré / Inset carpet</t>
         </is>
       </c>
-      <c r="H35" s="14" t="inlineStr">
+      <c r="H35" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-COULOIRS</t>
         </is>
       </c>
-      <c r="I35" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
+      <c r="I35" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
               <color rgb="00292B2B"/>
               <sz val="1000"/>
             </rPr>
@@ -2355,65 +2445,69 @@
           </r>
         </is>
       </c>
-      <c r="J35" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K35" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L35" s="17" t="inlineStr"/>
-      <c r="M35" s="17" t="inlineStr"/>
-      <c r="N35" s="17" t="inlineStr"/>
-      <c r="O35" s="17" t="inlineStr"/>
-      <c r="P35" s="17" t="inlineStr"/>
-      <c r="Q35" s="17" t="inlineStr"/>
-      <c r="R35" s="17" t="inlineStr"/>
-      <c r="S35" s="14" t="inlineStr">
+      <c r="J35" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K35" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L35" s="18" t="inlineStr"/>
+      <c r="M35" s="19" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="N35" s="18" t="inlineStr"/>
+      <c r="O35" s="18" t="inlineStr"/>
+      <c r="P35" s="18" t="inlineStr"/>
+      <c r="Q35" s="18" t="inlineStr"/>
+      <c r="R35" s="18" t="inlineStr"/>
+      <c r="S35" s="15" t="inlineStr">
         <is>
           <t>Confirm carpet remains Wood Couture scope (open decision noted in earlier Fit-out audit)</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="60" customHeight="1">
-      <c r="A36" s="13" t="n">
+    <row r="36" ht="34" customHeight="1">
+      <c r="A36" s="14" t="n">
         <v>23</v>
       </c>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="B36" s="14" t="inlineStr">
         <is>
           <t>A-ST-03c / A-ST-06c</t>
         </is>
       </c>
-      <c r="C36" s="13" t="inlineStr"/>
-      <c r="D36" s="13" t="inlineStr">
+      <c r="C36" s="14" t="inlineStr"/>
+      <c r="D36" s="14" t="inlineStr">
         <is>
           <t>Stone</t>
         </is>
       </c>
-      <c r="E36" s="14" t="inlineStr">
+      <c r="E36" s="15" t="inlineStr">
         <is>
           <t>Travertin osso (vein cut / cross cut) — NOUVEAU 21 Jul</t>
         </is>
       </c>
-      <c r="F36" s="14" t="inlineStr">
+      <c r="F36" s="15" t="inlineStr">
         <is>
           <t>Travertine osso (vein cut / cross cut) — NEW 21 Jul</t>
         </is>
       </c>
-      <c r="G36" s="13" t="inlineStr">
+      <c r="G36" s="14" t="inlineStr">
         <is>
           <t>Adouci / Honed</t>
         </is>
       </c>
-      <c r="H36" s="14" t="inlineStr"/>
-      <c r="I36" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
+      <c r="H36" s="15" t="inlineStr"/>
+      <c r="I36" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
               <color rgb="00E4572E"/>
               <sz val="1000"/>
               <u val="single"/>
@@ -2422,65 +2516,69 @@
           </r>
         </is>
       </c>
-      <c r="J36" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K36" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L36" s="17" t="inlineStr"/>
-      <c r="M36" s="17" t="inlineStr"/>
-      <c r="N36" s="17" t="inlineStr"/>
-      <c r="O36" s="17" t="inlineStr"/>
-      <c r="P36" s="17" t="inlineStr"/>
-      <c r="Q36" s="17" t="inlineStr"/>
-      <c r="R36" s="17" t="inlineStr"/>
-      <c r="S36" s="14" t="inlineStr">
+      <c r="J36" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K36" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L36" s="18" t="inlineStr"/>
+      <c r="M36" s="19" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="N36" s="18" t="inlineStr"/>
+      <c r="O36" s="18" t="inlineStr"/>
+      <c r="P36" s="18" t="inlineStr"/>
+      <c r="Q36" s="18" t="inlineStr"/>
+      <c r="R36" s="18" t="inlineStr"/>
+      <c r="S36" s="15" t="inlineStr">
         <is>
           <t>New codes as of 21 Jul 2026 — location/application not yet confirmed, ask Adil</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="60" customHeight="1">
-      <c r="A37" s="13" t="n">
+    <row r="37" ht="34" customHeight="1">
+      <c r="A37" s="14" t="n">
         <v>24</v>
       </c>
-      <c r="B37" s="13" t="inlineStr">
+      <c r="B37" s="14" t="inlineStr">
         <is>
           <t>A-WD-03c</t>
         </is>
       </c>
-      <c r="C37" s="13" t="inlineStr"/>
-      <c r="D37" s="13" t="inlineStr">
+      <c r="C37" s="14" t="inlineStr"/>
+      <c r="D37" s="14" t="inlineStr">
         <is>
           <t>Wood</t>
         </is>
       </c>
-      <c r="E37" s="14" t="inlineStr">
+      <c r="E37" s="15" t="inlineStr">
         <is>
           <t>Tatawi peint en blanc — NOUVEAU 21 Jul</t>
         </is>
       </c>
-      <c r="F37" s="14" t="inlineStr">
+      <c r="F37" s="15" t="inlineStr">
         <is>
           <t>White-painted Tatawi wood — NEW 21 Jul</t>
         </is>
       </c>
-      <c r="G37" s="13" t="inlineStr">
+      <c r="G37" s="14" t="inlineStr">
         <is>
           <t>Mat</t>
         </is>
       </c>
-      <c r="H37" s="14" t="inlineStr"/>
-      <c r="I37" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
+      <c r="H37" s="15" t="inlineStr"/>
+      <c r="I37" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
               <color rgb="00E4572E"/>
               <sz val="1000"/>
               <u val="single"/>
@@ -2489,24 +2587,28 @@
           </r>
         </is>
       </c>
-      <c r="J37" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K37" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L37" s="17" t="inlineStr"/>
-      <c r="M37" s="17" t="inlineStr"/>
-      <c r="N37" s="17" t="inlineStr"/>
-      <c r="O37" s="17" t="inlineStr"/>
-      <c r="P37" s="17" t="inlineStr"/>
-      <c r="Q37" s="17" t="inlineStr"/>
-      <c r="R37" s="17" t="inlineStr"/>
-      <c r="S37" s="14" t="inlineStr">
+      <c r="J37" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K37" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L37" s="18" t="inlineStr"/>
+      <c r="M37" s="19" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="N37" s="18" t="inlineStr"/>
+      <c r="O37" s="18" t="inlineStr"/>
+      <c r="P37" s="18" t="inlineStr"/>
+      <c r="Q37" s="18" t="inlineStr"/>
+      <c r="R37" s="18" t="inlineStr"/>
+      <c r="S37" s="15" t="inlineStr">
         <is>
           <t>New code as of 21 Jul 2026 — location/application not yet confirmed, ask Adil</t>
         </is>

</xml_diff>

<commit_message>
Fitout Material Package: fix real formatting bug, fix severe rich-text rendering bug, add thumbnails
- Revert Cambria/Calibri misdiagnosis: Playfair Display/Lato + uniform 150pt row height
- Fix Localization column rendering as a single stray character per row: InlineFont sz=1000
  was being read by Excel as a literal 1000pt font, not 10.00pt. Changed to sz=11.
- Add thumbnails: 21/24 rows, extracted directly from the source material list PDF by
  matching each material code to its PHOTO-column cell and cropping that region.
  Replacement occurrences (substitutions) used over originals where a code appears twice.
- Remaining 3 rows (A-WD-01d, A-GL-04a, A-CA-01) have no source photo in any document reviewed.
- Visually verified via Excel COM -> PDF export.
</commit_message>
<xml_diff>
--- a/material_package_fitout/260727_K5M_Material Package_Fitout.xlsx
+++ b/material_package_fitout/260727_K5M_Material Package_Fitout.xlsx
@@ -26,42 +26,41 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Cambria"/>
-      <b val="1"/>
+      <name val="Playfair Display"/>
       <color rgb="00FFFFFF"/>
-      <sz val="18"/>
+      <sz val="16"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Lato"/>
       <i val="1"/>
       <color rgb="00292B2B"/>
       <sz val="9"/>
     </font>
     <font>
-      <name val="Cambria"/>
+      <name val="Playfair Display"/>
       <b val="1"/>
       <color rgb="00292B2B"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Lato"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Lato"/>
       <color rgb="00292B2B"/>
-      <sz val="10"/>
+      <sz val="11"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Lato"/>
       <b val="1"/>
       <color rgb="00292B2B"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Lato"/>
       <i val="1"/>
       <color rgb="00E4572E"/>
       <sz val="8"/>
@@ -141,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -173,9 +172,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -262,6 +258,536 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="571500" cy="547914"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="571500" cy="547914"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="571500" cy="538842"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="571500" cy="547914"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="571500" cy="537028"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="571500" cy="551542"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="571500" cy="555171"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="571500" cy="551542"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>22</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="571500" cy="431799"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>23</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="571500" cy="547914"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>24</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="571500" cy="549728"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="571500" cy="547914"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>26</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="571500" cy="537028"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="571500" cy="533400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>28</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="571500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId15"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="571500" cy="533400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId16"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>31</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="571500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId17"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>32</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="571500" cy="537028"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId18"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>33</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="571500" cy="551542"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="19" name="Image 19" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId19"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="571500" cy="547914"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="20" name="Image 20" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId20"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>36</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="571500" cy="551542"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="21" name="Image 21" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId21"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -577,7 +1103,7 @@
     <col width="34" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="44" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>K5M — FIT-OUT MATERIAL PACKAGE</t>
@@ -799,7 +1325,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="62" customHeight="1">
+    <row r="14" ht="150" customHeight="1">
       <c r="A14" s="14" t="n">
         <v>1</v>
       </c>
@@ -814,12 +1340,12 @@
           <t>Stone</t>
         </is>
       </c>
-      <c r="E14" s="15" t="inlineStr">
+      <c r="E14" s="14" t="inlineStr">
         <is>
           <t>Beige clair</t>
         </is>
       </c>
-      <c r="F14" s="15" t="inlineStr">
+      <c r="F14" s="14" t="inlineStr">
         <is>
           <t>Light beige stone</t>
         </is>
@@ -829,69 +1355,69 @@
           <t>Adouci / Honed</t>
         </is>
       </c>
-      <c r="H14" s="15" t="inlineStr">
+      <c r="H14" s="14" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT-A/? (seuil), K5M-T1B1-SDB-B/6, K5M-T1B1-SDB-B/12, K5M-T1B1-CHA-C/2, K5M-T1B1-CHA-C/3</t>
         </is>
       </c>
-      <c r="I14" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
+      <c r="I14" s="15" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Lato"/>
               <color rgb="00292B2B"/>
-              <sz val="1000"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">Entrée: seuil. </t>
           </r>
           <r>
             <rPr>
-              <rFont val="Calibri"/>
+              <rFont val="Lato"/>
               <color rgb="00E4572E"/>
-              <sz val="1000"/>
+              <sz val="11"/>
               <u val="single"/>
             </rPr>
             <t xml:space="preserve">SDB: arche toilette/douche, niche (conflicts with BOQ A-ST-07a on niche — see FM-007). </t>
           </r>
           <r>
             <rPr>
-              <rFont val="Calibri"/>
+              <rFont val="Lato"/>
               <color rgb="00E4572E"/>
-              <sz val="1000"/>
+              <sz val="11"/>
               <u val="single"/>
             </rPr>
             <t>Chambre: seuil (C/3, joint code conflict — see FM-010), plinthe (C/2, conflicts with A-ST-01e/A-ST-02c in updated list — see FM-009).</t>
           </r>
         </is>
       </c>
-      <c r="J14" s="17" t="inlineStr">
+      <c r="J14" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K14" s="17" t="inlineStr">
+      <c r="K14" s="16" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L14" s="18" t="inlineStr"/>
-      <c r="M14" s="19" t="inlineStr">
+      <c r="L14" s="17" t="inlineStr"/>
+      <c r="M14" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N14" s="18" t="inlineStr"/>
-      <c r="O14" s="18" t="inlineStr"/>
-      <c r="P14" s="18" t="inlineStr"/>
-      <c r="Q14" s="18" t="inlineStr"/>
-      <c r="R14" s="18" t="inlineStr"/>
-      <c r="S14" s="15" t="inlineStr">
+      <c r="N14" s="17" t="inlineStr"/>
+      <c r="O14" s="17" t="inlineStr"/>
+      <c r="P14" s="17" t="inlineStr"/>
+      <c r="Q14" s="17" t="inlineStr"/>
+      <c r="R14" s="17" t="inlineStr"/>
+      <c r="S14" s="14" t="inlineStr">
         <is>
           <t>See FM-007, FM-009, FM-010 — all still open, to re-raise with Adil</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="48" customHeight="1">
+    <row r="15" ht="150" customHeight="1">
       <c r="A15" s="14" t="n">
         <v>2</v>
       </c>
@@ -906,12 +1432,12 @@
           <t>Stone</t>
         </is>
       </c>
-      <c r="E15" s="15" t="inlineStr">
+      <c r="E15" s="14" t="inlineStr">
         <is>
           <t>Beige clair</t>
         </is>
       </c>
-      <c r="F15" s="15" t="inlineStr">
+      <c r="F15" s="14" t="inlineStr">
         <is>
           <t>Light beige stone</t>
         </is>
@@ -921,60 +1447,60 @@
           <t>Anti-dérapant / Anti-slip</t>
         </is>
       </c>
-      <c r="H15" s="15" t="inlineStr">
+      <c r="H15" s="14" t="inlineStr">
         <is>
           <t>K5M-T1B1-SDB-B/2, K5M-T1B1-SDB-B/5</t>
         </is>
       </c>
-      <c r="I15" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
+      <c r="I15" s="15" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Lato"/>
               <color rgb="00292B2B"/>
-              <sz val="1000"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">SDB: sol douche (shower floor). </t>
           </r>
           <r>
             <rPr>
-              <rFont val="Calibri"/>
+              <rFont val="Lato"/>
               <color rgb="00E4572E"/>
-              <sz val="1000"/>
+              <sz val="11"/>
               <u val="single"/>
             </rPr>
             <t>Threshold at B/5 conflicts with DD-100's A-ST-01c on the same opening — see FM-005. Anti-slip classification not defined — see FM-012.</t>
           </r>
         </is>
       </c>
-      <c r="J15" s="17" t="inlineStr">
+      <c r="J15" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K15" s="17" t="inlineStr">
+      <c r="K15" s="16" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L15" s="18" t="inlineStr"/>
-      <c r="M15" s="19" t="inlineStr">
+      <c r="L15" s="17" t="inlineStr"/>
+      <c r="M15" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N15" s="18" t="inlineStr"/>
-      <c r="O15" s="18" t="inlineStr"/>
-      <c r="P15" s="18" t="inlineStr"/>
-      <c r="Q15" s="18" t="inlineStr"/>
-      <c r="R15" s="18" t="inlineStr"/>
-      <c r="S15" s="15" t="inlineStr">
+      <c r="N15" s="17" t="inlineStr"/>
+      <c r="O15" s="17" t="inlineStr"/>
+      <c r="P15" s="17" t="inlineStr"/>
+      <c r="Q15" s="17" t="inlineStr"/>
+      <c r="R15" s="17" t="inlineStr"/>
+      <c r="S15" s="14" t="inlineStr">
         <is>
           <t>See FM-005, FM-012</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="34" customHeight="1">
+    <row r="16" ht="150" customHeight="1">
       <c r="A16" s="14" t="n">
         <v>3</v>
       </c>
@@ -989,12 +1515,12 @@
           <t>Stone</t>
         </is>
       </c>
-      <c r="E16" s="15" t="inlineStr">
+      <c r="E16" s="14" t="inlineStr">
         <is>
           <t>Beige clair</t>
         </is>
       </c>
-      <c r="F16" s="15" t="inlineStr">
+      <c r="F16" s="14" t="inlineStr">
         <is>
           <t>Light beige stone</t>
         </is>
@@ -1004,47 +1530,47 @@
           <t>Martelé / Hammered</t>
         </is>
       </c>
-      <c r="H16" s="15" t="inlineStr">
+      <c r="H16" s="14" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT-A/1, K5M-T1B1-SDB-B/1</t>
         </is>
       </c>
-      <c r="I16" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
+      <c r="I16" s="15" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Lato"/>
               <color rgb="00292B2B"/>
-              <sz val="1000"/>
+              <sz val="11"/>
             </rPr>
             <t>Entrée: sol. SDB: sol. Hall/corridor floor per BOQ item 1 (Hall Ascenseurs).</t>
           </r>
         </is>
       </c>
-      <c r="J16" s="17" t="inlineStr">
+      <c r="J16" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K16" s="17" t="inlineStr">
+      <c r="K16" s="16" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L16" s="18" t="inlineStr"/>
-      <c r="M16" s="19" t="inlineStr">
+      <c r="L16" s="17" t="inlineStr"/>
+      <c r="M16" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N16" s="18" t="inlineStr"/>
-      <c r="O16" s="18" t="inlineStr"/>
-      <c r="P16" s="18" t="inlineStr"/>
-      <c r="Q16" s="18" t="inlineStr"/>
-      <c r="R16" s="18" t="inlineStr"/>
-      <c r="S16" s="15" t="inlineStr"/>
-    </row>
-    <row r="17" ht="34" customHeight="1">
+      <c r="N16" s="17" t="inlineStr"/>
+      <c r="O16" s="17" t="inlineStr"/>
+      <c r="P16" s="17" t="inlineStr"/>
+      <c r="Q16" s="17" t="inlineStr"/>
+      <c r="R16" s="17" t="inlineStr"/>
+      <c r="S16" s="14" t="inlineStr"/>
+    </row>
+    <row r="17" ht="150" customHeight="1">
       <c r="A17" s="14" t="n">
         <v>4</v>
       </c>
@@ -1059,12 +1585,12 @@
           <t>Stone</t>
         </is>
       </c>
-      <c r="E17" s="15" t="inlineStr">
+      <c r="E17" s="14" t="inlineStr">
         <is>
           <t>Beige foncé</t>
         </is>
       </c>
-      <c r="F17" s="15" t="inlineStr">
+      <c r="F17" s="14" t="inlineStr">
         <is>
           <t>Dark beige stone</t>
         </is>
@@ -1074,60 +1600,60 @@
           <t>Adouci / Honed</t>
         </is>
       </c>
-      <c r="H17" s="15" t="inlineStr">
+      <c r="H17" s="14" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT-A/1, K5M-T1B1-SDB-B/1, K5M-T1B1-SDB-B/3, K5M-T1B1-CHA-C/2</t>
         </is>
       </c>
-      <c r="I17" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
+      <c r="I17" s="15" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Lato"/>
               <color rgb="00292B2B"/>
-              <sz val="1000"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">Entrée: sol. SDB: sol, plinthe. </t>
           </r>
           <r>
             <rPr>
-              <rFont val="Calibri"/>
+              <rFont val="Lato"/>
               <color rgb="00E4572E"/>
-              <sz val="1000"/>
+              <sz val="11"/>
               <u val="single"/>
             </rPr>
             <t>Chambre: plinthe (C/2) — conflicts with A-ST-01c/A-ST-01e, see FM-009.</t>
           </r>
         </is>
       </c>
-      <c r="J17" s="17" t="inlineStr">
+      <c r="J17" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K17" s="17" t="inlineStr">
+      <c r="K17" s="16" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L17" s="18" t="inlineStr"/>
-      <c r="M17" s="19" t="inlineStr">
+      <c r="L17" s="17" t="inlineStr"/>
+      <c r="M17" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N17" s="18" t="inlineStr"/>
-      <c r="O17" s="18" t="inlineStr"/>
-      <c r="P17" s="18" t="inlineStr"/>
-      <c r="Q17" s="18" t="inlineStr"/>
-      <c r="R17" s="18" t="inlineStr"/>
-      <c r="S17" s="15" t="inlineStr">
+      <c r="N17" s="17" t="inlineStr"/>
+      <c r="O17" s="17" t="inlineStr"/>
+      <c r="P17" s="17" t="inlineStr"/>
+      <c r="Q17" s="17" t="inlineStr"/>
+      <c r="R17" s="17" t="inlineStr"/>
+      <c r="S17" s="14" t="inlineStr">
         <is>
           <t>See FM-009</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="62" customHeight="1">
+    <row r="18" ht="150" customHeight="1">
       <c r="A18" s="14" t="n">
         <v>5</v>
       </c>
@@ -1142,12 +1668,12 @@
           <t>Stone</t>
         </is>
       </c>
-      <c r="E18" s="15" t="inlineStr">
+      <c r="E18" s="14" t="inlineStr">
         <is>
           <t>Onyx miel — REMPLACÉ PAR Taj Mahal</t>
         </is>
       </c>
-      <c r="F18" s="15" t="inlineStr">
+      <c r="F18" s="14" t="inlineStr">
         <is>
           <t>Onyx Honey — REPLACED BY Taj Mahal</t>
         </is>
@@ -1157,68 +1683,68 @@
           <t>Poli / Polished</t>
         </is>
       </c>
-      <c r="H18" s="15" t="inlineStr">
+      <c r="H18" s="14" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT-A (arche/porte-bagage), K5M-T1B1-SDB-B/7, K5M-T1B1-SDB-B/8, K5M-T1B1-SDB-B/9, K5M-T1B1-SDB-B/10, K5M-T1B1-SDB-B/11, K5M-T1B1-SDB-B/12, K5M-T1B1-CHA-C/4</t>
         </is>
       </c>
-      <c r="I18" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
+      <c r="I18" s="15" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Lato"/>
               <color rgb="00292B2B"/>
-              <sz val="1000"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">Entrée: arche, porte-bagage. SDB: banc (B/7, B/8), tablette WC (B/9), vasque (B/10), arche vasque (B/11). </t>
           </r>
           <r>
             <rPr>
-              <rFont val="Calibri"/>
+              <rFont val="Lato"/>
               <color rgb="00E4572E"/>
-              <sz val="1000"/>
+              <sz val="11"/>
               <u val="single"/>
             </rPr>
             <t>SDB niche (B/12) — same code shown twice in updated list (superseded honey-onyx row retained alongside Taj Mahal replacement) — see FM-002 and FM-007.</t>
           </r>
           <r>
             <rPr>
-              <rFont val="Calibri"/>
+              <rFont val="Lato"/>
               <color rgb="00292B2B"/>
-              <sz val="1000"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve"> Chambre: arche (C/4).</t>
           </r>
         </is>
       </c>
-      <c r="J18" s="17" t="inlineStr">
+      <c r="J18" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K18" s="17" t="inlineStr">
+      <c r="K18" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L18" s="18" t="inlineStr"/>
-      <c r="M18" s="19" t="inlineStr">
+      <c r="L18" s="17" t="inlineStr"/>
+      <c r="M18" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N18" s="18" t="inlineStr"/>
-      <c r="O18" s="18" t="inlineStr"/>
-      <c r="P18" s="18" t="inlineStr"/>
-      <c r="Q18" s="18" t="inlineStr"/>
-      <c r="R18" s="18" t="inlineStr"/>
-      <c r="S18" s="15" t="inlineStr">
+      <c r="N18" s="17" t="inlineStr"/>
+      <c r="O18" s="17" t="inlineStr"/>
+      <c r="P18" s="17" t="inlineStr"/>
+      <c r="Q18" s="17" t="inlineStr"/>
+      <c r="R18" s="17" t="inlineStr"/>
+      <c r="S18" s="14" t="inlineStr">
         <is>
           <t>SUBSTITUTED as of 21 Jul 2026 update. See FM-002, FM-007 — confirm Taj Mahal applies everywhere, honey onyx no longer valid anywhere</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="48" customHeight="1">
+    <row r="19" ht="150" customHeight="1">
       <c r="A19" s="14" t="n">
         <v>6</v>
       </c>
@@ -1233,12 +1759,12 @@
           <t>Wood</t>
         </is>
       </c>
-      <c r="E19" s="15" t="inlineStr">
+      <c r="E19" s="14" t="inlineStr">
         <is>
           <t>Noyer — REMPLACÉ PAR chêne teinté moyen</t>
         </is>
       </c>
-      <c r="F19" s="15" t="inlineStr">
+      <c r="F19" s="14" t="inlineStr">
         <is>
           <t>Walnut — REPLACED BY medium-tinted oak</t>
         </is>
@@ -1248,61 +1774,61 @@
           <t>Satin</t>
         </is>
       </c>
-      <c r="H19" s="15" t="inlineStr">
+      <c r="H19" s="14" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT-A/7, K5M-T1B1-CHA-C/7</t>
         </is>
       </c>
-      <c r="I19" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
+      <c r="I19" s="15" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Lato"/>
               <color rgb="00E4572E"/>
-              <sz val="1000"/>
+              <sz val="11"/>
               <u val="single"/>
             </rPr>
             <t xml:space="preserve">Entrée: porte, architrave, plinthe (A/7). </t>
           </r>
           <r>
             <rPr>
-              <rFont val="Calibri"/>
+              <rFont val="Lato"/>
               <color rgb="00E4572E"/>
-              <sz val="1000"/>
+              <sz val="11"/>
               <u val="single"/>
             </rPr>
             <t>Chambre: tablette (C/7). BOQ uses three code variants (A-WD-01d, generic A-WD-01, A-WD-01b) for these — see FM-001.</t>
           </r>
         </is>
       </c>
-      <c r="J19" s="17" t="inlineStr">
+      <c r="J19" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K19" s="17" t="inlineStr">
+      <c r="K19" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L19" s="18" t="inlineStr"/>
-      <c r="M19" s="19" t="inlineStr">
+      <c r="L19" s="17" t="inlineStr"/>
+      <c r="M19" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N19" s="18" t="inlineStr"/>
-      <c r="O19" s="18" t="inlineStr"/>
-      <c r="P19" s="18" t="inlineStr"/>
-      <c r="Q19" s="18" t="inlineStr"/>
-      <c r="R19" s="18" t="inlineStr"/>
-      <c r="S19" s="15" t="inlineStr">
+      <c r="N19" s="17" t="inlineStr"/>
+      <c r="O19" s="17" t="inlineStr"/>
+      <c r="P19" s="17" t="inlineStr"/>
+      <c r="Q19" s="17" t="inlineStr"/>
+      <c r="R19" s="17" t="inlineStr"/>
+      <c r="S19" s="14" t="inlineStr">
         <is>
           <t>SUBSTITUTED as of 21 Jul 2026. See FM-001 — confirm all four applications follow this code/finish</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="34" customHeight="1">
+    <row r="20" ht="150" customHeight="1">
       <c r="A20" s="14" t="n">
         <v>7</v>
       </c>
@@ -1317,63 +1843,63 @@
           <t>Wood</t>
         </is>
       </c>
-      <c r="E20" s="15" t="inlineStr">
+      <c r="E20" s="14" t="inlineStr">
         <is>
           <t>(absent de la liste officielle des matériaux)</t>
         </is>
       </c>
-      <c r="F20" s="15" t="inlineStr">
+      <c r="F20" s="14" t="inlineStr">
         <is>
           <t>(does not appear in the official material list at all)</t>
         </is>
       </c>
       <c r="G20" s="14" t="inlineStr"/>
-      <c r="H20" s="15" t="inlineStr">
+      <c r="H20" s="14" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT-A/2, K5M-T1B1-ENT-A/4</t>
         </is>
       </c>
-      <c r="I20" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
+      <c r="I20" s="15" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Lato"/>
               <color rgb="00E4572E"/>
-              <sz val="1000"/>
+              <sz val="11"/>
               <u val="single"/>
             </rPr>
             <t xml:space="preserve">Entrée: plinthe (A/2), arche (A/4) — code only exists in the BOQ/RFI, not in any material list issue. </t>
           </r>
         </is>
       </c>
-      <c r="J20" s="17" t="inlineStr">
+      <c r="J20" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K20" s="17" t="inlineStr">
+      <c r="K20" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L20" s="18" t="inlineStr"/>
-      <c r="M20" s="19" t="inlineStr">
+      <c r="L20" s="17" t="inlineStr"/>
+      <c r="M20" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N20" s="18" t="inlineStr"/>
-      <c r="O20" s="18" t="inlineStr"/>
-      <c r="P20" s="18" t="inlineStr"/>
-      <c r="Q20" s="18" t="inlineStr"/>
-      <c r="R20" s="18" t="inlineStr"/>
-      <c r="S20" s="15" t="inlineStr">
+      <c r="N20" s="17" t="inlineStr"/>
+      <c r="O20" s="17" t="inlineStr"/>
+      <c r="P20" s="17" t="inlineStr"/>
+      <c r="Q20" s="17" t="inlineStr"/>
+      <c r="R20" s="17" t="inlineStr"/>
+      <c r="S20" s="14" t="inlineStr">
         <is>
           <t>See FM-001. RFI already flags: no material reference image provided for this code</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="48" customHeight="1">
+    <row r="21" ht="150" customHeight="1">
       <c r="A21" s="14" t="n">
         <v>8</v>
       </c>
@@ -1388,12 +1914,12 @@
           <t>Wood</t>
         </is>
       </c>
-      <c r="E21" s="15" t="inlineStr">
+      <c r="E21" s="14" t="inlineStr">
         <is>
           <t>Chêne cérusé blanc</t>
         </is>
       </c>
-      <c r="F21" s="15" t="inlineStr">
+      <c r="F21" s="14" t="inlineStr">
         <is>
           <t>White cerused oak</t>
         </is>
@@ -1403,60 +1929,60 @@
           <t>Mat / Matte</t>
         </is>
       </c>
-      <c r="H21" s="15" t="inlineStr">
+      <c r="H21" s="14" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT-A/8, K5M-T1B1-SDB-B/14, K5M-T1B1-CHA-C/6</t>
         </is>
       </c>
-      <c r="I21" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
+      <c r="I21" s="15" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Lato"/>
               <color rgb="00292B2B"/>
-              <sz val="1000"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">Entrée: contour/tiroir/dressings (A/8). SDB: contour portes (B/14). </t>
           </r>
           <r>
             <rPr>
-              <rFont val="Calibri"/>
+              <rFont val="Lato"/>
               <color rgb="00E4572E"/>
-              <sz val="1000"/>
+              <sz val="11"/>
               <u val="single"/>
             </rPr>
             <t>Chambre: wall panels per BOQ (C/6), but updated material-list location only mentions banquette, not wall panelling — see FM-011.</t>
           </r>
         </is>
       </c>
-      <c r="J21" s="17" t="inlineStr">
+      <c r="J21" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K21" s="17" t="inlineStr">
+      <c r="K21" s="16" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L21" s="18" t="inlineStr"/>
-      <c r="M21" s="19" t="inlineStr">
+      <c r="L21" s="17" t="inlineStr"/>
+      <c r="M21" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N21" s="18" t="inlineStr"/>
-      <c r="O21" s="18" t="inlineStr"/>
-      <c r="P21" s="18" t="inlineStr"/>
-      <c r="Q21" s="18" t="inlineStr"/>
-      <c r="R21" s="18" t="inlineStr"/>
-      <c r="S21" s="15" t="inlineStr">
+      <c r="N21" s="17" t="inlineStr"/>
+      <c r="O21" s="17" t="inlineStr"/>
+      <c r="P21" s="17" t="inlineStr"/>
+      <c r="Q21" s="17" t="inlineStr"/>
+      <c r="R21" s="17" t="inlineStr"/>
+      <c r="S21" s="14" t="inlineStr">
         <is>
           <t>See FM-011</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="34" customHeight="1">
+    <row r="22" ht="150" customHeight="1">
       <c r="A22" s="14" t="n">
         <v>9</v>
       </c>
@@ -1471,12 +1997,12 @@
           <t>Wood</t>
         </is>
       </c>
-      <c r="E22" s="15" t="inlineStr">
+      <c r="E22" s="14" t="inlineStr">
         <is>
           <t>Parquet chêne teinté moyen (Hakwood Idéal)</t>
         </is>
       </c>
-      <c r="F22" s="15" t="inlineStr">
+      <c r="F22" s="14" t="inlineStr">
         <is>
           <t>Medium-tinted oak parquet (Hakwood Idéal)</t>
         </is>
@@ -1486,61 +2012,61 @@
           <t>Satin</t>
         </is>
       </c>
-      <c r="H22" s="15" t="inlineStr">
+      <c r="H22" s="14" t="inlineStr">
         <is>
           <t>K5M-T1B1-CHA-C/1</t>
         </is>
       </c>
-      <c r="I22" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
+      <c r="I22" s="15" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Lato"/>
               <color rgb="00E4572E"/>
-              <sz val="1000"/>
+              <sz val="11"/>
               <u val="single"/>
             </rPr>
             <t xml:space="preserve">Chambre: sol (floor). </t>
           </r>
           <r>
             <rPr>
-              <rFont val="Calibri"/>
+              <rFont val="Lato"/>
               <color rgb="00E4572E"/>
-              <sz val="1000"/>
+              <sz val="11"/>
               <u val="single"/>
             </rPr>
             <t>BOQ cites A-WD-04d, which does not appear anywhere in DD-100 or the material lists — see FM-008.</t>
           </r>
         </is>
       </c>
-      <c r="J22" s="17" t="inlineStr">
+      <c r="J22" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K22" s="17" t="inlineStr">
+      <c r="K22" s="16" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L22" s="18" t="inlineStr"/>
-      <c r="M22" s="19" t="inlineStr">
+      <c r="L22" s="17" t="inlineStr"/>
+      <c r="M22" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N22" s="18" t="inlineStr"/>
-      <c r="O22" s="18" t="inlineStr"/>
-      <c r="P22" s="18" t="inlineStr"/>
-      <c r="Q22" s="18" t="inlineStr"/>
-      <c r="R22" s="18" t="inlineStr"/>
-      <c r="S22" s="15" t="inlineStr">
+      <c r="N22" s="17" t="inlineStr"/>
+      <c r="O22" s="17" t="inlineStr"/>
+      <c r="P22" s="17" t="inlineStr"/>
+      <c r="Q22" s="17" t="inlineStr"/>
+      <c r="R22" s="17" t="inlineStr"/>
+      <c r="S22" s="14" t="inlineStr">
         <is>
           <t>SUBSTITUTED from dark-tinted to medium-tinted oak, 21 Jul 2026, real product ref (Hakwood, Idéal). See FM-008</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="62" customHeight="1">
+    <row r="23" ht="150" customHeight="1">
       <c r="A23" s="14" t="n">
         <v>10</v>
       </c>
@@ -1555,12 +2081,12 @@
           <t>Metal</t>
         </is>
       </c>
-      <c r="E23" s="15" t="inlineStr">
+      <c r="E23" s="14" t="inlineStr">
         <is>
           <t>Acier inoxydable poli</t>
         </is>
       </c>
-      <c r="F23" s="15" t="inlineStr">
+      <c r="F23" s="14" t="inlineStr">
         <is>
           <t>Polished stainless steel</t>
         </is>
@@ -1570,61 +2096,61 @@
           <t>Finition poli miroir</t>
         </is>
       </c>
-      <c r="H23" s="15" t="inlineStr">
+      <c r="H23" s="14" t="inlineStr">
         <is>
           <t>K5M-T1B1-SDB-B/8, K5M-T1B1-SDB-B/14</t>
         </is>
       </c>
-      <c r="I23" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
+      <c r="I23" s="15" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Lato"/>
               <color rgb="00E4572E"/>
-              <sz val="1000"/>
+              <sz val="11"/>
               <u val="single"/>
             </rPr>
             <t>SDB: bench structure/base (B/8) — not explicitly confirmed in updated material-list locations, see FM-006. Door handle/frame (B/14).</t>
           </r>
           <r>
             <rPr>
-              <rFont val="Calibri"/>
+              <rFont val="Lato"/>
               <color rgb="00E4572E"/>
-              <sz val="1000"/>
+              <sz val="11"/>
               <u val="single"/>
             </rPr>
             <t xml:space="preserve"> Original (27 Oct 2025) list located this at Entrée tringle instead — location moved in the 21 Jul update; A-ME-01h now covers the Entrée tringle.</t>
           </r>
         </is>
       </c>
-      <c r="J23" s="17" t="inlineStr">
+      <c r="J23" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K23" s="17" t="inlineStr">
+      <c r="K23" s="16" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L23" s="18" t="inlineStr"/>
-      <c r="M23" s="19" t="inlineStr">
+      <c r="L23" s="17" t="inlineStr"/>
+      <c r="M23" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N23" s="18" t="inlineStr"/>
-      <c r="O23" s="18" t="inlineStr"/>
-      <c r="P23" s="18" t="inlineStr"/>
-      <c r="Q23" s="18" t="inlineStr"/>
-      <c r="R23" s="18" t="inlineStr"/>
-      <c r="S23" s="15" t="inlineStr">
+      <c r="N23" s="17" t="inlineStr"/>
+      <c r="O23" s="17" t="inlineStr"/>
+      <c r="P23" s="17" t="inlineStr"/>
+      <c r="Q23" s="17" t="inlineStr"/>
+      <c r="R23" s="17" t="inlineStr"/>
+      <c r="S23" s="14" t="inlineStr">
         <is>
           <t>See FM-006. Location changed between material list versions — confirm current assignment</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="34" customHeight="1">
+    <row r="24" ht="150" customHeight="1">
       <c r="A24" s="14" t="n">
         <v>11</v>
       </c>
@@ -1639,12 +2165,12 @@
           <t>Metal</t>
         </is>
       </c>
-      <c r="E24" s="15" t="inlineStr">
+      <c r="E24" s="14" t="inlineStr">
         <is>
           <t>Acier inoxydable brossé (NOUVEAU 21 Jul)</t>
         </is>
       </c>
-      <c r="F24" s="15" t="inlineStr">
+      <c r="F24" s="14" t="inlineStr">
         <is>
           <t>Brushed stainless steel (NEW 21 Jul)</t>
         </is>
@@ -1654,52 +2180,52 @@
           <t>Finition brossé</t>
         </is>
       </c>
-      <c r="H24" s="15" t="inlineStr">
+      <c r="H24" s="14" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT</t>
         </is>
       </c>
-      <c r="I24" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
+      <c r="I24" s="15" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Lato"/>
               <color rgb="00E4572E"/>
-              <sz val="1000"/>
+              <sz val="11"/>
               <u val="single"/>
             </rPr>
             <t>Entrée: tringle (rail) — new code introduced 21 Jul 2026, appears to take over this location from A-ME-01a.</t>
           </r>
         </is>
       </c>
-      <c r="J24" s="17" t="inlineStr">
+      <c r="J24" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K24" s="17" t="inlineStr">
+      <c r="K24" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L24" s="18" t="inlineStr"/>
-      <c r="M24" s="19" t="inlineStr">
+      <c r="L24" s="17" t="inlineStr"/>
+      <c r="M24" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N24" s="18" t="inlineStr"/>
-      <c r="O24" s="18" t="inlineStr"/>
-      <c r="P24" s="18" t="inlineStr"/>
-      <c r="Q24" s="18" t="inlineStr"/>
-      <c r="R24" s="18" t="inlineStr"/>
-      <c r="S24" s="15" t="inlineStr">
+      <c r="N24" s="17" t="inlineStr"/>
+      <c r="O24" s="17" t="inlineStr"/>
+      <c r="P24" s="17" t="inlineStr"/>
+      <c r="Q24" s="17" t="inlineStr"/>
+      <c r="R24" s="17" t="inlineStr"/>
+      <c r="S24" s="14" t="inlineStr">
         <is>
           <t>New code as of 21 Jul 2026 update — confirm with Adil this is the correct replacement for the rail location</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="34" customHeight="1">
+    <row r="25" ht="150" customHeight="1">
       <c r="A25" s="14" t="n">
         <v>12</v>
       </c>
@@ -1714,12 +2240,12 @@
           <t>Metal</t>
         </is>
       </c>
-      <c r="E25" s="15" t="inlineStr">
+      <c r="E25" s="14" t="inlineStr">
         <is>
           <t>Laiton patiné foncé</t>
         </is>
       </c>
-      <c r="F25" s="15" t="inlineStr">
+      <c r="F25" s="14" t="inlineStr">
         <is>
           <t>Dark patinated brass</t>
         </is>
@@ -1729,47 +2255,47 @@
           <t>Vernis mat / Matte varnish</t>
         </is>
       </c>
-      <c r="H25" s="15" t="inlineStr">
+      <c r="H25" s="14" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT-A/7, K5M-T1B1-ENT-A/8, K5M-T1B1-SDB-B/13, K5M-T1B1-CHA-C/7</t>
         </is>
       </c>
-      <c r="I25" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
+      <c r="I25" s="15" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Lato"/>
               <color rgb="00292B2B"/>
-              <sz val="1000"/>
+              <sz val="11"/>
             </rPr>
             <t>Entrée: door joint/trim (A/7, A/8). SDB: mirror joint/trim (B/13). Chambre: mirror joint/trim (C/7).</t>
           </r>
         </is>
       </c>
-      <c r="J25" s="17" t="inlineStr">
+      <c r="J25" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K25" s="17" t="inlineStr">
+      <c r="K25" s="16" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L25" s="18" t="inlineStr"/>
-      <c r="M25" s="19" t="inlineStr">
+      <c r="L25" s="17" t="inlineStr"/>
+      <c r="M25" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N25" s="18" t="inlineStr"/>
-      <c r="O25" s="18" t="inlineStr"/>
-      <c r="P25" s="18" t="inlineStr"/>
-      <c r="Q25" s="18" t="inlineStr"/>
-      <c r="R25" s="18" t="inlineStr"/>
-      <c r="S25" s="15" t="inlineStr"/>
-    </row>
-    <row r="26" ht="34" customHeight="1">
+      <c r="N25" s="17" t="inlineStr"/>
+      <c r="O25" s="17" t="inlineStr"/>
+      <c r="P25" s="17" t="inlineStr"/>
+      <c r="Q25" s="17" t="inlineStr"/>
+      <c r="R25" s="17" t="inlineStr"/>
+      <c r="S25" s="14" t="inlineStr"/>
+    </row>
+    <row r="26" ht="150" customHeight="1">
       <c r="A26" s="14" t="n">
         <v>13</v>
       </c>
@@ -1784,12 +2310,12 @@
           <t>Metal</t>
         </is>
       </c>
-      <c r="E26" s="15" t="inlineStr">
+      <c r="E26" s="14" t="inlineStr">
         <is>
           <t>Laiton patiné foncé martelé</t>
         </is>
       </c>
-      <c r="F26" s="15" t="inlineStr">
+      <c r="F26" s="14" t="inlineStr">
         <is>
           <t>Dark patinated hammered brass</t>
         </is>
@@ -1799,51 +2325,51 @@
           <t>Martelé, vernis mat</t>
         </is>
       </c>
-      <c r="H26" s="15" t="inlineStr">
+      <c r="H26" s="14" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT-A/8, K5M-T1B1-SDB-B/14</t>
         </is>
       </c>
-      <c r="I26" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
+      <c r="I26" s="15" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Lato"/>
               <color rgb="00292B2B"/>
-              <sz val="1000"/>
+              <sz val="11"/>
             </rPr>
             <t>Entrée: handle (A/8). SDB: handle (B/14).</t>
           </r>
         </is>
       </c>
-      <c r="J26" s="17" t="inlineStr">
+      <c r="J26" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K26" s="17" t="inlineStr">
+      <c r="K26" s="16" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L26" s="18" t="inlineStr"/>
-      <c r="M26" s="19" t="inlineStr">
+      <c r="L26" s="17" t="inlineStr"/>
+      <c r="M26" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N26" s="18" t="inlineStr"/>
-      <c r="O26" s="18" t="inlineStr"/>
-      <c r="P26" s="18" t="inlineStr"/>
-      <c r="Q26" s="18" t="inlineStr"/>
-      <c r="R26" s="18" t="inlineStr"/>
-      <c r="S26" s="15" t="inlineStr">
+      <c r="N26" s="17" t="inlineStr"/>
+      <c r="O26" s="17" t="inlineStr"/>
+      <c r="P26" s="17" t="inlineStr"/>
+      <c r="Q26" s="17" t="inlineStr"/>
+      <c r="R26" s="17" t="inlineStr"/>
+      <c r="S26" s="14" t="inlineStr">
         <is>
           <t>Compound finish: dark patina base + hammered (martelé) texture applied on top — the only clear compound case in Fit-out</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="34" customHeight="1">
+    <row r="27" ht="150" customHeight="1">
       <c r="A27" s="14" t="n">
         <v>14</v>
       </c>
@@ -1858,12 +2384,12 @@
           <t>Glass/Mirror</t>
         </is>
       </c>
-      <c r="E27" s="15" t="inlineStr">
+      <c r="E27" s="14" t="inlineStr">
         <is>
           <t>Miroir extra-clair</t>
         </is>
       </c>
-      <c r="F27" s="15" t="inlineStr">
+      <c r="F27" s="14" t="inlineStr">
         <is>
           <t>Extra-clear mirror</t>
         </is>
@@ -1873,52 +2399,52 @@
           <t>Extra-clair</t>
         </is>
       </c>
-      <c r="H27" s="15" t="inlineStr">
+      <c r="H27" s="14" t="inlineStr">
         <is>
           <t>K5M-T1B1-SDB-B/13, K5M-T1B1-CHA-C/7</t>
         </is>
       </c>
-      <c r="I27" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
+      <c r="I27" s="15" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Lato"/>
               <color rgb="00E4572E"/>
-              <sz val="1000"/>
+              <sz val="11"/>
               <u val="single"/>
             </rPr>
             <t>SDB: mirror (B/13, three-part with light between — confirm no light suspension is our scope). Chambre: mirror in banquette arch (C/7).</t>
           </r>
         </is>
       </c>
-      <c r="J27" s="17" t="inlineStr">
+      <c r="J27" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K27" s="17" t="inlineStr">
+      <c r="K27" s="16" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L27" s="18" t="inlineStr"/>
-      <c r="M27" s="19" t="inlineStr">
+      <c r="L27" s="17" t="inlineStr"/>
+      <c r="M27" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N27" s="18" t="inlineStr"/>
-      <c r="O27" s="18" t="inlineStr"/>
-      <c r="P27" s="18" t="inlineStr"/>
-      <c r="Q27" s="18" t="inlineStr"/>
-      <c r="R27" s="18" t="inlineStr"/>
-      <c r="S27" s="15" t="inlineStr">
+      <c r="N27" s="17" t="inlineStr"/>
+      <c r="O27" s="17" t="inlineStr"/>
+      <c r="P27" s="17" t="inlineStr"/>
+      <c r="Q27" s="17" t="inlineStr"/>
+      <c r="R27" s="17" t="inlineStr"/>
+      <c r="S27" s="14" t="inlineStr">
         <is>
           <t>Confirm scope boundary on B/13's inter-panel lighting (per RFI remark)</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="20" customHeight="1">
+    <row r="28" ht="150" customHeight="1">
       <c r="A28" s="14" t="n">
         <v>15</v>
       </c>
@@ -1933,12 +2459,12 @@
           <t>Glass/Mirror</t>
         </is>
       </c>
-      <c r="E28" s="15" t="inlineStr">
+      <c r="E28" s="14" t="inlineStr">
         <is>
           <t>Miroir extra-clair antique</t>
         </is>
       </c>
-      <c r="F28" s="15" t="inlineStr">
+      <c r="F28" s="14" t="inlineStr">
         <is>
           <t>Antique extra-clear mirror</t>
         </is>
@@ -1948,47 +2474,47 @@
           <t>Antique</t>
         </is>
       </c>
-      <c r="H28" s="15" t="inlineStr">
+      <c r="H28" s="14" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT</t>
         </is>
       </c>
-      <c r="I28" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
+      <c r="I28" s="15" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Lato"/>
               <color rgb="00292B2B"/>
-              <sz val="1000"/>
+              <sz val="11"/>
             </rPr>
             <t>Entrée: mini-bar interior panel.</t>
           </r>
         </is>
       </c>
-      <c r="J28" s="17" t="inlineStr">
+      <c r="J28" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K28" s="17" t="inlineStr">
+      <c r="K28" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L28" s="18" t="inlineStr"/>
-      <c r="M28" s="19" t="inlineStr">
+      <c r="L28" s="17" t="inlineStr"/>
+      <c r="M28" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N28" s="18" t="inlineStr"/>
-      <c r="O28" s="18" t="inlineStr"/>
-      <c r="P28" s="18" t="inlineStr"/>
-      <c r="Q28" s="18" t="inlineStr"/>
-      <c r="R28" s="18" t="inlineStr"/>
-      <c r="S28" s="15" t="inlineStr"/>
-    </row>
-    <row r="29" ht="34" customHeight="1">
+      <c r="N28" s="17" t="inlineStr"/>
+      <c r="O28" s="17" t="inlineStr"/>
+      <c r="P28" s="17" t="inlineStr"/>
+      <c r="Q28" s="17" t="inlineStr"/>
+      <c r="R28" s="17" t="inlineStr"/>
+      <c r="S28" s="14" t="inlineStr"/>
+    </row>
+    <row r="29" ht="150" customHeight="1">
       <c r="A29" s="14" t="n">
         <v>16</v>
       </c>
@@ -2003,59 +2529,59 @@
           <t>Glass</t>
         </is>
       </c>
-      <c r="E29" s="15" t="inlineStr">
+      <c r="E29" s="14" t="inlineStr">
         <is>
           <t>Verre extra-clair + lin</t>
         </is>
       </c>
-      <c r="F29" s="15" t="inlineStr">
+      <c r="F29" s="14" t="inlineStr">
         <is>
           <t>Extra-clear glass + linen</t>
         </is>
       </c>
       <c r="G29" s="14" t="inlineStr"/>
-      <c r="H29" s="15" t="inlineStr">
+      <c r="H29" s="14" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT-A/8, K5M-T1B1-SDB-B/14</t>
         </is>
       </c>
-      <c r="I29" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
+      <c r="I29" s="15" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Lato"/>
               <color rgb="00E4572E"/>
-              <sz val="1000"/>
+              <sz val="11"/>
               <u val="single"/>
             </rPr>
             <t>Entrée: door/dressing panels (A/8). SDB: door panels (B/14). Glass reference image still needed.</t>
           </r>
         </is>
       </c>
-      <c r="J29" s="17" t="inlineStr">
+      <c r="J29" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K29" s="17" t="inlineStr">
+      <c r="K29" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L29" s="18" t="inlineStr"/>
-      <c r="M29" s="19" t="inlineStr">
+      <c r="L29" s="17" t="inlineStr"/>
+      <c r="M29" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N29" s="18" t="inlineStr"/>
-      <c r="O29" s="18" t="inlineStr"/>
-      <c r="P29" s="18" t="inlineStr"/>
-      <c r="Q29" s="18" t="inlineStr"/>
-      <c r="R29" s="18" t="inlineStr"/>
-      <c r="S29" s="15" t="inlineStr"/>
-    </row>
-    <row r="30" ht="20" customHeight="1">
+      <c r="N29" s="17" t="inlineStr"/>
+      <c r="O29" s="17" t="inlineStr"/>
+      <c r="P29" s="17" t="inlineStr"/>
+      <c r="Q29" s="17" t="inlineStr"/>
+      <c r="R29" s="17" t="inlineStr"/>
+      <c r="S29" s="14" t="inlineStr"/>
+    </row>
+    <row r="30" ht="150" customHeight="1">
       <c r="A30" s="14" t="n">
         <v>17</v>
       </c>
@@ -2070,58 +2596,58 @@
           <t>Glass</t>
         </is>
       </c>
-      <c r="E30" s="15" t="inlineStr">
+      <c r="E30" s="14" t="inlineStr">
         <is>
           <t>Verre extra-clair</t>
         </is>
       </c>
-      <c r="F30" s="15" t="inlineStr">
+      <c r="F30" s="14" t="inlineStr">
         <is>
           <t>Extra-clear glass</t>
         </is>
       </c>
       <c r="G30" s="14" t="inlineStr"/>
-      <c r="H30" s="15" t="inlineStr">
+      <c r="H30" s="14" t="inlineStr">
         <is>
           <t>K5M-T1B1-SDB</t>
         </is>
       </c>
-      <c r="I30" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
+      <c r="I30" s="15" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Lato"/>
               <color rgb="00292B2B"/>
-              <sz val="1000"/>
+              <sz val="11"/>
             </rPr>
             <t>SDB: niche shelf.</t>
           </r>
         </is>
       </c>
-      <c r="J30" s="17" t="inlineStr">
+      <c r="J30" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K30" s="17" t="inlineStr">
+      <c r="K30" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L30" s="18" t="inlineStr"/>
-      <c r="M30" s="19" t="inlineStr">
+      <c r="L30" s="17" t="inlineStr"/>
+      <c r="M30" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N30" s="18" t="inlineStr"/>
-      <c r="O30" s="18" t="inlineStr"/>
-      <c r="P30" s="18" t="inlineStr"/>
-      <c r="Q30" s="18" t="inlineStr"/>
-      <c r="R30" s="18" t="inlineStr"/>
-      <c r="S30" s="15" t="inlineStr"/>
-    </row>
-    <row r="31" ht="34" customHeight="1">
+      <c r="N30" s="17" t="inlineStr"/>
+      <c r="O30" s="17" t="inlineStr"/>
+      <c r="P30" s="17" t="inlineStr"/>
+      <c r="Q30" s="17" t="inlineStr"/>
+      <c r="R30" s="17" t="inlineStr"/>
+      <c r="S30" s="14" t="inlineStr"/>
+    </row>
+    <row r="31" ht="150" customHeight="1">
       <c r="A31" s="14" t="n">
         <v>18</v>
       </c>
@@ -2136,62 +2662,62 @@
           <t>Paint</t>
         </is>
       </c>
-      <c r="E31" s="15" t="inlineStr">
+      <c r="E31" s="14" t="inlineStr">
         <is>
           <t>Peinture texturée blanche</t>
         </is>
       </c>
-      <c r="F31" s="15" t="inlineStr">
+      <c r="F31" s="14" t="inlineStr">
         <is>
           <t>White textured paint</t>
         </is>
       </c>
       <c r="G31" s="14" t="inlineStr"/>
-      <c r="H31" s="15" t="inlineStr">
+      <c r="H31" s="14" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT, K5M-T1B1-SDB, K5M-T1B1-CHA</t>
         </is>
       </c>
-      <c r="I31" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
+      <c r="I31" s="15" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Lato"/>
               <color rgb="00292B2B"/>
-              <sz val="1000"/>
+              <sz val="11"/>
             </rPr>
             <t>Entrée: ceiling+wall (excluded from BOQ). SDB: ceiling/cornice/wall (excluded). Chambre: cornice (excluded).</t>
           </r>
         </is>
       </c>
-      <c r="J31" s="17" t="inlineStr">
+      <c r="J31" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K31" s="17" t="inlineStr">
+      <c r="K31" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="L31" s="18" t="inlineStr"/>
-      <c r="M31" s="19" t="inlineStr">
+      <c r="L31" s="17" t="inlineStr"/>
+      <c r="M31" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N31" s="18" t="inlineStr"/>
-      <c r="O31" s="18" t="inlineStr"/>
-      <c r="P31" s="18" t="inlineStr"/>
-      <c r="Q31" s="18" t="inlineStr"/>
-      <c r="R31" s="18" t="inlineStr"/>
-      <c r="S31" s="15" t="inlineStr">
+      <c r="N31" s="17" t="inlineStr"/>
+      <c r="O31" s="17" t="inlineStr"/>
+      <c r="P31" s="17" t="inlineStr"/>
+      <c r="Q31" s="17" t="inlineStr"/>
+      <c r="R31" s="17" t="inlineStr"/>
+      <c r="S31" s="14" t="inlineStr">
         <is>
           <t>Painting is EXCLUDED from the awarded BOQ scope per client — tracked here for material reference only</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="20" customHeight="1">
+    <row r="32" ht="150" customHeight="1">
       <c r="A32" s="14" t="n">
         <v>19</v>
       </c>
@@ -2206,62 +2732,62 @@
           <t>Paint</t>
         </is>
       </c>
-      <c r="E32" s="15" t="inlineStr">
+      <c r="E32" s="14" t="inlineStr">
         <is>
           <t>Peinture texturée beige</t>
         </is>
       </c>
-      <c r="F32" s="15" t="inlineStr">
+      <c r="F32" s="14" t="inlineStr">
         <is>
           <t>Beige textured paint</t>
         </is>
       </c>
       <c r="G32" s="14" t="inlineStr"/>
-      <c r="H32" s="15" t="inlineStr">
+      <c r="H32" s="14" t="inlineStr">
         <is>
           <t>K5M-T1B1-CHA</t>
         </is>
       </c>
-      <c r="I32" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
+      <c r="I32" s="15" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Lato"/>
               <color rgb="00292B2B"/>
-              <sz val="1000"/>
+              <sz val="11"/>
             </rPr>
             <t>Chambre: ceiling (excluded from BOQ).</t>
           </r>
         </is>
       </c>
-      <c r="J32" s="17" t="inlineStr">
+      <c r="J32" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K32" s="17" t="inlineStr">
+      <c r="K32" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="L32" s="18" t="inlineStr"/>
-      <c r="M32" s="19" t="inlineStr">
+      <c r="L32" s="17" t="inlineStr"/>
+      <c r="M32" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N32" s="18" t="inlineStr"/>
-      <c r="O32" s="18" t="inlineStr"/>
-      <c r="P32" s="18" t="inlineStr"/>
-      <c r="Q32" s="18" t="inlineStr"/>
-      <c r="R32" s="18" t="inlineStr"/>
-      <c r="S32" s="15" t="inlineStr">
+      <c r="N32" s="17" t="inlineStr"/>
+      <c r="O32" s="17" t="inlineStr"/>
+      <c r="P32" s="17" t="inlineStr"/>
+      <c r="Q32" s="17" t="inlineStr"/>
+      <c r="R32" s="17" t="inlineStr"/>
+      <c r="S32" s="14" t="inlineStr">
         <is>
           <t>Excluded from awarded BOQ scope</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="34" customHeight="1">
+    <row r="33" ht="150" customHeight="1">
       <c r="A33" s="14" t="n">
         <v>20</v>
       </c>
@@ -2276,63 +2802,63 @@
           <t>Wallpaper</t>
         </is>
       </c>
-      <c r="E33" s="15" t="inlineStr">
+      <c r="E33" s="14" t="inlineStr">
         <is>
           <t>Papier peint (Omexco)</t>
         </is>
       </c>
-      <c r="F33" s="15" t="inlineStr">
+      <c r="F33" s="14" t="inlineStr">
         <is>
           <t>Wallpaper (Omexco)</t>
         </is>
       </c>
       <c r="G33" s="14" t="inlineStr"/>
-      <c r="H33" s="15" t="inlineStr">
+      <c r="H33" s="14" t="inlineStr">
         <is>
           <t>K5M-T1B1-CHA-C/6</t>
         </is>
       </c>
-      <c r="I33" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
+      <c r="I33" s="15" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Lato"/>
               <color rgb="00E4572E"/>
-              <sz val="1000"/>
+              <sz val="11"/>
               <u val="single"/>
             </rPr>
             <t>Chambre: wall — explicitly EXCLUDED from our BOQ offer per C/6 remark.</t>
           </r>
         </is>
       </c>
-      <c r="J33" s="17" t="inlineStr">
+      <c r="J33" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K33" s="17" t="inlineStr">
+      <c r="K33" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="L33" s="18" t="inlineStr"/>
-      <c r="M33" s="19" t="inlineStr">
+      <c r="L33" s="17" t="inlineStr"/>
+      <c r="M33" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N33" s="18" t="inlineStr"/>
-      <c r="O33" s="18" t="inlineStr"/>
-      <c r="P33" s="18" t="inlineStr"/>
-      <c r="Q33" s="18" t="inlineStr"/>
-      <c r="R33" s="18" t="inlineStr"/>
-      <c r="S33" s="15" t="inlineStr">
+      <c r="N33" s="17" t="inlineStr"/>
+      <c r="O33" s="17" t="inlineStr"/>
+      <c r="P33" s="17" t="inlineStr"/>
+      <c r="Q33" s="17" t="inlineStr"/>
+      <c r="R33" s="17" t="inlineStr"/>
+      <c r="S33" s="14" t="inlineStr">
         <is>
           <t>Supply/installation of this wallpaper is explicitly excluded in our BOQ offer (see C/6)</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="20" customHeight="1">
+    <row r="34" ht="150" customHeight="1">
       <c r="A34" s="14" t="n">
         <v>21</v>
       </c>
@@ -2347,58 +2873,58 @@
           <t>Wallpaper</t>
         </is>
       </c>
-      <c r="E34" s="15" t="inlineStr">
+      <c r="E34" s="14" t="inlineStr">
         <is>
           <t>Papier peint (Biobject)</t>
         </is>
       </c>
-      <c r="F34" s="15" t="inlineStr">
+      <c r="F34" s="14" t="inlineStr">
         <is>
           <t>Wallpaper (Biobject)</t>
         </is>
       </c>
       <c r="G34" s="14" t="inlineStr"/>
-      <c r="H34" s="15" t="inlineStr">
+      <c r="H34" s="14" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT</t>
         </is>
       </c>
-      <c r="I34" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
+      <c r="I34" s="15" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Lato"/>
               <color rgb="00292B2B"/>
-              <sz val="1000"/>
+              <sz val="11"/>
             </rPr>
             <t>Entrée: luggage-rack drawer interior panel.</t>
           </r>
         </is>
       </c>
-      <c r="J34" s="17" t="inlineStr">
+      <c r="J34" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K34" s="17" t="inlineStr">
+      <c r="K34" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L34" s="18" t="inlineStr"/>
-      <c r="M34" s="19" t="inlineStr">
+      <c r="L34" s="17" t="inlineStr"/>
+      <c r="M34" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N34" s="18" t="inlineStr"/>
-      <c r="O34" s="18" t="inlineStr"/>
-      <c r="P34" s="18" t="inlineStr"/>
-      <c r="Q34" s="18" t="inlineStr"/>
-      <c r="R34" s="18" t="inlineStr"/>
-      <c r="S34" s="15" t="inlineStr"/>
-    </row>
-    <row r="35" ht="48" customHeight="1">
+      <c r="N34" s="17" t="inlineStr"/>
+      <c r="O34" s="17" t="inlineStr"/>
+      <c r="P34" s="17" t="inlineStr"/>
+      <c r="Q34" s="17" t="inlineStr"/>
+      <c r="R34" s="17" t="inlineStr"/>
+      <c r="S34" s="14" t="inlineStr"/>
+    </row>
+    <row r="35" ht="150" customHeight="1">
       <c r="A35" s="14" t="n">
         <v>22</v>
       </c>
@@ -2413,12 +2939,12 @@
           <t>Carpet</t>
         </is>
       </c>
-      <c r="E35" s="15" t="inlineStr">
+      <c r="E35" s="14" t="inlineStr">
         <is>
           <t>Moquette (Design Carpet - Ali Laraqui)</t>
         </is>
       </c>
-      <c r="F35" s="15" t="inlineStr">
+      <c r="F35" s="14" t="inlineStr">
         <is>
           <t>Carpet (Design Carpet - Ali Laraqui)</t>
         </is>
@@ -2428,51 +2954,51 @@
           <t>Tapis encastré / Inset carpet</t>
         </is>
       </c>
-      <c r="H35" s="15" t="inlineStr">
+      <c r="H35" s="14" t="inlineStr">
         <is>
           <t>K5M-T1B1-COULOIRS</t>
         </is>
       </c>
-      <c r="I35" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
+      <c r="I35" s="15" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Lato"/>
               <color rgb="00292B2B"/>
-              <sz val="1000"/>
+              <sz val="11"/>
             </rPr>
             <t>Corridors (Hall/bedroom corridors) — inset carpet. Also appears in Victoire's 21 Jul global soft-materials list alongside FF&amp;E fabric codes — kept in Fit-out only per our scope-separation rule.</t>
           </r>
         </is>
       </c>
-      <c r="J35" s="17" t="inlineStr">
+      <c r="J35" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K35" s="17" t="inlineStr">
+      <c r="K35" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L35" s="18" t="inlineStr"/>
-      <c r="M35" s="19" t="inlineStr">
+      <c r="L35" s="17" t="inlineStr"/>
+      <c r="M35" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N35" s="18" t="inlineStr"/>
-      <c r="O35" s="18" t="inlineStr"/>
-      <c r="P35" s="18" t="inlineStr"/>
-      <c r="Q35" s="18" t="inlineStr"/>
-      <c r="R35" s="18" t="inlineStr"/>
-      <c r="S35" s="15" t="inlineStr">
+      <c r="N35" s="17" t="inlineStr"/>
+      <c r="O35" s="17" t="inlineStr"/>
+      <c r="P35" s="17" t="inlineStr"/>
+      <c r="Q35" s="17" t="inlineStr"/>
+      <c r="R35" s="17" t="inlineStr"/>
+      <c r="S35" s="14" t="inlineStr">
         <is>
           <t>Confirm carpet remains Wood Couture scope (open decision noted in earlier Fit-out audit)</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="34" customHeight="1">
+    <row r="36" ht="150" customHeight="1">
       <c r="A36" s="14" t="n">
         <v>23</v>
       </c>
@@ -2487,12 +3013,12 @@
           <t>Stone</t>
         </is>
       </c>
-      <c r="E36" s="15" t="inlineStr">
+      <c r="E36" s="14" t="inlineStr">
         <is>
           <t>Travertin osso (vein cut / cross cut) — NOUVEAU 21 Jul</t>
         </is>
       </c>
-      <c r="F36" s="15" t="inlineStr">
+      <c r="F36" s="14" t="inlineStr">
         <is>
           <t>Travertine osso (vein cut / cross cut) — NEW 21 Jul</t>
         </is>
@@ -2502,48 +3028,48 @@
           <t>Adouci / Honed</t>
         </is>
       </c>
-      <c r="H36" s="15" t="inlineStr"/>
-      <c r="I36" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
+      <c r="H36" s="14" t="inlineStr"/>
+      <c r="I36" s="15" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Lato"/>
               <color rgb="00E4572E"/>
-              <sz val="1000"/>
+              <sz val="11"/>
               <u val="single"/>
             </rPr>
             <t>No location assigned yet in any document reviewed.</t>
           </r>
         </is>
       </c>
-      <c r="J36" s="17" t="inlineStr">
+      <c r="J36" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K36" s="17" t="inlineStr">
+      <c r="K36" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L36" s="18" t="inlineStr"/>
-      <c r="M36" s="19" t="inlineStr">
+      <c r="L36" s="17" t="inlineStr"/>
+      <c r="M36" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N36" s="18" t="inlineStr"/>
-      <c r="O36" s="18" t="inlineStr"/>
-      <c r="P36" s="18" t="inlineStr"/>
-      <c r="Q36" s="18" t="inlineStr"/>
-      <c r="R36" s="18" t="inlineStr"/>
-      <c r="S36" s="15" t="inlineStr">
+      <c r="N36" s="17" t="inlineStr"/>
+      <c r="O36" s="17" t="inlineStr"/>
+      <c r="P36" s="17" t="inlineStr"/>
+      <c r="Q36" s="17" t="inlineStr"/>
+      <c r="R36" s="17" t="inlineStr"/>
+      <c r="S36" s="14" t="inlineStr">
         <is>
           <t>New codes as of 21 Jul 2026 — location/application not yet confirmed, ask Adil</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="34" customHeight="1">
+    <row r="37" ht="150" customHeight="1">
       <c r="A37" s="14" t="n">
         <v>24</v>
       </c>
@@ -2558,12 +3084,12 @@
           <t>Wood</t>
         </is>
       </c>
-      <c r="E37" s="15" t="inlineStr">
+      <c r="E37" s="14" t="inlineStr">
         <is>
           <t>Tatawi peint en blanc — NOUVEAU 21 Jul</t>
         </is>
       </c>
-      <c r="F37" s="15" t="inlineStr">
+      <c r="F37" s="14" t="inlineStr">
         <is>
           <t>White-painted Tatawi wood — NEW 21 Jul</t>
         </is>
@@ -2573,42 +3099,42 @@
           <t>Mat</t>
         </is>
       </c>
-      <c r="H37" s="15" t="inlineStr"/>
-      <c r="I37" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
+      <c r="H37" s="14" t="inlineStr"/>
+      <c r="I37" s="15" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Lato"/>
               <color rgb="00E4572E"/>
-              <sz val="1000"/>
+              <sz val="11"/>
               <u val="single"/>
             </rPr>
             <t>No location assigned yet in any document reviewed.</t>
           </r>
         </is>
       </c>
-      <c r="J37" s="17" t="inlineStr">
+      <c r="J37" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K37" s="17" t="inlineStr">
+      <c r="K37" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L37" s="18" t="inlineStr"/>
-      <c r="M37" s="19" t="inlineStr">
+      <c r="L37" s="17" t="inlineStr"/>
+      <c r="M37" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N37" s="18" t="inlineStr"/>
-      <c r="O37" s="18" t="inlineStr"/>
-      <c r="P37" s="18" t="inlineStr"/>
-      <c r="Q37" s="18" t="inlineStr"/>
-      <c r="R37" s="18" t="inlineStr"/>
-      <c r="S37" s="15" t="inlineStr">
+      <c r="N37" s="17" t="inlineStr"/>
+      <c r="O37" s="17" t="inlineStr"/>
+      <c r="P37" s="17" t="inlineStr"/>
+      <c r="Q37" s="17" t="inlineStr"/>
+      <c r="R37" s="17" t="inlineStr"/>
+      <c r="S37" s="14" t="inlineStr">
         <is>
           <t>New code as of 21 Jul 2026 — location/application not yet confirmed, ask Adil</t>
         </is>
@@ -2622,5 +3148,6 @@
     <mergeCell ref="A12:S12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fitout Material Package: apply user review feedback
- Remove paint/wallpaper/carpet (out of scope): 24 -> 19 rows, listed in EXCLUDED footnote
- Fix High-Res Available Y -> N (only low-res PDF crops exist, not true high-res)
- Fully translate Localization column to English (was mixing French location nouns)
- Localization header now cites source explicitly: "per DD-100, dated 21.07.2026"
- Add disclaimer: FM-xxx are internal cross-references, not official RFI numbers
  (confirmed via full repo/branch search - not found in any real RFI log)
- Mark Control Sample / High-Res as N/A for rows with no confirmed scope/task code
- Add Status column conditional formatting matching legend colors (auto-recolors on edit)
- Fix pre-existing bug: Total row was silently overwritten by a merged caveat note
</commit_message>
<xml_diff>
--- a/material_package_fitout/260727_K5M_Material Package_Fitout.xlsx
+++ b/material_package_fitout/260727_K5M_Material Package_Fitout.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -63,6 +63,12 @@
       <name val="Lato"/>
       <i val="1"/>
       <color rgb="00E4572E"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Lato"/>
+      <i val="1"/>
+      <color rgb="00292B2B"/>
       <sz val="8"/>
     </font>
   </fonts>
@@ -140,7 +146,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -167,6 +173,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -184,10 +191,97 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="6">
+    <dxf>
+      <font>
+        <name val="Lato"/>
+        <b val="1"/>
+        <color rgb="00FFFFFF"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="0073BA9B"/>
+          <bgColor rgb="0073BA9B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Lato"/>
+        <b val="1"/>
+        <color rgb="00FFFFFF"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00BC8A7E"/>
+          <bgColor rgb="00BC8A7E"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Lato"/>
+        <b val="1"/>
+        <color rgb="00FFFFFF"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00E4572E"/>
+          <bgColor rgb="00E4572E"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Lato"/>
+        <b val="1"/>
+        <color rgb="00292B2B"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFF07C"/>
+          <bgColor rgb="00FFF07C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Lato"/>
+        <b val="1"/>
+        <color rgb="00FFFFFF"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="0026547C"/>
+          <bgColor rgb="0026547C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Lato"/>
+        <b val="1"/>
+        <color rgb="00FFFFFF"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00A7A7A7"/>
+          <bgColor rgb="00A7A7A7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -266,7 +360,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>13</row>
+      <row>15</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="571500" cy="547914"/>
@@ -291,7 +385,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>14</row>
+      <row>16</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="571500" cy="547914"/>
@@ -316,7 +410,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>15</row>
+      <row>17</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="571500" cy="538842"/>
@@ -341,7 +435,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>16</row>
+      <row>18</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="571500" cy="547914"/>
@@ -366,7 +460,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>17</row>
+      <row>19</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="571500" cy="537028"/>
@@ -391,7 +485,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>18</row>
+      <row>20</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="571500" cy="551542"/>
@@ -416,7 +510,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>20</row>
+      <row>22</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="571500" cy="555171"/>
@@ -441,7 +535,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>21</row>
+      <row>23</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="571500" cy="551542"/>
@@ -466,7 +560,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>22</row>
+      <row>24</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="571500" cy="431799"/>
@@ -491,7 +585,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>23</row>
+      <row>25</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="571500" cy="547914"/>
@@ -516,7 +610,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>24</row>
+      <row>26</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="571500" cy="549728"/>
@@ -541,7 +635,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>25</row>
+      <row>27</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="571500" cy="547914"/>
@@ -566,7 +660,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>26</row>
+      <row>28</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="571500" cy="537028"/>
@@ -591,7 +685,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>27</row>
+      <row>29</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="571500" cy="533400"/>
@@ -616,7 +710,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>28</row>
+      <row>30</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="571500" cy="571500"/>
@@ -641,10 +735,10 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>30</row>
+      <row>32</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="571500" cy="533400"/>
+    <ext cx="571500" cy="547914"/>
     <pic>
       <nvPicPr>
         <cNvPr id="16" name="Image 16" descr="Picture"/>
@@ -666,10 +760,10 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>31</row>
+      <row>33</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="571500" cy="571500"/>
+    <ext cx="571500" cy="551542"/>
     <pic>
       <nvPicPr>
         <cNvPr id="17" name="Image 17" descr="Picture"/>
@@ -677,106 +771,6 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId17"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>32</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="571500" cy="537028"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="18" name="Image 18" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId18"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>33</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="571500" cy="551542"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="19" name="Image 19" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId19"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>35</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="571500" cy="547914"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="20" name="Image 20" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId20"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>36</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="571500" cy="551542"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="21" name="Image 21" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId21"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1113,7 +1107,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of 27 July 2026 — first version. Localization sourced from DD-100 only (governs over BOQ text per G&amp;B/Victoire, 23 Jul). Underlined localizations are still unresolved / to be re-raised with Adil directly — not force-resolved here.</t>
+          <t>As of 27 July 2026 — V2: paint/wallpaper/carpet removed (out of Fit-out scope). Localization is sourced only from the DD-100-tagged material list dated 21.07.2026 (DD-100 governs over BOQ text where they conflict, per G&amp;B/Victoire 23 Jul) — never from the BOQ or Victoire's separate global soft-materials list. Underlined localizations are still unresolved / to be re-raised with Adil directly — not force-resolved here.</t>
         </is>
       </c>
     </row>
@@ -1136,7 +1130,7 @@
         </is>
       </c>
       <c r="C5" s="5">
-        <f>COUNTIF(M13:M200,"A")</f>
+        <f>COUNTIF(M16:M200,"A")</f>
         <v/>
       </c>
     </row>
@@ -1152,7 +1146,7 @@
         </is>
       </c>
       <c r="C6" s="5">
-        <f>COUNTIF(M13:M200,"B")</f>
+        <f>COUNTIF(M16:M200,"B")</f>
         <v/>
       </c>
     </row>
@@ -1168,7 +1162,7 @@
         </is>
       </c>
       <c r="C7" s="5">
-        <f>COUNTIF(M13:M200,"C")</f>
+        <f>COUNTIF(M16:M200,"C")</f>
         <v/>
       </c>
     </row>
@@ -1184,7 +1178,7 @@
         </is>
       </c>
       <c r="C8" s="5">
-        <f>COUNTIF(M13:M200,"S")</f>
+        <f>COUNTIF(M16:M200,"S")</f>
         <v/>
       </c>
     </row>
@@ -1200,7 +1194,7 @@
         </is>
       </c>
       <c r="C9" s="5">
-        <f>COUNTIF(M13:M200,"T")</f>
+        <f>COUNTIF(M16:M200,"T")</f>
         <v/>
       </c>
     </row>
@@ -1216,151 +1210,169 @@
         </is>
       </c>
       <c r="C10" s="5">
-        <f>COUNTIF(M13:M200,"O")</f>
+        <f>COUNTIF(M16:M200,"O")</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C11" s="3">
+        <f>COUNTA(M16:M200)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>Same proposed status-color extension as the FFE sheet (B/S colors not officially brand-defined) — confirm or replace. Status defaulted to T (To be Submitted) for every row as a starting point.</t>
         </is>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13" ht="68" customHeight="1">
+    <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
+          <t>FM-xxx labels used in Localization/Remarks are internal cross-references created for this sheet only — not official RFI numbers from any project RFI log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15" ht="68" customHeight="1">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>Material Code</t>
         </is>
       </c>
-      <c r="C13" s="12" t="inlineStr">
+      <c r="C15" s="13" t="inlineStr">
         <is>
           <t>Thumbnail</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr">
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="E13" s="12" t="inlineStr">
+      <c r="E15" s="13" t="inlineStr">
         <is>
           <t>Description (FR)</t>
         </is>
       </c>
-      <c r="F13" s="12" t="inlineStr">
+      <c r="F15" s="13" t="inlineStr">
         <is>
           <t>Description (EN)</t>
         </is>
       </c>
-      <c r="G13" s="12" t="inlineStr">
+      <c r="G15" s="13" t="inlineStr">
         <is>
           <t>Finish / Vernish</t>
         </is>
       </c>
-      <c r="H13" s="12" t="inlineStr">
+      <c r="H15" s="13" t="inlineStr">
         <is>
           <t>Applicable Task Code(s) (WDCO)</t>
         </is>
       </c>
-      <c r="I13" s="12" t="inlineStr">
-        <is>
-          <t>Localization per DD-100 (underlined = still under scrutiny with Adil)</t>
-        </is>
-      </c>
-      <c r="J13" s="12" t="inlineStr">
+      <c r="I15" s="13" t="inlineStr">
+        <is>
+          <t>Localization per DD-100, dated 21.07.2026 (underlined = still under scrutiny with Adil)</t>
+        </is>
+      </c>
+      <c r="J15" s="13" t="inlineStr">
         <is>
           <t>Control Sample (Y/N)</t>
         </is>
       </c>
-      <c r="K13" s="12" t="inlineStr">
+      <c r="K15" s="13" t="inlineStr">
         <is>
           <t>High-Res Available (Y/N)</t>
         </is>
       </c>
-      <c r="L13" s="12" t="inlineStr">
+      <c r="L15" s="13" t="inlineStr">
         <is>
           <t>High-Res Link</t>
         </is>
       </c>
-      <c r="M13" s="13" t="inlineStr">
+      <c r="M15" s="14" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="N13" s="13" t="inlineStr">
+      <c r="N15" s="14" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="O13" s="13" t="inlineStr">
+      <c r="O15" s="14" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="P13" s="13" t="inlineStr">
+      <c r="P15" s="14" t="inlineStr">
         <is>
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="Q13" s="13" t="inlineStr">
+      <c r="Q15" s="14" t="inlineStr">
         <is>
           <t>2026-08-17</t>
         </is>
       </c>
-      <c r="R13" s="13" t="inlineStr">
+      <c r="R15" s="14" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="S13" s="12" t="inlineStr">
+      <c r="S15" s="13" t="inlineStr">
         <is>
           <t>Remarks / Open Issues</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="150" customHeight="1">
-      <c r="A14" s="14" t="n">
+    <row r="16" ht="150" customHeight="1">
+      <c r="A16" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="B14" s="14" t="inlineStr">
+      <c r="B16" s="15" t="inlineStr">
         <is>
           <t>A-ST-01c</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
-      <c r="D14" s="14" t="inlineStr">
+      <c r="C16" s="15" t="inlineStr"/>
+      <c r="D16" s="15" t="inlineStr">
         <is>
           <t>Stone</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr">
+      <c r="E16" s="15" t="inlineStr">
         <is>
           <t>Beige clair</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
+      <c r="F16" s="15" t="inlineStr">
         <is>
           <t>Light beige stone</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr">
+      <c r="G16" s="15" t="inlineStr">
         <is>
           <t>Adouci / Honed</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>K5M-T1B1-ENT-A/? (seuil), K5M-T1B1-SDB-B/6, K5M-T1B1-SDB-B/12, K5M-T1B1-CHA-C/2, K5M-T1B1-CHA-C/3</t>
-        </is>
-      </c>
-      <c r="I14" s="15" t="inlineStr">
+      <c r="H16" s="15" t="inlineStr">
+        <is>
+          <t>K5M-T1B1-ENT-A/? (threshold), K5M-T1B1-SDB-B/6, K5M-T1B1-SDB-B/12, K5M-T1B1-CHA-C/2, K5M-T1B1-CHA-C/3</t>
+        </is>
+      </c>
+      <c r="I16" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1368,7 +1380,7 @@
               <color rgb="00292B2B"/>
               <sz val="11"/>
             </rPr>
-            <t xml:space="preserve">Entrée: seuil. </t>
+            <t xml:space="preserve">Entrance: threshold. </t>
           </r>
           <r>
             <rPr>
@@ -1377,7 +1389,7 @@
               <sz val="11"/>
               <u val="single"/>
             </rPr>
-            <t xml:space="preserve">SDB: arche toilette/douche, niche (conflicts with BOQ A-ST-07a on niche — see FM-007). </t>
+            <t xml:space="preserve">Bathroom: toilet/shower arch, niche (conflicts with BOQ A-ST-07a on niche — see FM-007). </t>
           </r>
           <r>
             <rPr>
@@ -1386,73 +1398,73 @@
               <sz val="11"/>
               <u val="single"/>
             </rPr>
-            <t>Chambre: seuil (C/3, joint code conflict — see FM-010), plinthe (C/2, conflicts with A-ST-01e/A-ST-02c in updated list — see FM-009).</t>
+            <t>Bedroom: threshold (C/3, joint code conflict — see FM-010), baseboard (C/2, conflicts with A-ST-01e/A-ST-02c in updated list — see FM-009).</t>
           </r>
         </is>
       </c>
-      <c r="J14" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K14" s="16" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="L14" s="17" t="inlineStr"/>
-      <c r="M14" s="18" t="inlineStr">
+      <c r="J16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L16" s="18" t="inlineStr"/>
+      <c r="M16" s="19" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N14" s="17" t="inlineStr"/>
-      <c r="O14" s="17" t="inlineStr"/>
-      <c r="P14" s="17" t="inlineStr"/>
-      <c r="Q14" s="17" t="inlineStr"/>
-      <c r="R14" s="17" t="inlineStr"/>
-      <c r="S14" s="14" t="inlineStr">
+      <c r="N16" s="18" t="inlineStr"/>
+      <c r="O16" s="18" t="inlineStr"/>
+      <c r="P16" s="18" t="inlineStr"/>
+      <c r="Q16" s="18" t="inlineStr"/>
+      <c r="R16" s="18" t="inlineStr"/>
+      <c r="S16" s="15" t="inlineStr">
         <is>
           <t>See FM-007, FM-009, FM-010 — all still open, to re-raise with Adil</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="150" customHeight="1">
-      <c r="A15" s="14" t="n">
+    <row r="17" ht="150" customHeight="1">
+      <c r="A17" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B15" s="14" t="inlineStr">
+      <c r="B17" s="15" t="inlineStr">
         <is>
           <t>A-ST-01d</t>
         </is>
       </c>
-      <c r="C15" s="14" t="inlineStr"/>
-      <c r="D15" s="14" t="inlineStr">
+      <c r="C17" s="15" t="inlineStr"/>
+      <c r="D17" s="15" t="inlineStr">
         <is>
           <t>Stone</t>
         </is>
       </c>
-      <c r="E15" s="14" t="inlineStr">
+      <c r="E17" s="15" t="inlineStr">
         <is>
           <t>Beige clair</t>
         </is>
       </c>
-      <c r="F15" s="14" t="inlineStr">
+      <c r="F17" s="15" t="inlineStr">
         <is>
           <t>Light beige stone</t>
         </is>
       </c>
-      <c r="G15" s="14" t="inlineStr">
+      <c r="G17" s="15" t="inlineStr">
         <is>
           <t>Anti-dérapant / Anti-slip</t>
         </is>
       </c>
-      <c r="H15" s="14" t="inlineStr">
+      <c r="H17" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-SDB-B/2, K5M-T1B1-SDB-B/5</t>
         </is>
       </c>
-      <c r="I15" s="15" t="inlineStr">
+      <c r="I17" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1460,7 +1472,7 @@
               <color rgb="00292B2B"/>
               <sz val="11"/>
             </rPr>
-            <t xml:space="preserve">SDB: sol douche (shower floor). </t>
+            <t xml:space="preserve">Bathroom: shower floor. </t>
           </r>
           <r>
             <rPr>
@@ -1473,69 +1485,69 @@
           </r>
         </is>
       </c>
-      <c r="J15" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K15" s="16" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="L15" s="17" t="inlineStr"/>
-      <c r="M15" s="18" t="inlineStr">
+      <c r="J17" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K17" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L17" s="18" t="inlineStr"/>
+      <c r="M17" s="19" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N15" s="17" t="inlineStr"/>
-      <c r="O15" s="17" t="inlineStr"/>
-      <c r="P15" s="17" t="inlineStr"/>
-      <c r="Q15" s="17" t="inlineStr"/>
-      <c r="R15" s="17" t="inlineStr"/>
-      <c r="S15" s="14" t="inlineStr">
+      <c r="N17" s="18" t="inlineStr"/>
+      <c r="O17" s="18" t="inlineStr"/>
+      <c r="P17" s="18" t="inlineStr"/>
+      <c r="Q17" s="18" t="inlineStr"/>
+      <c r="R17" s="18" t="inlineStr"/>
+      <c r="S17" s="15" t="inlineStr">
         <is>
           <t>See FM-005, FM-012</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="150" customHeight="1">
-      <c r="A16" s="14" t="n">
+    <row r="18" ht="150" customHeight="1">
+      <c r="A18" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="B16" s="14" t="inlineStr">
+      <c r="B18" s="15" t="inlineStr">
         <is>
           <t>A-ST-01e</t>
         </is>
       </c>
-      <c r="C16" s="14" t="inlineStr"/>
-      <c r="D16" s="14" t="inlineStr">
+      <c r="C18" s="15" t="inlineStr"/>
+      <c r="D18" s="15" t="inlineStr">
         <is>
           <t>Stone</t>
         </is>
       </c>
-      <c r="E16" s="14" t="inlineStr">
+      <c r="E18" s="15" t="inlineStr">
         <is>
           <t>Beige clair</t>
         </is>
       </c>
-      <c r="F16" s="14" t="inlineStr">
+      <c r="F18" s="15" t="inlineStr">
         <is>
           <t>Light beige stone</t>
         </is>
       </c>
-      <c r="G16" s="14" t="inlineStr">
+      <c r="G18" s="15" t="inlineStr">
         <is>
           <t>Martelé / Hammered</t>
         </is>
       </c>
-      <c r="H16" s="14" t="inlineStr">
+      <c r="H18" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT-A/1, K5M-T1B1-SDB-B/1</t>
         </is>
       </c>
-      <c r="I16" s="15" t="inlineStr">
+      <c r="I18" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1543,69 +1555,69 @@
               <color rgb="00292B2B"/>
               <sz val="11"/>
             </rPr>
-            <t>Entrée: sol. SDB: sol. Hall/corridor floor per BOQ item 1 (Hall Ascenseurs).</t>
+            <t>Entrance: floor. Bathroom: floor. Hall/corridor floor per BOQ item 1 (Elevator Hall).</t>
           </r>
         </is>
       </c>
-      <c r="J16" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K16" s="16" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="L16" s="17" t="inlineStr"/>
-      <c r="M16" s="18" t="inlineStr">
+      <c r="J18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr"/>
+      <c r="M18" s="19" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N16" s="17" t="inlineStr"/>
-      <c r="O16" s="17" t="inlineStr"/>
-      <c r="P16" s="17" t="inlineStr"/>
-      <c r="Q16" s="17" t="inlineStr"/>
-      <c r="R16" s="17" t="inlineStr"/>
-      <c r="S16" s="14" t="inlineStr"/>
-    </row>
-    <row r="17" ht="150" customHeight="1">
-      <c r="A17" s="14" t="n">
+      <c r="N18" s="18" t="inlineStr"/>
+      <c r="O18" s="18" t="inlineStr"/>
+      <c r="P18" s="18" t="inlineStr"/>
+      <c r="Q18" s="18" t="inlineStr"/>
+      <c r="R18" s="18" t="inlineStr"/>
+      <c r="S18" s="15" t="inlineStr"/>
+    </row>
+    <row r="19" ht="150" customHeight="1">
+      <c r="A19" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B17" s="14" t="inlineStr">
+      <c r="B19" s="15" t="inlineStr">
         <is>
           <t>A-ST-02c</t>
         </is>
       </c>
-      <c r="C17" s="14" t="inlineStr"/>
-      <c r="D17" s="14" t="inlineStr">
+      <c r="C19" s="15" t="inlineStr"/>
+      <c r="D19" s="15" t="inlineStr">
         <is>
           <t>Stone</t>
         </is>
       </c>
-      <c r="E17" s="14" t="inlineStr">
+      <c r="E19" s="15" t="inlineStr">
         <is>
           <t>Beige foncé</t>
         </is>
       </c>
-      <c r="F17" s="14" t="inlineStr">
+      <c r="F19" s="15" t="inlineStr">
         <is>
           <t>Dark beige stone</t>
         </is>
       </c>
-      <c r="G17" s="14" t="inlineStr">
+      <c r="G19" s="15" t="inlineStr">
         <is>
           <t>Adouci / Honed</t>
         </is>
       </c>
-      <c r="H17" s="14" t="inlineStr">
+      <c r="H19" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT-A/1, K5M-T1B1-SDB-B/1, K5M-T1B1-SDB-B/3, K5M-T1B1-CHA-C/2</t>
         </is>
       </c>
-      <c r="I17" s="15" t="inlineStr">
+      <c r="I19" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1613,7 +1625,7 @@
               <color rgb="00292B2B"/>
               <sz val="11"/>
             </rPr>
-            <t xml:space="preserve">Entrée: sol. SDB: sol, plinthe. </t>
+            <t xml:space="preserve">Entrance: floor. Bathroom: floor, baseboard. </t>
           </r>
           <r>
             <rPr>
@@ -1622,73 +1634,73 @@
               <sz val="11"/>
               <u val="single"/>
             </rPr>
-            <t>Chambre: plinthe (C/2) — conflicts with A-ST-01c/A-ST-01e, see FM-009.</t>
+            <t>Bedroom: baseboard (C/2) — conflicts with A-ST-01c/A-ST-01e, see FM-009.</t>
           </r>
         </is>
       </c>
-      <c r="J17" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K17" s="16" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="L17" s="17" t="inlineStr"/>
-      <c r="M17" s="18" t="inlineStr">
+      <c r="J19" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K19" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L19" s="18" t="inlineStr"/>
+      <c r="M19" s="19" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N17" s="17" t="inlineStr"/>
-      <c r="O17" s="17" t="inlineStr"/>
-      <c r="P17" s="17" t="inlineStr"/>
-      <c r="Q17" s="17" t="inlineStr"/>
-      <c r="R17" s="17" t="inlineStr"/>
-      <c r="S17" s="14" t="inlineStr">
+      <c r="N19" s="18" t="inlineStr"/>
+      <c r="O19" s="18" t="inlineStr"/>
+      <c r="P19" s="18" t="inlineStr"/>
+      <c r="Q19" s="18" t="inlineStr"/>
+      <c r="R19" s="18" t="inlineStr"/>
+      <c r="S19" s="15" t="inlineStr">
         <is>
           <t>See FM-009</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="150" customHeight="1">
-      <c r="A18" s="14" t="n">
+    <row r="20" ht="150" customHeight="1">
+      <c r="A20" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="B18" s="14" t="inlineStr">
+      <c r="B20" s="15" t="inlineStr">
         <is>
           <t>A-ST-07a</t>
         </is>
       </c>
-      <c r="C18" s="14" t="inlineStr"/>
-      <c r="D18" s="14" t="inlineStr">
+      <c r="C20" s="15" t="inlineStr"/>
+      <c r="D20" s="15" t="inlineStr">
         <is>
           <t>Stone</t>
         </is>
       </c>
-      <c r="E18" s="14" t="inlineStr">
+      <c r="E20" s="15" t="inlineStr">
         <is>
           <t>Onyx miel — REMPLACÉ PAR Taj Mahal</t>
         </is>
       </c>
-      <c r="F18" s="14" t="inlineStr">
+      <c r="F20" s="15" t="inlineStr">
         <is>
           <t>Onyx Honey — REPLACED BY Taj Mahal</t>
         </is>
       </c>
-      <c r="G18" s="14" t="inlineStr">
+      <c r="G20" s="15" t="inlineStr">
         <is>
           <t>Poli / Polished</t>
         </is>
       </c>
-      <c r="H18" s="14" t="inlineStr">
-        <is>
-          <t>K5M-T1B1-ENT-A (arche/porte-bagage), K5M-T1B1-SDB-B/7, K5M-T1B1-SDB-B/8, K5M-T1B1-SDB-B/9, K5M-T1B1-SDB-B/10, K5M-T1B1-SDB-B/11, K5M-T1B1-SDB-B/12, K5M-T1B1-CHA-C/4</t>
-        </is>
-      </c>
-      <c r="I18" s="15" t="inlineStr">
+      <c r="H20" s="15" t="inlineStr">
+        <is>
+          <t>K5M-T1B1-ENT-A (arch/luggage rack), K5M-T1B1-SDB-B/7, K5M-T1B1-SDB-B/8, K5M-T1B1-SDB-B/9, K5M-T1B1-SDB-B/10, K5M-T1B1-SDB-B/11, K5M-T1B1-SDB-B/12, K5M-T1B1-CHA-C/4</t>
+        </is>
+      </c>
+      <c r="I20" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1696,7 +1708,7 @@
               <color rgb="00292B2B"/>
               <sz val="11"/>
             </rPr>
-            <t xml:space="preserve">Entrée: arche, porte-bagage. SDB: banc (B/7, B/8), tablette WC (B/9), vasque (B/10), arche vasque (B/11). </t>
+            <t xml:space="preserve">Entrance: arch, luggage rack. Bathroom: bench (B/7, B/8), toilet shelf (B/9), sink (B/10), sink arch (B/11). </t>
           </r>
           <r>
             <rPr>
@@ -1705,7 +1717,7 @@
               <sz val="11"/>
               <u val="single"/>
             </rPr>
-            <t>SDB niche (B/12) — same code shown twice in updated list (superseded honey-onyx row retained alongside Taj Mahal replacement) — see FM-002 and FM-007.</t>
+            <t>Bathroom niche (B/12) — same code shown twice in updated list (superseded honey-onyx row retained alongside Taj Mahal replacement) — see FM-002 and FM-007.</t>
           </r>
           <r>
             <rPr>
@@ -1713,73 +1725,73 @@
               <color rgb="00292B2B"/>
               <sz val="11"/>
             </rPr>
-            <t xml:space="preserve"> Chambre: arche (C/4).</t>
+            <t xml:space="preserve"> Bedroom: arch (C/4).</t>
           </r>
         </is>
       </c>
-      <c r="J18" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K18" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L18" s="17" t="inlineStr"/>
-      <c r="M18" s="18" t="inlineStr">
+      <c r="J20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L20" s="18" t="inlineStr"/>
+      <c r="M20" s="19" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N18" s="17" t="inlineStr"/>
-      <c r="O18" s="17" t="inlineStr"/>
-      <c r="P18" s="17" t="inlineStr"/>
-      <c r="Q18" s="17" t="inlineStr"/>
-      <c r="R18" s="17" t="inlineStr"/>
-      <c r="S18" s="14" t="inlineStr">
+      <c r="N20" s="18" t="inlineStr"/>
+      <c r="O20" s="18" t="inlineStr"/>
+      <c r="P20" s="18" t="inlineStr"/>
+      <c r="Q20" s="18" t="inlineStr"/>
+      <c r="R20" s="18" t="inlineStr"/>
+      <c r="S20" s="15" t="inlineStr">
         <is>
           <t>SUBSTITUTED as of 21 Jul 2026 update. See FM-002, FM-007 — confirm Taj Mahal applies everywhere, honey onyx no longer valid anywhere</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="150" customHeight="1">
-      <c r="A19" s="14" t="n">
+    <row r="21" ht="150" customHeight="1">
+      <c r="A21" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="B19" s="14" t="inlineStr">
+      <c r="B21" s="15" t="inlineStr">
         <is>
           <t>A-WD-01b</t>
         </is>
       </c>
-      <c r="C19" s="14" t="inlineStr"/>
-      <c r="D19" s="14" t="inlineStr">
+      <c r="C21" s="15" t="inlineStr"/>
+      <c r="D21" s="15" t="inlineStr">
         <is>
           <t>Wood</t>
         </is>
       </c>
-      <c r="E19" s="14" t="inlineStr">
+      <c r="E21" s="15" t="inlineStr">
         <is>
           <t>Noyer — REMPLACÉ PAR chêne teinté moyen</t>
         </is>
       </c>
-      <c r="F19" s="14" t="inlineStr">
+      <c r="F21" s="15" t="inlineStr">
         <is>
           <t>Walnut — REPLACED BY medium-tinted oak</t>
         </is>
       </c>
-      <c r="G19" s="14" t="inlineStr">
+      <c r="G21" s="15" t="inlineStr">
         <is>
           <t>Satin</t>
         </is>
       </c>
-      <c r="H19" s="14" t="inlineStr">
+      <c r="H21" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT-A/7, K5M-T1B1-CHA-C/7</t>
         </is>
       </c>
-      <c r="I19" s="15" t="inlineStr">
+      <c r="I21" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1788,7 +1800,7 @@
               <sz val="11"/>
               <u val="single"/>
             </rPr>
-            <t xml:space="preserve">Entrée: porte, architrave, plinthe (A/7). </t>
+            <t xml:space="preserve">Entrance: door, architrave, baseboard (A/7). </t>
           </r>
           <r>
             <rPr>
@@ -1797,69 +1809,69 @@
               <sz val="11"/>
               <u val="single"/>
             </rPr>
-            <t>Chambre: tablette (C/7). BOQ uses three code variants (A-WD-01d, generic A-WD-01, A-WD-01b) for these — see FM-001.</t>
+            <t>Bedroom: shelf (C/7). BOQ uses three code variants (A-WD-01d, generic A-WD-01, A-WD-01b) for these — see FM-001.</t>
           </r>
         </is>
       </c>
-      <c r="J19" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K19" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L19" s="17" t="inlineStr"/>
-      <c r="M19" s="18" t="inlineStr">
+      <c r="J21" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K21" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L21" s="18" t="inlineStr"/>
+      <c r="M21" s="19" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N19" s="17" t="inlineStr"/>
-      <c r="O19" s="17" t="inlineStr"/>
-      <c r="P19" s="17" t="inlineStr"/>
-      <c r="Q19" s="17" t="inlineStr"/>
-      <c r="R19" s="17" t="inlineStr"/>
-      <c r="S19" s="14" t="inlineStr">
+      <c r="N21" s="18" t="inlineStr"/>
+      <c r="O21" s="18" t="inlineStr"/>
+      <c r="P21" s="18" t="inlineStr"/>
+      <c r="Q21" s="18" t="inlineStr"/>
+      <c r="R21" s="18" t="inlineStr"/>
+      <c r="S21" s="15" t="inlineStr">
         <is>
           <t>SUBSTITUTED as of 21 Jul 2026. See FM-001 — confirm all four applications follow this code/finish</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="150" customHeight="1">
-      <c r="A20" s="14" t="n">
+    <row r="22" ht="150" customHeight="1">
+      <c r="A22" s="15" t="n">
         <v>7</v>
       </c>
-      <c r="B20" s="14" t="inlineStr">
+      <c r="B22" s="15" t="inlineStr">
         <is>
           <t>A-WD-01d</t>
         </is>
       </c>
-      <c r="C20" s="14" t="inlineStr"/>
-      <c r="D20" s="14" t="inlineStr">
+      <c r="C22" s="15" t="inlineStr"/>
+      <c r="D22" s="15" t="inlineStr">
         <is>
           <t>Wood</t>
         </is>
       </c>
-      <c r="E20" s="14" t="inlineStr">
+      <c r="E22" s="15" t="inlineStr">
         <is>
           <t>(absent de la liste officielle des matériaux)</t>
         </is>
       </c>
-      <c r="F20" s="14" t="inlineStr">
+      <c r="F22" s="15" t="inlineStr">
         <is>
           <t>(does not appear in the official material list at all)</t>
         </is>
       </c>
-      <c r="G20" s="14" t="inlineStr"/>
-      <c r="H20" s="14" t="inlineStr">
+      <c r="G22" s="15" t="inlineStr"/>
+      <c r="H22" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT-A/2, K5M-T1B1-ENT-A/4</t>
         </is>
       </c>
-      <c r="I20" s="15" t="inlineStr">
+      <c r="I22" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1868,73 +1880,73 @@
               <sz val="11"/>
               <u val="single"/>
             </rPr>
-            <t xml:space="preserve">Entrée: plinthe (A/2), arche (A/4) — code only exists in the BOQ/RFI, not in any material list issue. </t>
+            <t xml:space="preserve">Entrance: baseboard (A/2), arch (A/4) — code only exists in the BOQ/RFI, not in any material list issue. </t>
           </r>
         </is>
       </c>
-      <c r="J20" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K20" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L20" s="17" t="inlineStr"/>
-      <c r="M20" s="18" t="inlineStr">
+      <c r="J22" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K22" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L22" s="18" t="inlineStr"/>
+      <c r="M22" s="19" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N20" s="17" t="inlineStr"/>
-      <c r="O20" s="17" t="inlineStr"/>
-      <c r="P20" s="17" t="inlineStr"/>
-      <c r="Q20" s="17" t="inlineStr"/>
-      <c r="R20" s="17" t="inlineStr"/>
-      <c r="S20" s="14" t="inlineStr">
+      <c r="N22" s="18" t="inlineStr"/>
+      <c r="O22" s="18" t="inlineStr"/>
+      <c r="P22" s="18" t="inlineStr"/>
+      <c r="Q22" s="18" t="inlineStr"/>
+      <c r="R22" s="18" t="inlineStr"/>
+      <c r="S22" s="15" t="inlineStr">
         <is>
           <t>See FM-001. RFI already flags: no material reference image provided for this code</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="150" customHeight="1">
-      <c r="A21" s="14" t="n">
+    <row r="23" ht="150" customHeight="1">
+      <c r="A23" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="B21" s="14" t="inlineStr">
+      <c r="B23" s="15" t="inlineStr">
         <is>
           <t>A-WD-02c</t>
         </is>
       </c>
-      <c r="C21" s="14" t="inlineStr"/>
-      <c r="D21" s="14" t="inlineStr">
+      <c r="C23" s="15" t="inlineStr"/>
+      <c r="D23" s="15" t="inlineStr">
         <is>
           <t>Wood</t>
         </is>
       </c>
-      <c r="E21" s="14" t="inlineStr">
+      <c r="E23" s="15" t="inlineStr">
         <is>
           <t>Chêne cérusé blanc</t>
         </is>
       </c>
-      <c r="F21" s="14" t="inlineStr">
+      <c r="F23" s="15" t="inlineStr">
         <is>
           <t>White cerused oak</t>
         </is>
       </c>
-      <c r="G21" s="14" t="inlineStr">
+      <c r="G23" s="15" t="inlineStr">
         <is>
           <t>Mat / Matte</t>
         </is>
       </c>
-      <c r="H21" s="14" t="inlineStr">
+      <c r="H23" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT-A/8, K5M-T1B1-SDB-B/14, K5M-T1B1-CHA-C/6</t>
         </is>
       </c>
-      <c r="I21" s="15" t="inlineStr">
+      <c r="I23" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1942,7 +1954,7 @@
               <color rgb="00292B2B"/>
               <sz val="11"/>
             </rPr>
-            <t xml:space="preserve">Entrée: contour/tiroir/dressings (A/8). SDB: contour portes (B/14). </t>
+            <t xml:space="preserve">Entrance: surround/drawer/closets (A/8). Bathroom: door surround (B/14). </t>
           </r>
           <r>
             <rPr>
@@ -1951,73 +1963,73 @@
               <sz val="11"/>
               <u val="single"/>
             </rPr>
-            <t>Chambre: wall panels per BOQ (C/6), but updated material-list location only mentions banquette, not wall panelling — see FM-011.</t>
+            <t>Bedroom: wall panels per BOQ (C/6), but updated material-list location only mentions banquette, not wall panelling — see FM-011.</t>
           </r>
         </is>
       </c>
-      <c r="J21" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K21" s="16" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="L21" s="17" t="inlineStr"/>
-      <c r="M21" s="18" t="inlineStr">
+      <c r="J23" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K23" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L23" s="18" t="inlineStr"/>
+      <c r="M23" s="19" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N21" s="17" t="inlineStr"/>
-      <c r="O21" s="17" t="inlineStr"/>
-      <c r="P21" s="17" t="inlineStr"/>
-      <c r="Q21" s="17" t="inlineStr"/>
-      <c r="R21" s="17" t="inlineStr"/>
-      <c r="S21" s="14" t="inlineStr">
+      <c r="N23" s="18" t="inlineStr"/>
+      <c r="O23" s="18" t="inlineStr"/>
+      <c r="P23" s="18" t="inlineStr"/>
+      <c r="Q23" s="18" t="inlineStr"/>
+      <c r="R23" s="18" t="inlineStr"/>
+      <c r="S23" s="15" t="inlineStr">
         <is>
           <t>See FM-011</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="150" customHeight="1">
-      <c r="A22" s="14" t="n">
+    <row r="24" ht="150" customHeight="1">
+      <c r="A24" s="15" t="n">
         <v>9</v>
       </c>
-      <c r="B22" s="14" t="inlineStr">
+      <c r="B24" s="15" t="inlineStr">
         <is>
           <t>A-WD-04b</t>
         </is>
       </c>
-      <c r="C22" s="14" t="inlineStr"/>
-      <c r="D22" s="14" t="inlineStr">
+      <c r="C24" s="15" t="inlineStr"/>
+      <c r="D24" s="15" t="inlineStr">
         <is>
           <t>Wood</t>
         </is>
       </c>
-      <c r="E22" s="14" t="inlineStr">
+      <c r="E24" s="15" t="inlineStr">
         <is>
           <t>Parquet chêne teinté moyen (Hakwood Idéal)</t>
         </is>
       </c>
-      <c r="F22" s="14" t="inlineStr">
+      <c r="F24" s="15" t="inlineStr">
         <is>
           <t>Medium-tinted oak parquet (Hakwood Idéal)</t>
         </is>
       </c>
-      <c r="G22" s="14" t="inlineStr">
+      <c r="G24" s="15" t="inlineStr">
         <is>
           <t>Satin</t>
         </is>
       </c>
-      <c r="H22" s="14" t="inlineStr">
+      <c r="H24" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-CHA-C/1</t>
         </is>
       </c>
-      <c r="I22" s="15" t="inlineStr">
+      <c r="I24" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2026,7 +2038,7 @@
               <sz val="11"/>
               <u val="single"/>
             </rPr>
-            <t xml:space="preserve">Chambre: sol (floor). </t>
+            <t xml:space="preserve">Bedroom floor. </t>
           </r>
           <r>
             <rPr>
@@ -2039,69 +2051,69 @@
           </r>
         </is>
       </c>
-      <c r="J22" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K22" s="16" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="L22" s="17" t="inlineStr"/>
-      <c r="M22" s="18" t="inlineStr">
+      <c r="J24" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K24" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L24" s="18" t="inlineStr"/>
+      <c r="M24" s="19" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N22" s="17" t="inlineStr"/>
-      <c r="O22" s="17" t="inlineStr"/>
-      <c r="P22" s="17" t="inlineStr"/>
-      <c r="Q22" s="17" t="inlineStr"/>
-      <c r="R22" s="17" t="inlineStr"/>
-      <c r="S22" s="14" t="inlineStr">
+      <c r="N24" s="18" t="inlineStr"/>
+      <c r="O24" s="18" t="inlineStr"/>
+      <c r="P24" s="18" t="inlineStr"/>
+      <c r="Q24" s="18" t="inlineStr"/>
+      <c r="R24" s="18" t="inlineStr"/>
+      <c r="S24" s="15" t="inlineStr">
         <is>
           <t>SUBSTITUTED from dark-tinted to medium-tinted oak, 21 Jul 2026, real product ref (Hakwood, Idéal). See FM-008</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="150" customHeight="1">
-      <c r="A23" s="14" t="n">
+    <row r="25" ht="150" customHeight="1">
+      <c r="A25" s="15" t="n">
         <v>10</v>
       </c>
-      <c r="B23" s="14" t="inlineStr">
+      <c r="B25" s="15" t="inlineStr">
         <is>
           <t>A-ME-01a</t>
         </is>
       </c>
-      <c r="C23" s="14" t="inlineStr"/>
-      <c r="D23" s="14" t="inlineStr">
+      <c r="C25" s="15" t="inlineStr"/>
+      <c r="D25" s="15" t="inlineStr">
         <is>
           <t>Metal</t>
         </is>
       </c>
-      <c r="E23" s="14" t="inlineStr">
+      <c r="E25" s="15" t="inlineStr">
         <is>
           <t>Acier inoxydable poli</t>
         </is>
       </c>
-      <c r="F23" s="14" t="inlineStr">
+      <c r="F25" s="15" t="inlineStr">
         <is>
           <t>Polished stainless steel</t>
         </is>
       </c>
-      <c r="G23" s="14" t="inlineStr">
+      <c r="G25" s="15" t="inlineStr">
         <is>
           <t>Finition poli miroir</t>
         </is>
       </c>
-      <c r="H23" s="14" t="inlineStr">
+      <c r="H25" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-SDB-B/8, K5M-T1B1-SDB-B/14</t>
         </is>
       </c>
-      <c r="I23" s="15" t="inlineStr">
+      <c r="I25" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2110,7 +2122,7 @@
               <sz val="11"/>
               <u val="single"/>
             </rPr>
-            <t>SDB: bench structure/base (B/8) — not explicitly confirmed in updated material-list locations, see FM-006. Door handle/frame (B/14).</t>
+            <t>Bathroom: bench structure/base (B/8) — not explicitly confirmed in updated material-list locations, see FM-006. Door handle/frame (B/14).</t>
           </r>
           <r>
             <rPr>
@@ -2119,73 +2131,73 @@
               <sz val="11"/>
               <u val="single"/>
             </rPr>
-            <t xml:space="preserve"> Original (27 Oct 2025) list located this at Entrée tringle instead — location moved in the 21 Jul update; A-ME-01h now covers the Entrée tringle.</t>
+            <t xml:space="preserve"> Original (27 Oct 2025) list located this at the Entrance rail instead — location moved in the 21 Jul update; A-ME-01h now covers the Entrance rail.</t>
           </r>
         </is>
       </c>
-      <c r="J23" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K23" s="16" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="L23" s="17" t="inlineStr"/>
-      <c r="M23" s="18" t="inlineStr">
+      <c r="J25" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K25" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L25" s="18" t="inlineStr"/>
+      <c r="M25" s="19" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N23" s="17" t="inlineStr"/>
-      <c r="O23" s="17" t="inlineStr"/>
-      <c r="P23" s="17" t="inlineStr"/>
-      <c r="Q23" s="17" t="inlineStr"/>
-      <c r="R23" s="17" t="inlineStr"/>
-      <c r="S23" s="14" t="inlineStr">
+      <c r="N25" s="18" t="inlineStr"/>
+      <c r="O25" s="18" t="inlineStr"/>
+      <c r="P25" s="18" t="inlineStr"/>
+      <c r="Q25" s="18" t="inlineStr"/>
+      <c r="R25" s="18" t="inlineStr"/>
+      <c r="S25" s="15" t="inlineStr">
         <is>
           <t>See FM-006. Location changed between material list versions — confirm current assignment</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="150" customHeight="1">
-      <c r="A24" s="14" t="n">
+    <row r="26" ht="150" customHeight="1">
+      <c r="A26" s="15" t="n">
         <v>11</v>
       </c>
-      <c r="B24" s="14" t="inlineStr">
+      <c r="B26" s="15" t="inlineStr">
         <is>
           <t>A-ME-01h</t>
         </is>
       </c>
-      <c r="C24" s="14" t="inlineStr"/>
-      <c r="D24" s="14" t="inlineStr">
+      <c r="C26" s="15" t="inlineStr"/>
+      <c r="D26" s="15" t="inlineStr">
         <is>
           <t>Metal</t>
         </is>
       </c>
-      <c r="E24" s="14" t="inlineStr">
+      <c r="E26" s="15" t="inlineStr">
         <is>
           <t>Acier inoxydable brossé (NOUVEAU 21 Jul)</t>
         </is>
       </c>
-      <c r="F24" s="14" t="inlineStr">
+      <c r="F26" s="15" t="inlineStr">
         <is>
           <t>Brushed stainless steel (NEW 21 Jul)</t>
         </is>
       </c>
-      <c r="G24" s="14" t="inlineStr">
+      <c r="G26" s="15" t="inlineStr">
         <is>
           <t>Finition brossé</t>
         </is>
       </c>
-      <c r="H24" s="14" t="inlineStr">
+      <c r="H26" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT</t>
         </is>
       </c>
-      <c r="I24" s="15" t="inlineStr">
+      <c r="I26" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2194,73 +2206,73 @@
               <sz val="11"/>
               <u val="single"/>
             </rPr>
-            <t>Entrée: tringle (rail) — new code introduced 21 Jul 2026, appears to take over this location from A-ME-01a.</t>
+            <t>Entrance: rail — new code introduced 21 Jul 2026, appears to take over this location from A-ME-01a.</t>
           </r>
         </is>
       </c>
-      <c r="J24" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K24" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L24" s="17" t="inlineStr"/>
-      <c r="M24" s="18" t="inlineStr">
+      <c r="J26" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K26" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L26" s="18" t="inlineStr"/>
+      <c r="M26" s="19" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N24" s="17" t="inlineStr"/>
-      <c r="O24" s="17" t="inlineStr"/>
-      <c r="P24" s="17" t="inlineStr"/>
-      <c r="Q24" s="17" t="inlineStr"/>
-      <c r="R24" s="17" t="inlineStr"/>
-      <c r="S24" s="14" t="inlineStr">
+      <c r="N26" s="18" t="inlineStr"/>
+      <c r="O26" s="18" t="inlineStr"/>
+      <c r="P26" s="18" t="inlineStr"/>
+      <c r="Q26" s="18" t="inlineStr"/>
+      <c r="R26" s="18" t="inlineStr"/>
+      <c r="S26" s="15" t="inlineStr">
         <is>
           <t>New code as of 21 Jul 2026 update — confirm with Adil this is the correct replacement for the rail location</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="150" customHeight="1">
-      <c r="A25" s="14" t="n">
+    <row r="27" ht="150" customHeight="1">
+      <c r="A27" s="15" t="n">
         <v>12</v>
       </c>
-      <c r="B25" s="14" t="inlineStr">
+      <c r="B27" s="15" t="inlineStr">
         <is>
           <t>A-ME-02h</t>
         </is>
       </c>
-      <c r="C25" s="14" t="inlineStr"/>
-      <c r="D25" s="14" t="inlineStr">
+      <c r="C27" s="15" t="inlineStr"/>
+      <c r="D27" s="15" t="inlineStr">
         <is>
           <t>Metal</t>
         </is>
       </c>
-      <c r="E25" s="14" t="inlineStr">
+      <c r="E27" s="15" t="inlineStr">
         <is>
           <t>Laiton patiné foncé</t>
         </is>
       </c>
-      <c r="F25" s="14" t="inlineStr">
+      <c r="F27" s="15" t="inlineStr">
         <is>
           <t>Dark patinated brass</t>
         </is>
       </c>
-      <c r="G25" s="14" t="inlineStr">
+      <c r="G27" s="15" t="inlineStr">
         <is>
           <t>Vernis mat / Matte varnish</t>
         </is>
       </c>
-      <c r="H25" s="14" t="inlineStr">
+      <c r="H27" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT-A/7, K5M-T1B1-ENT-A/8, K5M-T1B1-SDB-B/13, K5M-T1B1-CHA-C/7</t>
         </is>
       </c>
-      <c r="I25" s="15" t="inlineStr">
+      <c r="I27" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2268,69 +2280,69 @@
               <color rgb="00292B2B"/>
               <sz val="11"/>
             </rPr>
-            <t>Entrée: door joint/trim (A/7, A/8). SDB: mirror joint/trim (B/13). Chambre: mirror joint/trim (C/7).</t>
+            <t>Entrance: door joint/trim (A/7, A/8). Bathroom: mirror joint/trim (B/13). Bedroom: mirror joint/trim (C/7).</t>
           </r>
         </is>
       </c>
-      <c r="J25" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K25" s="16" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="L25" s="17" t="inlineStr"/>
-      <c r="M25" s="18" t="inlineStr">
+      <c r="J27" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K27" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L27" s="18" t="inlineStr"/>
+      <c r="M27" s="19" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N25" s="17" t="inlineStr"/>
-      <c r="O25" s="17" t="inlineStr"/>
-      <c r="P25" s="17" t="inlineStr"/>
-      <c r="Q25" s="17" t="inlineStr"/>
-      <c r="R25" s="17" t="inlineStr"/>
-      <c r="S25" s="14" t="inlineStr"/>
-    </row>
-    <row r="26" ht="150" customHeight="1">
-      <c r="A26" s="14" t="n">
+      <c r="N27" s="18" t="inlineStr"/>
+      <c r="O27" s="18" t="inlineStr"/>
+      <c r="P27" s="18" t="inlineStr"/>
+      <c r="Q27" s="18" t="inlineStr"/>
+      <c r="R27" s="18" t="inlineStr"/>
+      <c r="S27" s="15" t="inlineStr"/>
+    </row>
+    <row r="28" ht="150" customHeight="1">
+      <c r="A28" s="15" t="n">
         <v>13</v>
       </c>
-      <c r="B26" s="14" t="inlineStr">
+      <c r="B28" s="15" t="inlineStr">
         <is>
           <t>A-ME-02i</t>
         </is>
       </c>
-      <c r="C26" s="14" t="inlineStr"/>
-      <c r="D26" s="14" t="inlineStr">
+      <c r="C28" s="15" t="inlineStr"/>
+      <c r="D28" s="15" t="inlineStr">
         <is>
           <t>Metal</t>
         </is>
       </c>
-      <c r="E26" s="14" t="inlineStr">
+      <c r="E28" s="15" t="inlineStr">
         <is>
           <t>Laiton patiné foncé martelé</t>
         </is>
       </c>
-      <c r="F26" s="14" t="inlineStr">
+      <c r="F28" s="15" t="inlineStr">
         <is>
           <t>Dark patinated hammered brass</t>
         </is>
       </c>
-      <c r="G26" s="14" t="inlineStr">
+      <c r="G28" s="15" t="inlineStr">
         <is>
           <t>Martelé, vernis mat</t>
         </is>
       </c>
-      <c r="H26" s="14" t="inlineStr">
+      <c r="H28" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT-A/8, K5M-T1B1-SDB-B/14</t>
         </is>
       </c>
-      <c r="I26" s="15" t="inlineStr">
+      <c r="I28" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2338,73 +2350,73 @@
               <color rgb="00292B2B"/>
               <sz val="11"/>
             </rPr>
-            <t>Entrée: handle (A/8). SDB: handle (B/14).</t>
+            <t>Entrance: handle (A/8). Bathroom: handle (B/14).</t>
           </r>
         </is>
       </c>
-      <c r="J26" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K26" s="16" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="L26" s="17" t="inlineStr"/>
-      <c r="M26" s="18" t="inlineStr">
+      <c r="J28" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K28" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L28" s="18" t="inlineStr"/>
+      <c r="M28" s="19" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N26" s="17" t="inlineStr"/>
-      <c r="O26" s="17" t="inlineStr"/>
-      <c r="P26" s="17" t="inlineStr"/>
-      <c r="Q26" s="17" t="inlineStr"/>
-      <c r="R26" s="17" t="inlineStr"/>
-      <c r="S26" s="14" t="inlineStr">
+      <c r="N28" s="18" t="inlineStr"/>
+      <c r="O28" s="18" t="inlineStr"/>
+      <c r="P28" s="18" t="inlineStr"/>
+      <c r="Q28" s="18" t="inlineStr"/>
+      <c r="R28" s="18" t="inlineStr"/>
+      <c r="S28" s="15" t="inlineStr">
         <is>
           <t>Compound finish: dark patina base + hammered (martelé) texture applied on top — the only clear compound case in Fit-out</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="150" customHeight="1">
-      <c r="A27" s="14" t="n">
+    <row r="29" ht="150" customHeight="1">
+      <c r="A29" s="15" t="n">
         <v>14</v>
       </c>
-      <c r="B27" s="14" t="inlineStr">
+      <c r="B29" s="15" t="inlineStr">
         <is>
           <t>A-GL-01a</t>
         </is>
       </c>
-      <c r="C27" s="14" t="inlineStr"/>
-      <c r="D27" s="14" t="inlineStr">
+      <c r="C29" s="15" t="inlineStr"/>
+      <c r="D29" s="15" t="inlineStr">
         <is>
           <t>Glass/Mirror</t>
         </is>
       </c>
-      <c r="E27" s="14" t="inlineStr">
+      <c r="E29" s="15" t="inlineStr">
         <is>
           <t>Miroir extra-clair</t>
         </is>
       </c>
-      <c r="F27" s="14" t="inlineStr">
+      <c r="F29" s="15" t="inlineStr">
         <is>
           <t>Extra-clear mirror</t>
         </is>
       </c>
-      <c r="G27" s="14" t="inlineStr">
+      <c r="G29" s="15" t="inlineStr">
         <is>
           <t>Extra-clair</t>
         </is>
       </c>
-      <c r="H27" s="14" t="inlineStr">
+      <c r="H29" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-SDB-B/13, K5M-T1B1-CHA-C/7</t>
         </is>
       </c>
-      <c r="I27" s="15" t="inlineStr">
+      <c r="I29" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2413,73 +2425,73 @@
               <sz val="11"/>
               <u val="single"/>
             </rPr>
-            <t>SDB: mirror (B/13, three-part with light between — confirm no light suspension is our scope). Chambre: mirror in banquette arch (C/7).</t>
+            <t>Bathroom: mirror (B/13, three-part with light between — confirm no light suspension is our scope). Bedroom: mirror in banquette arch (C/7).</t>
           </r>
         </is>
       </c>
-      <c r="J27" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K27" s="16" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="L27" s="17" t="inlineStr"/>
-      <c r="M27" s="18" t="inlineStr">
+      <c r="J29" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K29" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L29" s="18" t="inlineStr"/>
+      <c r="M29" s="19" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N27" s="17" t="inlineStr"/>
-      <c r="O27" s="17" t="inlineStr"/>
-      <c r="P27" s="17" t="inlineStr"/>
-      <c r="Q27" s="17" t="inlineStr"/>
-      <c r="R27" s="17" t="inlineStr"/>
-      <c r="S27" s="14" t="inlineStr">
+      <c r="N29" s="18" t="inlineStr"/>
+      <c r="O29" s="18" t="inlineStr"/>
+      <c r="P29" s="18" t="inlineStr"/>
+      <c r="Q29" s="18" t="inlineStr"/>
+      <c r="R29" s="18" t="inlineStr"/>
+      <c r="S29" s="15" t="inlineStr">
         <is>
           <t>Confirm scope boundary on B/13's inter-panel lighting (per RFI remark)</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="150" customHeight="1">
-      <c r="A28" s="14" t="n">
+    <row r="30" ht="150" customHeight="1">
+      <c r="A30" s="15" t="n">
         <v>15</v>
       </c>
-      <c r="B28" s="14" t="inlineStr">
+      <c r="B30" s="15" t="inlineStr">
         <is>
           <t>A-GL-02a</t>
         </is>
       </c>
-      <c r="C28" s="14" t="inlineStr"/>
-      <c r="D28" s="14" t="inlineStr">
+      <c r="C30" s="15" t="inlineStr"/>
+      <c r="D30" s="15" t="inlineStr">
         <is>
           <t>Glass/Mirror</t>
         </is>
       </c>
-      <c r="E28" s="14" t="inlineStr">
+      <c r="E30" s="15" t="inlineStr">
         <is>
           <t>Miroir extra-clair antique</t>
         </is>
       </c>
-      <c r="F28" s="14" t="inlineStr">
+      <c r="F30" s="15" t="inlineStr">
         <is>
           <t>Antique extra-clear mirror</t>
         </is>
       </c>
-      <c r="G28" s="14" t="inlineStr">
+      <c r="G30" s="15" t="inlineStr">
         <is>
           <t>Antique</t>
         </is>
       </c>
-      <c r="H28" s="14" t="inlineStr">
+      <c r="H30" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT</t>
         </is>
       </c>
-      <c r="I28" s="15" t="inlineStr">
+      <c r="I30" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2487,65 +2499,65 @@
               <color rgb="00292B2B"/>
               <sz val="11"/>
             </rPr>
-            <t>Entrée: mini-bar interior panel.</t>
+            <t>Entrance: mini-bar interior panel.</t>
           </r>
         </is>
       </c>
-      <c r="J28" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K28" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L28" s="17" t="inlineStr"/>
-      <c r="M28" s="18" t="inlineStr">
+      <c r="J30" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K30" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L30" s="18" t="inlineStr"/>
+      <c r="M30" s="19" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N28" s="17" t="inlineStr"/>
-      <c r="O28" s="17" t="inlineStr"/>
-      <c r="P28" s="17" t="inlineStr"/>
-      <c r="Q28" s="17" t="inlineStr"/>
-      <c r="R28" s="17" t="inlineStr"/>
-      <c r="S28" s="14" t="inlineStr"/>
-    </row>
-    <row r="29" ht="150" customHeight="1">
-      <c r="A29" s="14" t="n">
+      <c r="N30" s="18" t="inlineStr"/>
+      <c r="O30" s="18" t="inlineStr"/>
+      <c r="P30" s="18" t="inlineStr"/>
+      <c r="Q30" s="18" t="inlineStr"/>
+      <c r="R30" s="18" t="inlineStr"/>
+      <c r="S30" s="15" t="inlineStr"/>
+    </row>
+    <row r="31" ht="150" customHeight="1">
+      <c r="A31" s="15" t="n">
         <v>16</v>
       </c>
-      <c r="B29" s="14" t="inlineStr">
+      <c r="B31" s="15" t="inlineStr">
         <is>
           <t>A-GL-03a</t>
         </is>
       </c>
-      <c r="C29" s="14" t="inlineStr"/>
-      <c r="D29" s="14" t="inlineStr">
+      <c r="C31" s="15" t="inlineStr"/>
+      <c r="D31" s="15" t="inlineStr">
         <is>
           <t>Glass</t>
         </is>
       </c>
-      <c r="E29" s="14" t="inlineStr">
+      <c r="E31" s="15" t="inlineStr">
         <is>
           <t>Verre extra-clair + lin</t>
         </is>
       </c>
-      <c r="F29" s="14" t="inlineStr">
+      <c r="F31" s="15" t="inlineStr">
         <is>
           <t>Extra-clear glass + linen</t>
         </is>
       </c>
-      <c r="G29" s="14" t="inlineStr"/>
-      <c r="H29" s="14" t="inlineStr">
+      <c r="G31" s="15" t="inlineStr"/>
+      <c r="H31" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-ENT-A/8, K5M-T1B1-SDB-B/14</t>
         </is>
       </c>
-      <c r="I29" s="15" t="inlineStr">
+      <c r="I31" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2554,65 +2566,65 @@
               <sz val="11"/>
               <u val="single"/>
             </rPr>
-            <t>Entrée: door/dressing panels (A/8). SDB: door panels (B/14). Glass reference image still needed.</t>
+            <t>Entrance: door/closet panels (A/8). Bathroom: door panels (B/14). Glass reference image still needed.</t>
           </r>
         </is>
       </c>
-      <c r="J29" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K29" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L29" s="17" t="inlineStr"/>
-      <c r="M29" s="18" t="inlineStr">
+      <c r="J31" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K31" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L31" s="18" t="inlineStr"/>
+      <c r="M31" s="19" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N29" s="17" t="inlineStr"/>
-      <c r="O29" s="17" t="inlineStr"/>
-      <c r="P29" s="17" t="inlineStr"/>
-      <c r="Q29" s="17" t="inlineStr"/>
-      <c r="R29" s="17" t="inlineStr"/>
-      <c r="S29" s="14" t="inlineStr"/>
-    </row>
-    <row r="30" ht="150" customHeight="1">
-      <c r="A30" s="14" t="n">
+      <c r="N31" s="18" t="inlineStr"/>
+      <c r="O31" s="18" t="inlineStr"/>
+      <c r="P31" s="18" t="inlineStr"/>
+      <c r="Q31" s="18" t="inlineStr"/>
+      <c r="R31" s="18" t="inlineStr"/>
+      <c r="S31" s="15" t="inlineStr"/>
+    </row>
+    <row r="32" ht="150" customHeight="1">
+      <c r="A32" s="15" t="n">
         <v>17</v>
       </c>
-      <c r="B30" s="14" t="inlineStr">
+      <c r="B32" s="15" t="inlineStr">
         <is>
           <t>A-GL-04a</t>
         </is>
       </c>
-      <c r="C30" s="14" t="inlineStr"/>
-      <c r="D30" s="14" t="inlineStr">
+      <c r="C32" s="15" t="inlineStr"/>
+      <c r="D32" s="15" t="inlineStr">
         <is>
           <t>Glass</t>
         </is>
       </c>
-      <c r="E30" s="14" t="inlineStr">
+      <c r="E32" s="15" t="inlineStr">
         <is>
           <t>Verre extra-clair</t>
         </is>
       </c>
-      <c r="F30" s="14" t="inlineStr">
+      <c r="F32" s="15" t="inlineStr">
         <is>
           <t>Extra-clear glass</t>
         </is>
       </c>
-      <c r="G30" s="14" t="inlineStr"/>
-      <c r="H30" s="14" t="inlineStr">
+      <c r="G32" s="15" t="inlineStr"/>
+      <c r="H32" s="15" t="inlineStr">
         <is>
           <t>K5M-T1B1-SDB</t>
         </is>
       </c>
-      <c r="I30" s="15" t="inlineStr">
+      <c r="I32" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2620,416 +2632,65 @@
               <color rgb="00292B2B"/>
               <sz val="11"/>
             </rPr>
-            <t>SDB: niche shelf.</t>
+            <t>Bathroom: niche shelf.</t>
           </r>
         </is>
       </c>
-      <c r="J30" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K30" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L30" s="17" t="inlineStr"/>
-      <c r="M30" s="18" t="inlineStr">
+      <c r="J32" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K32" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L32" s="18" t="inlineStr"/>
+      <c r="M32" s="19" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N30" s="17" t="inlineStr"/>
-      <c r="O30" s="17" t="inlineStr"/>
-      <c r="P30" s="17" t="inlineStr"/>
-      <c r="Q30" s="17" t="inlineStr"/>
-      <c r="R30" s="17" t="inlineStr"/>
-      <c r="S30" s="14" t="inlineStr"/>
-    </row>
-    <row r="31" ht="150" customHeight="1">
-      <c r="A31" s="14" t="n">
+      <c r="N32" s="18" t="inlineStr"/>
+      <c r="O32" s="18" t="inlineStr"/>
+      <c r="P32" s="18" t="inlineStr"/>
+      <c r="Q32" s="18" t="inlineStr"/>
+      <c r="R32" s="18" t="inlineStr"/>
+      <c r="S32" s="15" t="inlineStr"/>
+    </row>
+    <row r="33" ht="150" customHeight="1">
+      <c r="A33" s="15" t="n">
         <v>18</v>
       </c>
-      <c r="B31" s="14" t="inlineStr">
-        <is>
-          <t>A-PT-01</t>
-        </is>
-      </c>
-      <c r="C31" s="14" t="inlineStr"/>
-      <c r="D31" s="14" t="inlineStr">
-        <is>
-          <t>Paint</t>
-        </is>
-      </c>
-      <c r="E31" s="14" t="inlineStr">
-        <is>
-          <t>Peinture texturée blanche</t>
-        </is>
-      </c>
-      <c r="F31" s="14" t="inlineStr">
-        <is>
-          <t>White textured paint</t>
-        </is>
-      </c>
-      <c r="G31" s="14" t="inlineStr"/>
-      <c r="H31" s="14" t="inlineStr">
-        <is>
-          <t>K5M-T1B1-ENT, K5M-T1B1-SDB, K5M-T1B1-CHA</t>
-        </is>
-      </c>
-      <c r="I31" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
-              <color rgb="00292B2B"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Entrée: ceiling+wall (excluded from BOQ). SDB: ceiling/cornice/wall (excluded). Chambre: cornice (excluded).</t>
-          </r>
-        </is>
-      </c>
-      <c r="J31" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K31" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L31" s="17" t="inlineStr"/>
-      <c r="M31" s="18" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="N31" s="17" t="inlineStr"/>
-      <c r="O31" s="17" t="inlineStr"/>
-      <c r="P31" s="17" t="inlineStr"/>
-      <c r="Q31" s="17" t="inlineStr"/>
-      <c r="R31" s="17" t="inlineStr"/>
-      <c r="S31" s="14" t="inlineStr">
-        <is>
-          <t>Painting is EXCLUDED from the awarded BOQ scope per client — tracked here for material reference only</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="150" customHeight="1">
-      <c r="A32" s="14" t="n">
-        <v>19</v>
-      </c>
-      <c r="B32" s="14" t="inlineStr">
-        <is>
-          <t>A-PT-02</t>
-        </is>
-      </c>
-      <c r="C32" s="14" t="inlineStr"/>
-      <c r="D32" s="14" t="inlineStr">
-        <is>
-          <t>Paint</t>
-        </is>
-      </c>
-      <c r="E32" s="14" t="inlineStr">
-        <is>
-          <t>Peinture texturée beige</t>
-        </is>
-      </c>
-      <c r="F32" s="14" t="inlineStr">
-        <is>
-          <t>Beige textured paint</t>
-        </is>
-      </c>
-      <c r="G32" s="14" t="inlineStr"/>
-      <c r="H32" s="14" t="inlineStr">
-        <is>
-          <t>K5M-T1B1-CHA</t>
-        </is>
-      </c>
-      <c r="I32" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
-              <color rgb="00292B2B"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Chambre: ceiling (excluded from BOQ).</t>
-          </r>
-        </is>
-      </c>
-      <c r="J32" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K32" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L32" s="17" t="inlineStr"/>
-      <c r="M32" s="18" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="N32" s="17" t="inlineStr"/>
-      <c r="O32" s="17" t="inlineStr"/>
-      <c r="P32" s="17" t="inlineStr"/>
-      <c r="Q32" s="17" t="inlineStr"/>
-      <c r="R32" s="17" t="inlineStr"/>
-      <c r="S32" s="14" t="inlineStr">
-        <is>
-          <t>Excluded from awarded BOQ scope</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="150" customHeight="1">
-      <c r="A33" s="14" t="n">
-        <v>20</v>
-      </c>
-      <c r="B33" s="14" t="inlineStr">
-        <is>
-          <t>A-WP-01</t>
-        </is>
-      </c>
-      <c r="C33" s="14" t="inlineStr"/>
-      <c r="D33" s="14" t="inlineStr">
-        <is>
-          <t>Wallpaper</t>
-        </is>
-      </c>
-      <c r="E33" s="14" t="inlineStr">
-        <is>
-          <t>Papier peint (Omexco)</t>
-        </is>
-      </c>
-      <c r="F33" s="14" t="inlineStr">
-        <is>
-          <t>Wallpaper (Omexco)</t>
-        </is>
-      </c>
-      <c r="G33" s="14" t="inlineStr"/>
-      <c r="H33" s="14" t="inlineStr">
-        <is>
-          <t>K5M-T1B1-CHA-C/6</t>
-        </is>
-      </c>
-      <c r="I33" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
-              <color rgb="00E4572E"/>
-              <sz val="11"/>
-              <u val="single"/>
-            </rPr>
-            <t>Chambre: wall — explicitly EXCLUDED from our BOQ offer per C/6 remark.</t>
-          </r>
-        </is>
-      </c>
-      <c r="J33" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K33" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L33" s="17" t="inlineStr"/>
-      <c r="M33" s="18" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="N33" s="17" t="inlineStr"/>
-      <c r="O33" s="17" t="inlineStr"/>
-      <c r="P33" s="17" t="inlineStr"/>
-      <c r="Q33" s="17" t="inlineStr"/>
-      <c r="R33" s="17" t="inlineStr"/>
-      <c r="S33" s="14" t="inlineStr">
-        <is>
-          <t>Supply/installation of this wallpaper is explicitly excluded in our BOQ offer (see C/6)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="150" customHeight="1">
-      <c r="A34" s="14" t="n">
-        <v>21</v>
-      </c>
-      <c r="B34" s="14" t="inlineStr">
-        <is>
-          <t>A-WP-02</t>
-        </is>
-      </c>
-      <c r="C34" s="14" t="inlineStr"/>
-      <c r="D34" s="14" t="inlineStr">
-        <is>
-          <t>Wallpaper</t>
-        </is>
-      </c>
-      <c r="E34" s="14" t="inlineStr">
-        <is>
-          <t>Papier peint (Biobject)</t>
-        </is>
-      </c>
-      <c r="F34" s="14" t="inlineStr">
-        <is>
-          <t>Wallpaper (Biobject)</t>
-        </is>
-      </c>
-      <c r="G34" s="14" t="inlineStr"/>
-      <c r="H34" s="14" t="inlineStr">
-        <is>
-          <t>K5M-T1B1-ENT</t>
-        </is>
-      </c>
-      <c r="I34" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
-              <color rgb="00292B2B"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Entrée: luggage-rack drawer interior panel.</t>
-          </r>
-        </is>
-      </c>
-      <c r="J34" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K34" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L34" s="17" t="inlineStr"/>
-      <c r="M34" s="18" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="N34" s="17" t="inlineStr"/>
-      <c r="O34" s="17" t="inlineStr"/>
-      <c r="P34" s="17" t="inlineStr"/>
-      <c r="Q34" s="17" t="inlineStr"/>
-      <c r="R34" s="17" t="inlineStr"/>
-      <c r="S34" s="14" t="inlineStr"/>
-    </row>
-    <row r="35" ht="150" customHeight="1">
-      <c r="A35" s="14" t="n">
-        <v>22</v>
-      </c>
-      <c r="B35" s="14" t="inlineStr">
-        <is>
-          <t>A-CA-01</t>
-        </is>
-      </c>
-      <c r="C35" s="14" t="inlineStr"/>
-      <c r="D35" s="14" t="inlineStr">
-        <is>
-          <t>Carpet</t>
-        </is>
-      </c>
-      <c r="E35" s="14" t="inlineStr">
-        <is>
-          <t>Moquette (Design Carpet - Ali Laraqui)</t>
-        </is>
-      </c>
-      <c r="F35" s="14" t="inlineStr">
-        <is>
-          <t>Carpet (Design Carpet - Ali Laraqui)</t>
-        </is>
-      </c>
-      <c r="G35" s="14" t="inlineStr">
-        <is>
-          <t>Tapis encastré / Inset carpet</t>
-        </is>
-      </c>
-      <c r="H35" s="14" t="inlineStr">
-        <is>
-          <t>K5M-T1B1-COULOIRS</t>
-        </is>
-      </c>
-      <c r="I35" s="15" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
-              <color rgb="00292B2B"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Corridors (Hall/bedroom corridors) — inset carpet. Also appears in Victoire's 21 Jul global soft-materials list alongside FF&amp;E fabric codes — kept in Fit-out only per our scope-separation rule.</t>
-          </r>
-        </is>
-      </c>
-      <c r="J35" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K35" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L35" s="17" t="inlineStr"/>
-      <c r="M35" s="18" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="N35" s="17" t="inlineStr"/>
-      <c r="O35" s="17" t="inlineStr"/>
-      <c r="P35" s="17" t="inlineStr"/>
-      <c r="Q35" s="17" t="inlineStr"/>
-      <c r="R35" s="17" t="inlineStr"/>
-      <c r="S35" s="14" t="inlineStr">
-        <is>
-          <t>Confirm carpet remains Wood Couture scope (open decision noted in earlier Fit-out audit)</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="150" customHeight="1">
-      <c r="A36" s="14" t="n">
-        <v>23</v>
-      </c>
-      <c r="B36" s="14" t="inlineStr">
+      <c r="B33" s="15" t="inlineStr">
         <is>
           <t>A-ST-03c / A-ST-06c</t>
         </is>
       </c>
-      <c r="C36" s="14" t="inlineStr"/>
-      <c r="D36" s="14" t="inlineStr">
+      <c r="C33" s="15" t="inlineStr"/>
+      <c r="D33" s="15" t="inlineStr">
         <is>
           <t>Stone</t>
         </is>
       </c>
-      <c r="E36" s="14" t="inlineStr">
+      <c r="E33" s="15" t="inlineStr">
         <is>
           <t>Travertin osso (vein cut / cross cut) — NOUVEAU 21 Jul</t>
         </is>
       </c>
-      <c r="F36" s="14" t="inlineStr">
+      <c r="F33" s="15" t="inlineStr">
         <is>
           <t>Travertine osso (vein cut / cross cut) — NEW 21 Jul</t>
         </is>
       </c>
-      <c r="G36" s="14" t="inlineStr">
+      <c r="G33" s="15" t="inlineStr">
         <is>
           <t>Adouci / Honed</t>
         </is>
       </c>
-      <c r="H36" s="14" t="inlineStr"/>
-      <c r="I36" s="15" t="inlineStr">
+      <c r="H33" s="15" t="inlineStr"/>
+      <c r="I33" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3042,65 +2703,65 @@
           </r>
         </is>
       </c>
-      <c r="J36" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K36" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L36" s="17" t="inlineStr"/>
-      <c r="M36" s="18" t="inlineStr">
+      <c r="J33" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K33" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L33" s="18" t="inlineStr"/>
+      <c r="M33" s="19" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N36" s="17" t="inlineStr"/>
-      <c r="O36" s="17" t="inlineStr"/>
-      <c r="P36" s="17" t="inlineStr"/>
-      <c r="Q36" s="17" t="inlineStr"/>
-      <c r="R36" s="17" t="inlineStr"/>
-      <c r="S36" s="14" t="inlineStr">
-        <is>
-          <t>New codes as of 21 Jul 2026 — location/application not yet confirmed, ask Adil</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="150" customHeight="1">
-      <c r="A37" s="14" t="n">
-        <v>24</v>
-      </c>
-      <c r="B37" s="14" t="inlineStr">
+      <c r="N33" s="18" t="inlineStr"/>
+      <c r="O33" s="18" t="inlineStr"/>
+      <c r="P33" s="18" t="inlineStr"/>
+      <c r="Q33" s="18" t="inlineStr"/>
+      <c r="R33" s="18" t="inlineStr"/>
+      <c r="S33" s="15" t="inlineStr">
+        <is>
+          <t>New codes as of 21 Jul 2026 — no confirmed location or in-scope task code yet, so no sample/high-res sourcing needed until scope is confirmed with Adil</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="150" customHeight="1">
+      <c r="A34" s="15" t="n">
+        <v>19</v>
+      </c>
+      <c r="B34" s="15" t="inlineStr">
         <is>
           <t>A-WD-03c</t>
         </is>
       </c>
-      <c r="C37" s="14" t="inlineStr"/>
-      <c r="D37" s="14" t="inlineStr">
+      <c r="C34" s="15" t="inlineStr"/>
+      <c r="D34" s="15" t="inlineStr">
         <is>
           <t>Wood</t>
         </is>
       </c>
-      <c r="E37" s="14" t="inlineStr">
+      <c r="E34" s="15" t="inlineStr">
         <is>
           <t>Tatawi peint en blanc — NOUVEAU 21 Jul</t>
         </is>
       </c>
-      <c r="F37" s="14" t="inlineStr">
+      <c r="F34" s="15" t="inlineStr">
         <is>
           <t>White-painted Tatawi wood — NEW 21 Jul</t>
         </is>
       </c>
-      <c r="G37" s="14" t="inlineStr">
+      <c r="G34" s="15" t="inlineStr">
         <is>
           <t>Mat</t>
         </is>
       </c>
-      <c r="H37" s="14" t="inlineStr"/>
-      <c r="I37" s="15" t="inlineStr">
+      <c r="H34" s="15" t="inlineStr"/>
+      <c r="I34" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3113,40 +2774,77 @@
           </r>
         </is>
       </c>
-      <c r="J37" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K37" s="16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L37" s="17" t="inlineStr"/>
-      <c r="M37" s="18" t="inlineStr">
+      <c r="J34" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K34" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L34" s="18" t="inlineStr"/>
+      <c r="M34" s="19" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N37" s="17" t="inlineStr"/>
-      <c r="O37" s="17" t="inlineStr"/>
-      <c r="P37" s="17" t="inlineStr"/>
-      <c r="Q37" s="17" t="inlineStr"/>
-      <c r="R37" s="17" t="inlineStr"/>
-      <c r="S37" s="14" t="inlineStr">
-        <is>
-          <t>New code as of 21 Jul 2026 — location/application not yet confirmed, ask Adil</t>
+      <c r="N34" s="18" t="inlineStr"/>
+      <c r="O34" s="18" t="inlineStr"/>
+      <c r="P34" s="18" t="inlineStr"/>
+      <c r="Q34" s="18" t="inlineStr"/>
+      <c r="R34" s="18" t="inlineStr"/>
+      <c r="S34" s="15" t="inlineStr">
+        <is>
+          <t>New code as of 21 Jul 2026 — no confirmed location or in-scope task code yet, so no sample/high-res sourcing needed until scope is confirmed with Adil</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>EXCLUDED — paint, wallpaper, and carpet are not in Wood Couture's Fit-out scope; kept out of this tracker entirely</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="20" t="inlineStr">
+        <is>
+          <t>A-PT-01, A-PT-02 (paint), A-WP-01, A-WP-02 (wallpaper), A-CA-01 (carpet)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A11:H11"/>
+  <mergeCells count="7">
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A37:S37"/>
+    <mergeCell ref="A36:S36"/>
+    <mergeCell ref="A14:S14"/>
+    <mergeCell ref="A1:S1"/>
+    <mergeCell ref="A13:H13"/>
     <mergeCell ref="A2:S2"/>
-    <mergeCell ref="A1:S1"/>
-    <mergeCell ref="A12:S12"/>
   </mergeCells>
+  <conditionalFormatting sqref="M16:M34">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"A"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"B"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"C"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
+      <formula>"S"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
+      <formula>"T"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="5">
+      <formula>"O"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
FFE + Fitout Material Packages: anonymize, Lato-only styling, banquette fabrics
Both workbooks:
- Remove all design-team/client real names from content; replace with generic
  references (supplier/brand names kept, e.g. Dedar, Naturtex)
- Font locked to Lato size 11 everywhere; borders switched to solid black
- Remove Description (FR) column

FFE:
- Fabrics tab: remove Finish columns entirely (only FA-02 had any finish info,
  folded into its Remarks); Hard Materials keeps Finish/Vernis (FR) hidden
- Add PP-03 row (shop-drawing fabric swatch, no material-list code yet)

Fitout:
- Drop A-ST-03c/A-ST-06c and A-WD-03c (no confirmed scope): 19 -> 17 rows
- Update A-GL-03a remarks re: client approval sample box
- Add new Fabrics tab: FA-04, FA-05, FA-08 (banquette upholstery + cushions),
  since the banquette is Fit-out scope

Formatting is now considered locked per user direction; further updates should
be data-entry only.
</commit_message>
<xml_diff>
--- a/material_package_fitout/260727_K5M_Material Package_Fitout.xlsx
+++ b/material_package_fitout/260727_K5M_Material Package_Fitout.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Fitout Materials" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Fabrics" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,27 +27,22 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Playfair Display"/>
+      <name val="Lato"/>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="16"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Lato"/>
       <i val="1"/>
-      <color rgb="00292B2B"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Playfair Display"/>
-      <b val="1"/>
       <color rgb="00292B2B"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Lato"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
+      <color rgb="00292B2B"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Lato"/>
@@ -55,21 +51,9 @@
     </font>
     <font>
       <name val="Lato"/>
-      <b val="1"/>
-      <color rgb="00292B2B"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Lato"/>
       <i val="1"/>
       <color rgb="00E4572E"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="Lato"/>
-      <i val="1"/>
-      <color rgb="00292B2B"/>
-      <sz val="8"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="10">
@@ -130,68 +114,73 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9D0CC"/>
+        <color rgb="00000000"/>
       </left>
       <right style="thin">
-        <color rgb="00D9D0CC"/>
+        <color rgb="00000000"/>
       </right>
       <top style="thin">
-        <color rgb="00D9D0CC"/>
+        <color rgb="00000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9D0CC"/>
+        <color rgb="00000000"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -731,21 +720,26 @@
     </pic>
     <clientData/>
   </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>32</row>
+      <row>15</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="571500" cy="547914"/>
+    <ext cx="571500" cy="419100"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId16"/>
+        <a:blip cstate="print" r:embed="rId1"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -760,17 +754,42 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>33</row>
+      <row>16</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="571500" cy="551542"/>
+    <ext cx="571500" cy="333000"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId17"/>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="571500" cy="382500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1073,7 +1092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S37"/>
+  <dimension ref="A1:R35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1081,23 +1100,22 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="6" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="6" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
     <col width="7" customWidth="1" min="14" max="14"/>
     <col width="7" customWidth="1" min="15" max="15"/>
     <col width="7" customWidth="1" min="16" max="16"/>
     <col width="7" customWidth="1" min="17" max="17"/>
-    <col width="7" customWidth="1" min="18" max="18"/>
-    <col width="34" customWidth="1" min="19" max="19"/>
+    <col width="34" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
-    <row r="1" ht="44" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>K5M — FIT-OUT MATERIAL PACKAGE</t>
@@ -1107,7 +1125,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of 27 July 2026 — V2: paint/wallpaper/carpet removed (out of Fit-out scope). Localization is sourced only from the DD-100-tagged material list dated 21.07.2026 (DD-100 governs over BOQ text where they conflict, per G&amp;B/Victoire 23 Jul) — never from the BOQ or Victoire's separate global soft-materials list. Underlined localizations are still unresolved / to be re-raised with Adil directly — not force-resolved here.</t>
+          <t>As of 27 July 2026 — V3: Lato-only styling, Description (FR) removed, 2 unassigned-scope rows dropped. Localization is sourced only from the DD-100-tagged material list dated 21.07.2026 (DD-100 governs over BOQ text where they conflict, per the design team, 23 Jul) — never from the BOQ or the design team's separate global soft-materials list. Underlined localizations are still unresolved / to be re-raised with the design team directly — not force-resolved here.</t>
         </is>
       </c>
     </row>
@@ -1130,7 +1148,7 @@
         </is>
       </c>
       <c r="C5" s="5">
-        <f>COUNTIF(M16:M200,"A")</f>
+        <f>COUNTIF(L16:L200,"A")</f>
         <v/>
       </c>
     </row>
@@ -1146,7 +1164,7 @@
         </is>
       </c>
       <c r="C6" s="5">
-        <f>COUNTIF(M16:M200,"B")</f>
+        <f>COUNTIF(L16:L200,"B")</f>
         <v/>
       </c>
     </row>
@@ -1162,7 +1180,7 @@
         </is>
       </c>
       <c r="C7" s="5">
-        <f>COUNTIF(M16:M200,"C")</f>
+        <f>COUNTIF(L16:L200,"C")</f>
         <v/>
       </c>
     </row>
@@ -1178,7 +1196,7 @@
         </is>
       </c>
       <c r="C8" s="5">
-        <f>COUNTIF(M16:M200,"S")</f>
+        <f>COUNTIF(L16:L200,"S")</f>
         <v/>
       </c>
     </row>
@@ -1194,7 +1212,7 @@
         </is>
       </c>
       <c r="C9" s="5">
-        <f>COUNTIF(M16:M200,"T")</f>
+        <f>COUNTIF(L16:L200,"T")</f>
         <v/>
       </c>
     </row>
@@ -1210,7 +1228,7 @@
         </is>
       </c>
       <c r="C10" s="5">
-        <f>COUNTIF(M16:M200,"O")</f>
+        <f>COUNTIF(L16:L200,"O")</f>
         <v/>
       </c>
     </row>
@@ -1221,7 +1239,7 @@
         </is>
       </c>
       <c r="C11" s="3">
-        <f>COUNTA(M16:M200)</f>
+        <f>COUNTA(L16:L200)</f>
         <v/>
       </c>
     </row>
@@ -1233,7 +1251,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>FM-xxx labels used in Localization/Remarks are internal cross-references created for this sheet only — not official RFI numbers from any project RFI log.</t>
         </is>
@@ -1241,138 +1259,128 @@
     </row>
     <row r="14"/>
     <row r="15" ht="68" customHeight="1">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>Material Code</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr">
+      <c r="C15" s="12" t="inlineStr">
         <is>
           <t>Thumbnail</t>
         </is>
       </c>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="D15" s="12" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="E15" s="13" t="inlineStr">
-        <is>
-          <t>Description (FR)</t>
-        </is>
-      </c>
-      <c r="F15" s="13" t="inlineStr">
+      <c r="E15" s="12" t="inlineStr">
         <is>
           <t>Description (EN)</t>
         </is>
       </c>
-      <c r="G15" s="13" t="inlineStr">
+      <c r="F15" s="12" t="inlineStr">
         <is>
           <t>Finish / Vernish</t>
         </is>
       </c>
-      <c r="H15" s="13" t="inlineStr">
+      <c r="G15" s="12" t="inlineStr">
         <is>
           <t>Applicable Task Code(s) (WDCO)</t>
         </is>
       </c>
-      <c r="I15" s="13" t="inlineStr">
-        <is>
-          <t>Localization per DD-100, dated 21.07.2026 (underlined = still under scrutiny with Adil)</t>
-        </is>
-      </c>
-      <c r="J15" s="13" t="inlineStr">
+      <c r="H15" s="12" t="inlineStr">
+        <is>
+          <t>Localization per DD-100, dated 21.07.2026 (underlined = still under scrutiny with the design team)</t>
+        </is>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
         <is>
           <t>Control Sample (Y/N)</t>
         </is>
       </c>
-      <c r="K15" s="13" t="inlineStr">
+      <c r="J15" s="12" t="inlineStr">
         <is>
           <t>High-Res Available (Y/N)</t>
         </is>
       </c>
+      <c r="K15" s="12" t="inlineStr">
+        <is>
+          <t>High-Res Link</t>
+        </is>
+      </c>
       <c r="L15" s="13" t="inlineStr">
         <is>
-          <t>High-Res Link</t>
-        </is>
-      </c>
-      <c r="M15" s="14" t="inlineStr">
-        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="N15" s="14" t="inlineStr">
+      <c r="M15" s="13" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="O15" s="14" t="inlineStr">
+      <c r="N15" s="13" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="P15" s="14" t="inlineStr">
+      <c r="O15" s="13" t="inlineStr">
         <is>
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="Q15" s="14" t="inlineStr">
+      <c r="P15" s="13" t="inlineStr">
         <is>
           <t>2026-08-17</t>
         </is>
       </c>
-      <c r="R15" s="14" t="inlineStr">
+      <c r="Q15" s="13" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="S15" s="13" t="inlineStr">
+      <c r="R15" s="12" t="inlineStr">
         <is>
           <t>Remarks / Open Issues</t>
         </is>
       </c>
     </row>
     <row r="16" ht="150" customHeight="1">
-      <c r="A16" s="15" t="n">
+      <c r="A16" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="B16" s="15" t="inlineStr">
+      <c r="B16" s="14" t="inlineStr">
         <is>
           <t>A-ST-01c</t>
         </is>
       </c>
-      <c r="C16" s="15" t="inlineStr"/>
-      <c r="D16" s="15" t="inlineStr">
+      <c r="C16" s="14" t="inlineStr"/>
+      <c r="D16" s="14" t="inlineStr">
         <is>
           <t>Stone</t>
         </is>
       </c>
-      <c r="E16" s="15" t="inlineStr">
-        <is>
-          <t>Beige clair</t>
-        </is>
-      </c>
-      <c r="F16" s="15" t="inlineStr">
+      <c r="E16" s="14" t="inlineStr">
         <is>
           <t>Light beige stone</t>
         </is>
       </c>
-      <c r="G16" s="15" t="inlineStr">
+      <c r="F16" s="14" t="inlineStr">
         <is>
           <t>Adouci / Honed</t>
         </is>
       </c>
+      <c r="G16" s="14" t="inlineStr">
+        <is>
+          <t>K5M-T1B1-ENT-A/? (threshold), K5M-T1B1-SDB-B/6, K5M-T1B1-SDB-B/12, K5M-T1B1-CHA-C/2, K5M-T1B1-CHA-C/3</t>
+        </is>
+      </c>
       <c r="H16" s="15" t="inlineStr">
-        <is>
-          <t>K5M-T1B1-ENT-A/? (threshold), K5M-T1B1-SDB-B/6, K5M-T1B1-SDB-B/12, K5M-T1B1-CHA-C/2, K5M-T1B1-CHA-C/3</t>
-        </is>
-      </c>
-      <c r="I16" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1402,69 +1410,64 @@
           </r>
         </is>
       </c>
-      <c r="J16" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K16" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L16" s="18" t="inlineStr"/>
-      <c r="M16" s="19" t="inlineStr">
+      <c r="I16" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J16" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K16" s="17" t="inlineStr"/>
+      <c r="L16" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N16" s="18" t="inlineStr"/>
-      <c r="O16" s="18" t="inlineStr"/>
-      <c r="P16" s="18" t="inlineStr"/>
-      <c r="Q16" s="18" t="inlineStr"/>
-      <c r="R16" s="18" t="inlineStr"/>
-      <c r="S16" s="15" t="inlineStr">
-        <is>
-          <t>See FM-007, FM-009, FM-010 — all still open, to re-raise with Adil</t>
+      <c r="M16" s="17" t="inlineStr"/>
+      <c r="N16" s="17" t="inlineStr"/>
+      <c r="O16" s="17" t="inlineStr"/>
+      <c r="P16" s="17" t="inlineStr"/>
+      <c r="Q16" s="17" t="inlineStr"/>
+      <c r="R16" s="14" t="inlineStr">
+        <is>
+          <t>See FM-007, FM-009, FM-010 — all still open, to re-raise with the design team</t>
         </is>
       </c>
     </row>
     <row r="17" ht="150" customHeight="1">
-      <c r="A17" s="15" t="n">
+      <c r="A17" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="B17" s="15" t="inlineStr">
+      <c r="B17" s="14" t="inlineStr">
         <is>
           <t>A-ST-01d</t>
         </is>
       </c>
-      <c r="C17" s="15" t="inlineStr"/>
-      <c r="D17" s="15" t="inlineStr">
+      <c r="C17" s="14" t="inlineStr"/>
+      <c r="D17" s="14" t="inlineStr">
         <is>
           <t>Stone</t>
         </is>
       </c>
-      <c r="E17" s="15" t="inlineStr">
-        <is>
-          <t>Beige clair</t>
-        </is>
-      </c>
-      <c r="F17" s="15" t="inlineStr">
+      <c r="E17" s="14" t="inlineStr">
         <is>
           <t>Light beige stone</t>
         </is>
       </c>
-      <c r="G17" s="15" t="inlineStr">
+      <c r="F17" s="14" t="inlineStr">
         <is>
           <t>Anti-dérapant / Anti-slip</t>
         </is>
       </c>
+      <c r="G17" s="14" t="inlineStr">
+        <is>
+          <t>K5M-T1B1-SDB-B/2, K5M-T1B1-SDB-B/5</t>
+        </is>
+      </c>
       <c r="H17" s="15" t="inlineStr">
-        <is>
-          <t>K5M-T1B1-SDB-B/2, K5M-T1B1-SDB-B/5</t>
-        </is>
-      </c>
-      <c r="I17" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1485,69 +1488,64 @@
           </r>
         </is>
       </c>
-      <c r="J17" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K17" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L17" s="18" t="inlineStr"/>
-      <c r="M17" s="19" t="inlineStr">
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K17" s="17" t="inlineStr"/>
+      <c r="L17" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N17" s="18" t="inlineStr"/>
-      <c r="O17" s="18" t="inlineStr"/>
-      <c r="P17" s="18" t="inlineStr"/>
-      <c r="Q17" s="18" t="inlineStr"/>
-      <c r="R17" s="18" t="inlineStr"/>
-      <c r="S17" s="15" t="inlineStr">
+      <c r="M17" s="17" t="inlineStr"/>
+      <c r="N17" s="17" t="inlineStr"/>
+      <c r="O17" s="17" t="inlineStr"/>
+      <c r="P17" s="17" t="inlineStr"/>
+      <c r="Q17" s="17" t="inlineStr"/>
+      <c r="R17" s="14" t="inlineStr">
         <is>
           <t>See FM-005, FM-012</t>
         </is>
       </c>
     </row>
     <row r="18" ht="150" customHeight="1">
-      <c r="A18" s="15" t="n">
+      <c r="A18" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="B18" s="15" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>A-ST-01e</t>
         </is>
       </c>
-      <c r="C18" s="15" t="inlineStr"/>
-      <c r="D18" s="15" t="inlineStr">
+      <c r="C18" s="14" t="inlineStr"/>
+      <c r="D18" s="14" t="inlineStr">
         <is>
           <t>Stone</t>
         </is>
       </c>
-      <c r="E18" s="15" t="inlineStr">
-        <is>
-          <t>Beige clair</t>
-        </is>
-      </c>
-      <c r="F18" s="15" t="inlineStr">
+      <c r="E18" s="14" t="inlineStr">
         <is>
           <t>Light beige stone</t>
         </is>
       </c>
-      <c r="G18" s="15" t="inlineStr">
+      <c r="F18" s="14" t="inlineStr">
         <is>
           <t>Martelé / Hammered</t>
         </is>
       </c>
+      <c r="G18" s="14" t="inlineStr">
+        <is>
+          <t>K5M-T1B1-ENT-A/1, K5M-T1B1-SDB-B/1</t>
+        </is>
+      </c>
       <c r="H18" s="15" t="inlineStr">
-        <is>
-          <t>K5M-T1B1-ENT-A/1, K5M-T1B1-SDB-B/1</t>
-        </is>
-      </c>
-      <c r="I18" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1559,65 +1557,60 @@
           </r>
         </is>
       </c>
-      <c r="J18" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K18" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L18" s="18" t="inlineStr"/>
-      <c r="M18" s="19" t="inlineStr">
+      <c r="I18" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J18" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K18" s="17" t="inlineStr"/>
+      <c r="L18" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N18" s="18" t="inlineStr"/>
-      <c r="O18" s="18" t="inlineStr"/>
-      <c r="P18" s="18" t="inlineStr"/>
-      <c r="Q18" s="18" t="inlineStr"/>
-      <c r="R18" s="18" t="inlineStr"/>
-      <c r="S18" s="15" t="inlineStr"/>
+      <c r="M18" s="17" t="inlineStr"/>
+      <c r="N18" s="17" t="inlineStr"/>
+      <c r="O18" s="17" t="inlineStr"/>
+      <c r="P18" s="17" t="inlineStr"/>
+      <c r="Q18" s="17" t="inlineStr"/>
+      <c r="R18" s="14" t="inlineStr"/>
     </row>
     <row r="19" ht="150" customHeight="1">
-      <c r="A19" s="15" t="n">
+      <c r="A19" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="B19" s="15" t="inlineStr">
+      <c r="B19" s="14" t="inlineStr">
         <is>
           <t>A-ST-02c</t>
         </is>
       </c>
-      <c r="C19" s="15" t="inlineStr"/>
-      <c r="D19" s="15" t="inlineStr">
+      <c r="C19" s="14" t="inlineStr"/>
+      <c r="D19" s="14" t="inlineStr">
         <is>
           <t>Stone</t>
         </is>
       </c>
-      <c r="E19" s="15" t="inlineStr">
-        <is>
-          <t>Beige foncé</t>
-        </is>
-      </c>
-      <c r="F19" s="15" t="inlineStr">
+      <c r="E19" s="14" t="inlineStr">
         <is>
           <t>Dark beige stone</t>
         </is>
       </c>
-      <c r="G19" s="15" t="inlineStr">
+      <c r="F19" s="14" t="inlineStr">
         <is>
           <t>Adouci / Honed</t>
         </is>
       </c>
+      <c r="G19" s="14" t="inlineStr">
+        <is>
+          <t>K5M-T1B1-ENT-A/1, K5M-T1B1-SDB-B/1, K5M-T1B1-SDB-B/3, K5M-T1B1-CHA-C/2</t>
+        </is>
+      </c>
       <c r="H19" s="15" t="inlineStr">
-        <is>
-          <t>K5M-T1B1-ENT-A/1, K5M-T1B1-SDB-B/1, K5M-T1B1-SDB-B/3, K5M-T1B1-CHA-C/2</t>
-        </is>
-      </c>
-      <c r="I19" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1638,69 +1631,64 @@
           </r>
         </is>
       </c>
-      <c r="J19" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K19" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L19" s="18" t="inlineStr"/>
-      <c r="M19" s="19" t="inlineStr">
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K19" s="17" t="inlineStr"/>
+      <c r="L19" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N19" s="18" t="inlineStr"/>
-      <c r="O19" s="18" t="inlineStr"/>
-      <c r="P19" s="18" t="inlineStr"/>
-      <c r="Q19" s="18" t="inlineStr"/>
-      <c r="R19" s="18" t="inlineStr"/>
-      <c r="S19" s="15" t="inlineStr">
+      <c r="M19" s="17" t="inlineStr"/>
+      <c r="N19" s="17" t="inlineStr"/>
+      <c r="O19" s="17" t="inlineStr"/>
+      <c r="P19" s="17" t="inlineStr"/>
+      <c r="Q19" s="17" t="inlineStr"/>
+      <c r="R19" s="14" t="inlineStr">
         <is>
           <t>See FM-009</t>
         </is>
       </c>
     </row>
     <row r="20" ht="150" customHeight="1">
-      <c r="A20" s="15" t="n">
+      <c r="A20" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="B20" s="15" t="inlineStr">
+      <c r="B20" s="14" t="inlineStr">
         <is>
           <t>A-ST-07a</t>
         </is>
       </c>
-      <c r="C20" s="15" t="inlineStr"/>
-      <c r="D20" s="15" t="inlineStr">
+      <c r="C20" s="14" t="inlineStr"/>
+      <c r="D20" s="14" t="inlineStr">
         <is>
           <t>Stone</t>
         </is>
       </c>
-      <c r="E20" s="15" t="inlineStr">
-        <is>
-          <t>Onyx miel — REMPLACÉ PAR Taj Mahal</t>
-        </is>
-      </c>
-      <c r="F20" s="15" t="inlineStr">
+      <c r="E20" s="14" t="inlineStr">
         <is>
           <t>Onyx Honey — REPLACED BY Taj Mahal</t>
         </is>
       </c>
-      <c r="G20" s="15" t="inlineStr">
+      <c r="F20" s="14" t="inlineStr">
         <is>
           <t>Poli / Polished</t>
         </is>
       </c>
+      <c r="G20" s="14" t="inlineStr">
+        <is>
+          <t>K5M-T1B1-ENT-A (arch/luggage rack), K5M-T1B1-SDB-B/7, K5M-T1B1-SDB-B/8, K5M-T1B1-SDB-B/9, K5M-T1B1-SDB-B/10, K5M-T1B1-SDB-B/11, K5M-T1B1-SDB-B/12, K5M-T1B1-CHA-C/4</t>
+        </is>
+      </c>
       <c r="H20" s="15" t="inlineStr">
-        <is>
-          <t>K5M-T1B1-ENT-A (arch/luggage rack), K5M-T1B1-SDB-B/7, K5M-T1B1-SDB-B/8, K5M-T1B1-SDB-B/9, K5M-T1B1-SDB-B/10, K5M-T1B1-SDB-B/11, K5M-T1B1-SDB-B/12, K5M-T1B1-CHA-C/4</t>
-        </is>
-      </c>
-      <c r="I20" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1729,69 +1717,64 @@
           </r>
         </is>
       </c>
-      <c r="J20" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K20" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L20" s="18" t="inlineStr"/>
-      <c r="M20" s="19" t="inlineStr">
+      <c r="I20" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J20" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K20" s="17" t="inlineStr"/>
+      <c r="L20" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N20" s="18" t="inlineStr"/>
-      <c r="O20" s="18" t="inlineStr"/>
-      <c r="P20" s="18" t="inlineStr"/>
-      <c r="Q20" s="18" t="inlineStr"/>
-      <c r="R20" s="18" t="inlineStr"/>
-      <c r="S20" s="15" t="inlineStr">
+      <c r="M20" s="17" t="inlineStr"/>
+      <c r="N20" s="17" t="inlineStr"/>
+      <c r="O20" s="17" t="inlineStr"/>
+      <c r="P20" s="17" t="inlineStr"/>
+      <c r="Q20" s="17" t="inlineStr"/>
+      <c r="R20" s="14" t="inlineStr">
         <is>
           <t>SUBSTITUTED as of 21 Jul 2026 update. See FM-002, FM-007 — confirm Taj Mahal applies everywhere, honey onyx no longer valid anywhere</t>
         </is>
       </c>
     </row>
     <row r="21" ht="150" customHeight="1">
-      <c r="A21" s="15" t="n">
+      <c r="A21" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="B21" s="15" t="inlineStr">
+      <c r="B21" s="14" t="inlineStr">
         <is>
           <t>A-WD-01b</t>
         </is>
       </c>
-      <c r="C21" s="15" t="inlineStr"/>
-      <c r="D21" s="15" t="inlineStr">
+      <c r="C21" s="14" t="inlineStr"/>
+      <c r="D21" s="14" t="inlineStr">
         <is>
           <t>Wood</t>
         </is>
       </c>
-      <c r="E21" s="15" t="inlineStr">
-        <is>
-          <t>Noyer — REMPLACÉ PAR chêne teinté moyen</t>
-        </is>
-      </c>
-      <c r="F21" s="15" t="inlineStr">
+      <c r="E21" s="14" t="inlineStr">
         <is>
           <t>Walnut — REPLACED BY medium-tinted oak</t>
         </is>
       </c>
-      <c r="G21" s="15" t="inlineStr">
+      <c r="F21" s="14" t="inlineStr">
         <is>
           <t>Satin</t>
         </is>
       </c>
+      <c r="G21" s="14" t="inlineStr">
+        <is>
+          <t>K5M-T1B1-ENT-A/7, K5M-T1B1-CHA-C/7</t>
+        </is>
+      </c>
       <c r="H21" s="15" t="inlineStr">
-        <is>
-          <t>K5M-T1B1-ENT-A/7, K5M-T1B1-CHA-C/7</t>
-        </is>
-      </c>
-      <c r="I21" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1813,65 +1796,60 @@
           </r>
         </is>
       </c>
-      <c r="J21" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K21" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L21" s="18" t="inlineStr"/>
-      <c r="M21" s="19" t="inlineStr">
+      <c r="I21" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J21" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K21" s="17" t="inlineStr"/>
+      <c r="L21" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N21" s="18" t="inlineStr"/>
-      <c r="O21" s="18" t="inlineStr"/>
-      <c r="P21" s="18" t="inlineStr"/>
-      <c r="Q21" s="18" t="inlineStr"/>
-      <c r="R21" s="18" t="inlineStr"/>
-      <c r="S21" s="15" t="inlineStr">
+      <c r="M21" s="17" t="inlineStr"/>
+      <c r="N21" s="17" t="inlineStr"/>
+      <c r="O21" s="17" t="inlineStr"/>
+      <c r="P21" s="17" t="inlineStr"/>
+      <c r="Q21" s="17" t="inlineStr"/>
+      <c r="R21" s="14" t="inlineStr">
         <is>
           <t>SUBSTITUTED as of 21 Jul 2026. See FM-001 — confirm all four applications follow this code/finish</t>
         </is>
       </c>
     </row>
     <row r="22" ht="150" customHeight="1">
-      <c r="A22" s="15" t="n">
+      <c r="A22" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="B22" s="15" t="inlineStr">
+      <c r="B22" s="14" t="inlineStr">
         <is>
           <t>A-WD-01d</t>
         </is>
       </c>
-      <c r="C22" s="15" t="inlineStr"/>
-      <c r="D22" s="15" t="inlineStr">
+      <c r="C22" s="14" t="inlineStr"/>
+      <c r="D22" s="14" t="inlineStr">
         <is>
           <t>Wood</t>
         </is>
       </c>
-      <c r="E22" s="15" t="inlineStr">
-        <is>
-          <t>(absent de la liste officielle des matériaux)</t>
-        </is>
-      </c>
-      <c r="F22" s="15" t="inlineStr">
+      <c r="E22" s="14" t="inlineStr">
         <is>
           <t>(does not appear in the official material list at all)</t>
         </is>
       </c>
-      <c r="G22" s="15" t="inlineStr"/>
+      <c r="F22" s="14" t="inlineStr"/>
+      <c r="G22" s="14" t="inlineStr">
+        <is>
+          <t>K5M-T1B1-ENT-A/2, K5M-T1B1-ENT-A/4</t>
+        </is>
+      </c>
       <c r="H22" s="15" t="inlineStr">
-        <is>
-          <t>K5M-T1B1-ENT-A/2, K5M-T1B1-ENT-A/4</t>
-        </is>
-      </c>
-      <c r="I22" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1884,69 +1862,64 @@
           </r>
         </is>
       </c>
-      <c r="J22" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K22" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L22" s="18" t="inlineStr"/>
-      <c r="M22" s="19" t="inlineStr">
+      <c r="I22" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J22" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K22" s="17" t="inlineStr"/>
+      <c r="L22" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N22" s="18" t="inlineStr"/>
-      <c r="O22" s="18" t="inlineStr"/>
-      <c r="P22" s="18" t="inlineStr"/>
-      <c r="Q22" s="18" t="inlineStr"/>
-      <c r="R22" s="18" t="inlineStr"/>
-      <c r="S22" s="15" t="inlineStr">
+      <c r="M22" s="17" t="inlineStr"/>
+      <c r="N22" s="17" t="inlineStr"/>
+      <c r="O22" s="17" t="inlineStr"/>
+      <c r="P22" s="17" t="inlineStr"/>
+      <c r="Q22" s="17" t="inlineStr"/>
+      <c r="R22" s="14" t="inlineStr">
         <is>
           <t>See FM-001. RFI already flags: no material reference image provided for this code</t>
         </is>
       </c>
     </row>
     <row r="23" ht="150" customHeight="1">
-      <c r="A23" s="15" t="n">
+      <c r="A23" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="B23" s="15" t="inlineStr">
+      <c r="B23" s="14" t="inlineStr">
         <is>
           <t>A-WD-02c</t>
         </is>
       </c>
-      <c r="C23" s="15" t="inlineStr"/>
-      <c r="D23" s="15" t="inlineStr">
+      <c r="C23" s="14" t="inlineStr"/>
+      <c r="D23" s="14" t="inlineStr">
         <is>
           <t>Wood</t>
         </is>
       </c>
-      <c r="E23" s="15" t="inlineStr">
-        <is>
-          <t>Chêne cérusé blanc</t>
-        </is>
-      </c>
-      <c r="F23" s="15" t="inlineStr">
+      <c r="E23" s="14" t="inlineStr">
         <is>
           <t>White cerused oak</t>
         </is>
       </c>
-      <c r="G23" s="15" t="inlineStr">
+      <c r="F23" s="14" t="inlineStr">
         <is>
           <t>Mat / Matte</t>
         </is>
       </c>
+      <c r="G23" s="14" t="inlineStr">
+        <is>
+          <t>K5M-T1B1-ENT-A/8, K5M-T1B1-SDB-B/14, K5M-T1B1-CHA-C/6</t>
+        </is>
+      </c>
       <c r="H23" s="15" t="inlineStr">
-        <is>
-          <t>K5M-T1B1-ENT-A/8, K5M-T1B1-SDB-B/14, K5M-T1B1-CHA-C/6</t>
-        </is>
-      </c>
-      <c r="I23" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1967,69 +1940,64 @@
           </r>
         </is>
       </c>
-      <c r="J23" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K23" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L23" s="18" t="inlineStr"/>
-      <c r="M23" s="19" t="inlineStr">
+      <c r="I23" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J23" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K23" s="17" t="inlineStr"/>
+      <c r="L23" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N23" s="18" t="inlineStr"/>
-      <c r="O23" s="18" t="inlineStr"/>
-      <c r="P23" s="18" t="inlineStr"/>
-      <c r="Q23" s="18" t="inlineStr"/>
-      <c r="R23" s="18" t="inlineStr"/>
-      <c r="S23" s="15" t="inlineStr">
+      <c r="M23" s="17" t="inlineStr"/>
+      <c r="N23" s="17" t="inlineStr"/>
+      <c r="O23" s="17" t="inlineStr"/>
+      <c r="P23" s="17" t="inlineStr"/>
+      <c r="Q23" s="17" t="inlineStr"/>
+      <c r="R23" s="14" t="inlineStr">
         <is>
           <t>See FM-011</t>
         </is>
       </c>
     </row>
     <row r="24" ht="150" customHeight="1">
-      <c r="A24" s="15" t="n">
+      <c r="A24" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="B24" s="15" t="inlineStr">
+      <c r="B24" s="14" t="inlineStr">
         <is>
           <t>A-WD-04b</t>
         </is>
       </c>
-      <c r="C24" s="15" t="inlineStr"/>
-      <c r="D24" s="15" t="inlineStr">
+      <c r="C24" s="14" t="inlineStr"/>
+      <c r="D24" s="14" t="inlineStr">
         <is>
           <t>Wood</t>
         </is>
       </c>
-      <c r="E24" s="15" t="inlineStr">
-        <is>
-          <t>Parquet chêne teinté moyen (Hakwood Idéal)</t>
-        </is>
-      </c>
-      <c r="F24" s="15" t="inlineStr">
+      <c r="E24" s="14" t="inlineStr">
         <is>
           <t>Medium-tinted oak parquet (Hakwood Idéal)</t>
         </is>
       </c>
-      <c r="G24" s="15" t="inlineStr">
+      <c r="F24" s="14" t="inlineStr">
         <is>
           <t>Satin</t>
         </is>
       </c>
+      <c r="G24" s="14" t="inlineStr">
+        <is>
+          <t>K5M-T1B1-CHA-C/1</t>
+        </is>
+      </c>
       <c r="H24" s="15" t="inlineStr">
-        <is>
-          <t>K5M-T1B1-CHA-C/1</t>
-        </is>
-      </c>
-      <c r="I24" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2051,69 +2019,64 @@
           </r>
         </is>
       </c>
-      <c r="J24" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K24" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L24" s="18" t="inlineStr"/>
-      <c r="M24" s="19" t="inlineStr">
+      <c r="I24" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J24" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K24" s="17" t="inlineStr"/>
+      <c r="L24" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N24" s="18" t="inlineStr"/>
-      <c r="O24" s="18" t="inlineStr"/>
-      <c r="P24" s="18" t="inlineStr"/>
-      <c r="Q24" s="18" t="inlineStr"/>
-      <c r="R24" s="18" t="inlineStr"/>
-      <c r="S24" s="15" t="inlineStr">
+      <c r="M24" s="17" t="inlineStr"/>
+      <c r="N24" s="17" t="inlineStr"/>
+      <c r="O24" s="17" t="inlineStr"/>
+      <c r="P24" s="17" t="inlineStr"/>
+      <c r="Q24" s="17" t="inlineStr"/>
+      <c r="R24" s="14" t="inlineStr">
         <is>
           <t>SUBSTITUTED from dark-tinted to medium-tinted oak, 21 Jul 2026, real product ref (Hakwood, Idéal). See FM-008</t>
         </is>
       </c>
     </row>
     <row r="25" ht="150" customHeight="1">
-      <c r="A25" s="15" t="n">
+      <c r="A25" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="B25" s="15" t="inlineStr">
+      <c r="B25" s="14" t="inlineStr">
         <is>
           <t>A-ME-01a</t>
         </is>
       </c>
-      <c r="C25" s="15" t="inlineStr"/>
-      <c r="D25" s="15" t="inlineStr">
+      <c r="C25" s="14" t="inlineStr"/>
+      <c r="D25" s="14" t="inlineStr">
         <is>
           <t>Metal</t>
         </is>
       </c>
-      <c r="E25" s="15" t="inlineStr">
-        <is>
-          <t>Acier inoxydable poli</t>
-        </is>
-      </c>
-      <c r="F25" s="15" t="inlineStr">
+      <c r="E25" s="14" t="inlineStr">
         <is>
           <t>Polished stainless steel</t>
         </is>
       </c>
-      <c r="G25" s="15" t="inlineStr">
+      <c r="F25" s="14" t="inlineStr">
         <is>
           <t>Finition poli miroir</t>
         </is>
       </c>
+      <c r="G25" s="14" t="inlineStr">
+        <is>
+          <t>K5M-T1B1-SDB-B/8, K5M-T1B1-SDB-B/14</t>
+        </is>
+      </c>
       <c r="H25" s="15" t="inlineStr">
-        <is>
-          <t>K5M-T1B1-SDB-B/8, K5M-T1B1-SDB-B/14</t>
-        </is>
-      </c>
-      <c r="I25" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2135,69 +2098,64 @@
           </r>
         </is>
       </c>
-      <c r="J25" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K25" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L25" s="18" t="inlineStr"/>
-      <c r="M25" s="19" t="inlineStr">
+      <c r="I25" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J25" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K25" s="17" t="inlineStr"/>
+      <c r="L25" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N25" s="18" t="inlineStr"/>
-      <c r="O25" s="18" t="inlineStr"/>
-      <c r="P25" s="18" t="inlineStr"/>
-      <c r="Q25" s="18" t="inlineStr"/>
-      <c r="R25" s="18" t="inlineStr"/>
-      <c r="S25" s="15" t="inlineStr">
+      <c r="M25" s="17" t="inlineStr"/>
+      <c r="N25" s="17" t="inlineStr"/>
+      <c r="O25" s="17" t="inlineStr"/>
+      <c r="P25" s="17" t="inlineStr"/>
+      <c r="Q25" s="17" t="inlineStr"/>
+      <c r="R25" s="14" t="inlineStr">
         <is>
           <t>See FM-006. Location changed between material list versions — confirm current assignment</t>
         </is>
       </c>
     </row>
     <row r="26" ht="150" customHeight="1">
-      <c r="A26" s="15" t="n">
+      <c r="A26" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="B26" s="15" t="inlineStr">
+      <c r="B26" s="14" t="inlineStr">
         <is>
           <t>A-ME-01h</t>
         </is>
       </c>
-      <c r="C26" s="15" t="inlineStr"/>
-      <c r="D26" s="15" t="inlineStr">
+      <c r="C26" s="14" t="inlineStr"/>
+      <c r="D26" s="14" t="inlineStr">
         <is>
           <t>Metal</t>
         </is>
       </c>
-      <c r="E26" s="15" t="inlineStr">
-        <is>
-          <t>Acier inoxydable brossé (NOUVEAU 21 Jul)</t>
-        </is>
-      </c>
-      <c r="F26" s="15" t="inlineStr">
+      <c r="E26" s="14" t="inlineStr">
         <is>
           <t>Brushed stainless steel (NEW 21 Jul)</t>
         </is>
       </c>
-      <c r="G26" s="15" t="inlineStr">
+      <c r="F26" s="14" t="inlineStr">
         <is>
           <t>Finition brossé</t>
         </is>
       </c>
+      <c r="G26" s="14" t="inlineStr">
+        <is>
+          <t>K5M-T1B1-ENT</t>
+        </is>
+      </c>
       <c r="H26" s="15" t="inlineStr">
-        <is>
-          <t>K5M-T1B1-ENT</t>
-        </is>
-      </c>
-      <c r="I26" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2210,69 +2168,64 @@
           </r>
         </is>
       </c>
-      <c r="J26" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K26" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L26" s="18" t="inlineStr"/>
-      <c r="M26" s="19" t="inlineStr">
+      <c r="I26" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J26" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K26" s="17" t="inlineStr"/>
+      <c r="L26" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N26" s="18" t="inlineStr"/>
-      <c r="O26" s="18" t="inlineStr"/>
-      <c r="P26" s="18" t="inlineStr"/>
-      <c r="Q26" s="18" t="inlineStr"/>
-      <c r="R26" s="18" t="inlineStr"/>
-      <c r="S26" s="15" t="inlineStr">
-        <is>
-          <t>New code as of 21 Jul 2026 update — confirm with Adil this is the correct replacement for the rail location</t>
+      <c r="M26" s="17" t="inlineStr"/>
+      <c r="N26" s="17" t="inlineStr"/>
+      <c r="O26" s="17" t="inlineStr"/>
+      <c r="P26" s="17" t="inlineStr"/>
+      <c r="Q26" s="17" t="inlineStr"/>
+      <c r="R26" s="14" t="inlineStr">
+        <is>
+          <t>New code as of 21 Jul 2026 update — confirm with the design team this is the correct replacement for the rail location</t>
         </is>
       </c>
     </row>
     <row r="27" ht="150" customHeight="1">
-      <c r="A27" s="15" t="n">
+      <c r="A27" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="B27" s="15" t="inlineStr">
+      <c r="B27" s="14" t="inlineStr">
         <is>
           <t>A-ME-02h</t>
         </is>
       </c>
-      <c r="C27" s="15" t="inlineStr"/>
-      <c r="D27" s="15" t="inlineStr">
+      <c r="C27" s="14" t="inlineStr"/>
+      <c r="D27" s="14" t="inlineStr">
         <is>
           <t>Metal</t>
         </is>
       </c>
-      <c r="E27" s="15" t="inlineStr">
-        <is>
-          <t>Laiton patiné foncé</t>
-        </is>
-      </c>
-      <c r="F27" s="15" t="inlineStr">
+      <c r="E27" s="14" t="inlineStr">
         <is>
           <t>Dark patinated brass</t>
         </is>
       </c>
-      <c r="G27" s="15" t="inlineStr">
+      <c r="F27" s="14" t="inlineStr">
         <is>
           <t>Vernis mat / Matte varnish</t>
         </is>
       </c>
+      <c r="G27" s="14" t="inlineStr">
+        <is>
+          <t>K5M-T1B1-ENT-A/7, K5M-T1B1-ENT-A/8, K5M-T1B1-SDB-B/13, K5M-T1B1-CHA-C/7</t>
+        </is>
+      </c>
       <c r="H27" s="15" t="inlineStr">
-        <is>
-          <t>K5M-T1B1-ENT-A/7, K5M-T1B1-ENT-A/8, K5M-T1B1-SDB-B/13, K5M-T1B1-CHA-C/7</t>
-        </is>
-      </c>
-      <c r="I27" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2284,65 +2237,60 @@
           </r>
         </is>
       </c>
-      <c r="J27" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K27" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L27" s="18" t="inlineStr"/>
-      <c r="M27" s="19" t="inlineStr">
+      <c r="I27" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J27" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K27" s="17" t="inlineStr"/>
+      <c r="L27" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N27" s="18" t="inlineStr"/>
-      <c r="O27" s="18" t="inlineStr"/>
-      <c r="P27" s="18" t="inlineStr"/>
-      <c r="Q27" s="18" t="inlineStr"/>
-      <c r="R27" s="18" t="inlineStr"/>
-      <c r="S27" s="15" t="inlineStr"/>
+      <c r="M27" s="17" t="inlineStr"/>
+      <c r="N27" s="17" t="inlineStr"/>
+      <c r="O27" s="17" t="inlineStr"/>
+      <c r="P27" s="17" t="inlineStr"/>
+      <c r="Q27" s="17" t="inlineStr"/>
+      <c r="R27" s="14" t="inlineStr"/>
     </row>
     <row r="28" ht="150" customHeight="1">
-      <c r="A28" s="15" t="n">
+      <c r="A28" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="B28" s="15" t="inlineStr">
+      <c r="B28" s="14" t="inlineStr">
         <is>
           <t>A-ME-02i</t>
         </is>
       </c>
-      <c r="C28" s="15" t="inlineStr"/>
-      <c r="D28" s="15" t="inlineStr">
+      <c r="C28" s="14" t="inlineStr"/>
+      <c r="D28" s="14" t="inlineStr">
         <is>
           <t>Metal</t>
         </is>
       </c>
-      <c r="E28" s="15" t="inlineStr">
-        <is>
-          <t>Laiton patiné foncé martelé</t>
-        </is>
-      </c>
-      <c r="F28" s="15" t="inlineStr">
+      <c r="E28" s="14" t="inlineStr">
         <is>
           <t>Dark patinated hammered brass</t>
         </is>
       </c>
-      <c r="G28" s="15" t="inlineStr">
+      <c r="F28" s="14" t="inlineStr">
         <is>
           <t>Martelé, vernis mat</t>
         </is>
       </c>
+      <c r="G28" s="14" t="inlineStr">
+        <is>
+          <t>K5M-T1B1-ENT-A/8, K5M-T1B1-SDB-B/14</t>
+        </is>
+      </c>
       <c r="H28" s="15" t="inlineStr">
-        <is>
-          <t>K5M-T1B1-ENT-A/8, K5M-T1B1-SDB-B/14</t>
-        </is>
-      </c>
-      <c r="I28" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2354,69 +2302,64 @@
           </r>
         </is>
       </c>
-      <c r="J28" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K28" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L28" s="18" t="inlineStr"/>
-      <c r="M28" s="19" t="inlineStr">
+      <c r="I28" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J28" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K28" s="17" t="inlineStr"/>
+      <c r="L28" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N28" s="18" t="inlineStr"/>
-      <c r="O28" s="18" t="inlineStr"/>
-      <c r="P28" s="18" t="inlineStr"/>
-      <c r="Q28" s="18" t="inlineStr"/>
-      <c r="R28" s="18" t="inlineStr"/>
-      <c r="S28" s="15" t="inlineStr">
+      <c r="M28" s="17" t="inlineStr"/>
+      <c r="N28" s="17" t="inlineStr"/>
+      <c r="O28" s="17" t="inlineStr"/>
+      <c r="P28" s="17" t="inlineStr"/>
+      <c r="Q28" s="17" t="inlineStr"/>
+      <c r="R28" s="14" t="inlineStr">
         <is>
           <t>Compound finish: dark patina base + hammered (martelé) texture applied on top — the only clear compound case in Fit-out</t>
         </is>
       </c>
     </row>
     <row r="29" ht="150" customHeight="1">
-      <c r="A29" s="15" t="n">
+      <c r="A29" s="14" t="n">
         <v>14</v>
       </c>
-      <c r="B29" s="15" t="inlineStr">
+      <c r="B29" s="14" t="inlineStr">
         <is>
           <t>A-GL-01a</t>
         </is>
       </c>
-      <c r="C29" s="15" t="inlineStr"/>
-      <c r="D29" s="15" t="inlineStr">
+      <c r="C29" s="14" t="inlineStr"/>
+      <c r="D29" s="14" t="inlineStr">
         <is>
           <t>Glass/Mirror</t>
         </is>
       </c>
-      <c r="E29" s="15" t="inlineStr">
-        <is>
-          <t>Miroir extra-clair</t>
-        </is>
-      </c>
-      <c r="F29" s="15" t="inlineStr">
+      <c r="E29" s="14" t="inlineStr">
         <is>
           <t>Extra-clear mirror</t>
         </is>
       </c>
-      <c r="G29" s="15" t="inlineStr">
+      <c r="F29" s="14" t="inlineStr">
         <is>
           <t>Extra-clair</t>
         </is>
       </c>
+      <c r="G29" s="14" t="inlineStr">
+        <is>
+          <t>K5M-T1B1-SDB-B/13, K5M-T1B1-CHA-C/7</t>
+        </is>
+      </c>
       <c r="H29" s="15" t="inlineStr">
-        <is>
-          <t>K5M-T1B1-SDB-B/13, K5M-T1B1-CHA-C/7</t>
-        </is>
-      </c>
-      <c r="I29" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2429,69 +2372,64 @@
           </r>
         </is>
       </c>
-      <c r="J29" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K29" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L29" s="18" t="inlineStr"/>
-      <c r="M29" s="19" t="inlineStr">
+      <c r="I29" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J29" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K29" s="17" t="inlineStr"/>
+      <c r="L29" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N29" s="18" t="inlineStr"/>
-      <c r="O29" s="18" t="inlineStr"/>
-      <c r="P29" s="18" t="inlineStr"/>
-      <c r="Q29" s="18" t="inlineStr"/>
-      <c r="R29" s="18" t="inlineStr"/>
-      <c r="S29" s="15" t="inlineStr">
+      <c r="M29" s="17" t="inlineStr"/>
+      <c r="N29" s="17" t="inlineStr"/>
+      <c r="O29" s="17" t="inlineStr"/>
+      <c r="P29" s="17" t="inlineStr"/>
+      <c r="Q29" s="17" t="inlineStr"/>
+      <c r="R29" s="14" t="inlineStr">
         <is>
           <t>Confirm scope boundary on B/13's inter-panel lighting (per RFI remark)</t>
         </is>
       </c>
     </row>
     <row r="30" ht="150" customHeight="1">
-      <c r="A30" s="15" t="n">
+      <c r="A30" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="B30" s="15" t="inlineStr">
+      <c r="B30" s="14" t="inlineStr">
         <is>
           <t>A-GL-02a</t>
         </is>
       </c>
-      <c r="C30" s="15" t="inlineStr"/>
-      <c r="D30" s="15" t="inlineStr">
+      <c r="C30" s="14" t="inlineStr"/>
+      <c r="D30" s="14" t="inlineStr">
         <is>
           <t>Glass/Mirror</t>
         </is>
       </c>
-      <c r="E30" s="15" t="inlineStr">
-        <is>
-          <t>Miroir extra-clair antique</t>
-        </is>
-      </c>
-      <c r="F30" s="15" t="inlineStr">
+      <c r="E30" s="14" t="inlineStr">
         <is>
           <t>Antique extra-clear mirror</t>
         </is>
       </c>
-      <c r="G30" s="15" t="inlineStr">
+      <c r="F30" s="14" t="inlineStr">
         <is>
           <t>Antique</t>
         </is>
       </c>
+      <c r="G30" s="14" t="inlineStr">
+        <is>
+          <t>K5M-T1B1-ENT</t>
+        </is>
+      </c>
       <c r="H30" s="15" t="inlineStr">
-        <is>
-          <t>K5M-T1B1-ENT</t>
-        </is>
-      </c>
-      <c r="I30" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2503,61 +2441,56 @@
           </r>
         </is>
       </c>
-      <c r="J30" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K30" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L30" s="18" t="inlineStr"/>
-      <c r="M30" s="19" t="inlineStr">
+      <c r="I30" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J30" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K30" s="17" t="inlineStr"/>
+      <c r="L30" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N30" s="18" t="inlineStr"/>
-      <c r="O30" s="18" t="inlineStr"/>
-      <c r="P30" s="18" t="inlineStr"/>
-      <c r="Q30" s="18" t="inlineStr"/>
-      <c r="R30" s="18" t="inlineStr"/>
-      <c r="S30" s="15" t="inlineStr"/>
+      <c r="M30" s="17" t="inlineStr"/>
+      <c r="N30" s="17" t="inlineStr"/>
+      <c r="O30" s="17" t="inlineStr"/>
+      <c r="P30" s="17" t="inlineStr"/>
+      <c r="Q30" s="17" t="inlineStr"/>
+      <c r="R30" s="14" t="inlineStr"/>
     </row>
     <row r="31" ht="150" customHeight="1">
-      <c r="A31" s="15" t="n">
+      <c r="A31" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="B31" s="15" t="inlineStr">
+      <c r="B31" s="14" t="inlineStr">
         <is>
           <t>A-GL-03a</t>
         </is>
       </c>
-      <c r="C31" s="15" t="inlineStr"/>
-      <c r="D31" s="15" t="inlineStr">
+      <c r="C31" s="14" t="inlineStr"/>
+      <c r="D31" s="14" t="inlineStr">
         <is>
           <t>Glass</t>
         </is>
       </c>
-      <c r="E31" s="15" t="inlineStr">
-        <is>
-          <t>Verre extra-clair + lin</t>
-        </is>
-      </c>
-      <c r="F31" s="15" t="inlineStr">
+      <c r="E31" s="14" t="inlineStr">
         <is>
           <t>Extra-clear glass + linen</t>
         </is>
       </c>
-      <c r="G31" s="15" t="inlineStr"/>
+      <c r="F31" s="14" t="inlineStr"/>
+      <c r="G31" s="14" t="inlineStr">
+        <is>
+          <t>K5M-T1B1-ENT-A/8, K5M-T1B1-SDB-B/14</t>
+        </is>
+      </c>
       <c r="H31" s="15" t="inlineStr">
-        <is>
-          <t>K5M-T1B1-ENT-A/8, K5M-T1B1-SDB-B/14</t>
-        </is>
-      </c>
-      <c r="I31" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2570,61 +2503,60 @@
           </r>
         </is>
       </c>
-      <c r="J31" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K31" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L31" s="18" t="inlineStr"/>
-      <c r="M31" s="19" t="inlineStr">
+      <c r="I31" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J31" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K31" s="17" t="inlineStr"/>
+      <c r="L31" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N31" s="18" t="inlineStr"/>
-      <c r="O31" s="18" t="inlineStr"/>
-      <c r="P31" s="18" t="inlineStr"/>
-      <c r="Q31" s="18" t="inlineStr"/>
-      <c r="R31" s="18" t="inlineStr"/>
-      <c r="S31" s="15" t="inlineStr"/>
+      <c r="M31" s="17" t="inlineStr"/>
+      <c r="N31" s="17" t="inlineStr"/>
+      <c r="O31" s="17" t="inlineStr"/>
+      <c r="P31" s="17" t="inlineStr"/>
+      <c r="Q31" s="17" t="inlineStr"/>
+      <c r="R31" s="14" t="inlineStr">
+        <is>
+          <t>Have made this panel before — a sample should be produced and included in the same box being presented to the client for approval.</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="150" customHeight="1">
-      <c r="A32" s="15" t="n">
+      <c r="A32" s="14" t="n">
         <v>17</v>
       </c>
-      <c r="B32" s="15" t="inlineStr">
+      <c r="B32" s="14" t="inlineStr">
         <is>
           <t>A-GL-04a</t>
         </is>
       </c>
-      <c r="C32" s="15" t="inlineStr"/>
-      <c r="D32" s="15" t="inlineStr">
+      <c r="C32" s="14" t="inlineStr"/>
+      <c r="D32" s="14" t="inlineStr">
         <is>
           <t>Glass</t>
         </is>
       </c>
-      <c r="E32" s="15" t="inlineStr">
-        <is>
-          <t>Verre extra-clair</t>
-        </is>
-      </c>
-      <c r="F32" s="15" t="inlineStr">
+      <c r="E32" s="14" t="inlineStr">
         <is>
           <t>Extra-clear glass</t>
         </is>
       </c>
-      <c r="G32" s="15" t="inlineStr"/>
+      <c r="F32" s="14" t="inlineStr"/>
+      <c r="G32" s="14" t="inlineStr">
+        <is>
+          <t>K5M-T1B1-SDB</t>
+        </is>
+      </c>
       <c r="H32" s="15" t="inlineStr">
-        <is>
-          <t>K5M-T1B1-SDB</t>
-        </is>
-      </c>
-      <c r="I32" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2636,180 +2568,38 @@
           </r>
         </is>
       </c>
-      <c r="J32" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K32" s="17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L32" s="18" t="inlineStr"/>
-      <c r="M32" s="19" t="inlineStr">
+      <c r="I32" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J32" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K32" s="17" t="inlineStr"/>
+      <c r="L32" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="N32" s="18" t="inlineStr"/>
-      <c r="O32" s="18" t="inlineStr"/>
-      <c r="P32" s="18" t="inlineStr"/>
-      <c r="Q32" s="18" t="inlineStr"/>
-      <c r="R32" s="18" t="inlineStr"/>
-      <c r="S32" s="15" t="inlineStr"/>
-    </row>
-    <row r="33" ht="150" customHeight="1">
-      <c r="A33" s="15" t="n">
-        <v>18</v>
-      </c>
-      <c r="B33" s="15" t="inlineStr">
-        <is>
-          <t>A-ST-03c / A-ST-06c</t>
-        </is>
-      </c>
-      <c r="C33" s="15" t="inlineStr"/>
-      <c r="D33" s="15" t="inlineStr">
-        <is>
-          <t>Stone</t>
-        </is>
-      </c>
-      <c r="E33" s="15" t="inlineStr">
-        <is>
-          <t>Travertin osso (vein cut / cross cut) — NOUVEAU 21 Jul</t>
-        </is>
-      </c>
-      <c r="F33" s="15" t="inlineStr">
-        <is>
-          <t>Travertine osso (vein cut / cross cut) — NEW 21 Jul</t>
-        </is>
-      </c>
-      <c r="G33" s="15" t="inlineStr">
-        <is>
-          <t>Adouci / Honed</t>
-        </is>
-      </c>
-      <c r="H33" s="15" t="inlineStr"/>
-      <c r="I33" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
-              <color rgb="00E4572E"/>
-              <sz val="11"/>
-              <u val="single"/>
-            </rPr>
-            <t>No location assigned yet in any document reviewed.</t>
-          </r>
-        </is>
-      </c>
-      <c r="J33" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K33" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L33" s="18" t="inlineStr"/>
-      <c r="M33" s="19" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="N33" s="18" t="inlineStr"/>
-      <c r="O33" s="18" t="inlineStr"/>
-      <c r="P33" s="18" t="inlineStr"/>
-      <c r="Q33" s="18" t="inlineStr"/>
-      <c r="R33" s="18" t="inlineStr"/>
-      <c r="S33" s="15" t="inlineStr">
-        <is>
-          <t>New codes as of 21 Jul 2026 — no confirmed location or in-scope task code yet, so no sample/high-res sourcing needed until scope is confirmed with Adil</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="150" customHeight="1">
-      <c r="A34" s="15" t="n">
-        <v>19</v>
-      </c>
-      <c r="B34" s="15" t="inlineStr">
-        <is>
-          <t>A-WD-03c</t>
-        </is>
-      </c>
-      <c r="C34" s="15" t="inlineStr"/>
-      <c r="D34" s="15" t="inlineStr">
-        <is>
-          <t>Wood</t>
-        </is>
-      </c>
-      <c r="E34" s="15" t="inlineStr">
-        <is>
-          <t>Tatawi peint en blanc — NOUVEAU 21 Jul</t>
-        </is>
-      </c>
-      <c r="F34" s="15" t="inlineStr">
-        <is>
-          <t>White-painted Tatawi wood — NEW 21 Jul</t>
-        </is>
-      </c>
-      <c r="G34" s="15" t="inlineStr">
-        <is>
-          <t>Mat</t>
-        </is>
-      </c>
-      <c r="H34" s="15" t="inlineStr"/>
-      <c r="I34" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Lato"/>
-              <color rgb="00E4572E"/>
-              <sz val="11"/>
-              <u val="single"/>
-            </rPr>
-            <t>No location assigned yet in any document reviewed.</t>
-          </r>
-        </is>
-      </c>
-      <c r="J34" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K34" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L34" s="18" t="inlineStr"/>
-      <c r="M34" s="19" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="N34" s="18" t="inlineStr"/>
-      <c r="O34" s="18" t="inlineStr"/>
-      <c r="P34" s="18" t="inlineStr"/>
-      <c r="Q34" s="18" t="inlineStr"/>
-      <c r="R34" s="18" t="inlineStr"/>
-      <c r="S34" s="15" t="inlineStr">
-        <is>
-          <t>New code as of 21 Jul 2026 — no confirmed location or in-scope task code yet, so no sample/high-res sourcing needed until scope is confirmed with Adil</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="3" t="inlineStr">
+      <c r="M32" s="17" t="inlineStr"/>
+      <c r="N32" s="17" t="inlineStr"/>
+      <c r="O32" s="17" t="inlineStr"/>
+      <c r="P32" s="17" t="inlineStr"/>
+      <c r="Q32" s="17" t="inlineStr"/>
+      <c r="R32" s="14" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>EXCLUDED — paint, wallpaper, and carpet are not in Wood Couture's Fit-out scope; kept out of this tracker entirely</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="20" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="19" t="inlineStr">
         <is>
           <t>A-PT-01, A-PT-02 (paint), A-WP-01, A-WP-02 (wallpaper), A-CA-01 (carpet)</t>
         </is>
@@ -2818,14 +2608,435 @@
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A12:H12"/>
-    <mergeCell ref="A37:S37"/>
-    <mergeCell ref="A36:S36"/>
-    <mergeCell ref="A14:S14"/>
-    <mergeCell ref="A1:S1"/>
+    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A14:R14"/>
     <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A2:S2"/>
+    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="A34:R34"/>
+    <mergeCell ref="A35:R35"/>
   </mergeCells>
-  <conditionalFormatting sqref="M16:M34">
+  <conditionalFormatting sqref="L16:L32">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"A"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"B"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"C"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
+      <formula>"S"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
+      <formula>"T"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="5">
+      <formula>"O"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="7" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="44" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>K5M — FIT-OUT MATERIAL PACKAGE — FABRICS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>As of 27 July 2026 — V3, first version of this tab. The banquette is Fit-out scope, so its fabrics (upholstery + decorative cushions) are tracked here rather than only on the FFE Fabrics tab. None of these have a WDCO item code assigned yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>STATUS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="C5" s="5">
+        <f>COUNTIF(J16:J200,"A")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Approved with comments</t>
+        </is>
+      </c>
+      <c r="C6" s="5">
+        <f>COUNTIF(J16:J200,"B")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="C7" s="5">
+        <f>COUNTIF(J16:J200,"C")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Submitted</t>
+        </is>
+      </c>
+      <c r="C8" s="5">
+        <f>COUNTIF(J16:J200,"S")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>To be Submitted</t>
+        </is>
+      </c>
+      <c r="C9" s="5">
+        <f>COUNTIF(J16:J200,"T")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Omitted</t>
+        </is>
+      </c>
+      <c r="C10" s="5">
+        <f>COUNTIF(J16:J200,"O")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C11" s="3">
+        <f>COUNTA(J16:J200)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Colors for "Approved with comments" and "Submitted" are a proposed extension of the official Brand DNA status palette — confirm or replace. Status defaulted to T (To be Submitted) for every row as a starting point.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15" ht="68" customHeight="1">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>Material Code</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>Thumbnail</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>Description (EN)</t>
+        </is>
+      </c>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>Applicable Item Code(s) (WDCO)</t>
+        </is>
+      </c>
+      <c r="G15" s="12" t="inlineStr">
+        <is>
+          <t>Control Sample (Y/N)</t>
+        </is>
+      </c>
+      <c r="H15" s="12" t="inlineStr">
+        <is>
+          <t>High-Res Available (Y/N)</t>
+        </is>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>High-Res Link</t>
+        </is>
+      </c>
+      <c r="J15" s="13" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="K15" s="13" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="L15" s="13" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="M15" s="13" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="N15" s="13" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="O15" s="13" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="P15" s="12" t="inlineStr">
+        <is>
+          <t>Remarks / Open Issues</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="150" customHeight="1">
+      <c r="A16" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="B16" s="20" t="inlineStr">
+        <is>
+          <t>FA-04</t>
+        </is>
+      </c>
+      <c r="C16" s="20" t="inlineStr"/>
+      <c r="D16" s="20" t="inlineStr">
+        <is>
+          <t>Fabric</t>
+        </is>
+      </c>
+      <c r="E16" s="20" t="inlineStr">
+        <is>
+          <t>Anubis col. 203 (Les Créations de la Maison)</t>
+        </is>
+      </c>
+      <c r="F16" s="20" t="inlineStr"/>
+      <c r="G16" s="20" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H16" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I16" s="20" t="inlineStr"/>
+      <c r="J16" s="21" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="K16" s="17" t="inlineStr"/>
+      <c r="L16" s="17" t="inlineStr"/>
+      <c r="M16" s="17" t="inlineStr"/>
+      <c r="N16" s="17" t="inlineStr"/>
+      <c r="O16" s="17" t="inlineStr"/>
+      <c r="P16" s="14" t="inlineStr">
+        <is>
+          <t>Banquette upholstery fabric. This fabric also has a row on the FFE Fabrics tab (as a previously-fixed known gap); no WDCO item code is currently assigned to it — confirm correct item code with the team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="150" customHeight="1">
+      <c r="A17" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="B17" s="20" t="inlineStr">
+        <is>
+          <t>FA-05</t>
+        </is>
+      </c>
+      <c r="C17" s="20" t="inlineStr"/>
+      <c r="D17" s="20" t="inlineStr">
+        <is>
+          <t>Fabric</t>
+        </is>
+      </c>
+      <c r="E17" s="20" t="inlineStr">
+        <is>
+          <t>Tatin T25014/009 Tabacco (Dedar)</t>
+        </is>
+      </c>
+      <c r="F17" s="20" t="inlineStr"/>
+      <c r="G17" s="20" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H17" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I17" s="20" t="inlineStr"/>
+      <c r="J17" s="21" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="K17" s="17" t="inlineStr"/>
+      <c r="L17" s="17" t="inlineStr"/>
+      <c r="M17" s="17" t="inlineStr"/>
+      <c r="N17" s="17" t="inlineStr"/>
+      <c r="O17" s="17" t="inlineStr"/>
+      <c r="P17" s="14" t="inlineStr">
+        <is>
+          <t>Banquette decorative cushion fabric. No WDCO item code currently assigned — confirm with the team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="150" customHeight="1">
+      <c r="A18" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="B18" s="20" t="inlineStr">
+        <is>
+          <t>FA-08</t>
+        </is>
+      </c>
+      <c r="C18" s="20" t="inlineStr"/>
+      <c r="D18" s="20" t="inlineStr">
+        <is>
+          <t>Fabric</t>
+        </is>
+      </c>
+      <c r="E18" s="20" t="inlineStr">
+        <is>
+          <t>Lueurs de Montmartre M445 301 mordoré (Misia)</t>
+        </is>
+      </c>
+      <c r="F18" s="20" t="inlineStr"/>
+      <c r="G18" s="20" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H18" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I18" s="20" t="inlineStr"/>
+      <c r="J18" s="21" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="K18" s="17" t="inlineStr"/>
+      <c r="L18" s="17" t="inlineStr"/>
+      <c r="M18" s="17" t="inlineStr"/>
+      <c r="N18" s="17" t="inlineStr"/>
+      <c r="O18" s="17" t="inlineStr"/>
+      <c r="P18" s="14" t="inlineStr">
+        <is>
+          <t>Banquette decorative cushion fabric. No WDCO item code currently assigned — confirm with the team.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A14:P14"/>
+    <mergeCell ref="A2:P2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="J16:J18">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"A"</formula>
     </cfRule>

</xml_diff>